<commit_message>
feat: sort ASU faculty A to Z and add clickable hyperlinks in Excel
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Faculty A-Z" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Matched A-Z" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,12 +18,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -43,14 +51,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -466,12 +477,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lin Li</t>
+          <t>Aditi Chattopadhyay</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Regents Professor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -484,35 +495,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Lin.Li.10@asu.edu</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>aditi@asu.edu</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>inverse problems, multiscale modeling, optimization, transition</t>
+        </is>
+      </c>
       <c r="G2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/linli25</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/chattopa</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Aditi%20Chattopadhyay%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kunal Garg</t>
+          <t>Aikaterini Stefanaki</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Teaching Professor</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,27 +540,23 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>kgarg24@asu.edu</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>optimization</t>
-        </is>
-      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>astefan9@asu.edu</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/kgarg24</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kunal%20Garg%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/astefan9</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Aikaterini%20Stefanaki%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
@@ -570,7 +581,7 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Alberto.Scotti@asu.edu</t>
         </is>
@@ -583,12 +594,12 @@
       <c r="G4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>https://search.asu.edu/profile/adscotti</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Alberto%20Scotti%20Arizona%20State%20University</t>
         </is>
@@ -597,12 +608,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zhe Xu</t>
+          <t>Beomjin Kwon</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -615,35 +626,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>xzhe1@asu.edu</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>kwon@asu.edu</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>data-driven modeling, heat transfer, transport phenomena</t>
+        </is>
+      </c>
       <c r="G5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/xzhe1</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/bkwon2</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Beomjin%20Kwon%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aikaterini Stefanaki</t>
+          <t>Cindy (Xiangjia) Li</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Associate Teaching Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -656,35 +671,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>astefan9@asu.edu</t>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>xiangjia.li@asu.edu</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="b">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/astefan9</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Aikaterini%20Stefanaki%20Arizona%20State%20University</t>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/xiangji5</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Cindy%20%28Xiangjia%29%20Li%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ronald Calhoun</t>
+          <t>Derrick Speaks</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Teaching Professor</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -697,39 +712,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Ronald.Calhoun@asu.edu</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>fluid dynamics</t>
-        </is>
-      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Derrick.Speaks@asu.edu</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/rcalhou</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/dspeaks2</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Derrick%20Speaks%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wonmo Kang</t>
+          <t>Erik Andersen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Faculty Associate</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -742,23 +753,23 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Wonmo.Kang@asu.edu</t>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Erik.J.Andersen@asu.edu</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="b">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/wkang16</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Wonmo%20Kang%20Arizona%20State%20University</t>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/ejande22</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Erik%20Andersen%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
@@ -783,7 +794,7 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Gokul.Pathikonda@asu.edu</t>
         </is>
@@ -796,12 +807,12 @@
       <c r="G9" t="b">
         <v>1</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="1" t="inlineStr">
         <is>
           <t>https://search.asu.edu/profile/gpathiko</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="1" t="inlineStr">
         <is>
           <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University</t>
         </is>
@@ -810,12 +821,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yongming Liu</t>
+          <t>Hamidreza Marvi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -828,34 +839,30 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Yongming.Liu@asu.edu</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>uncertainty quantification</t>
-        </is>
-      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>hmarvi@asu.edu</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/yliu35</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/hmarvi</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hamidreza%20Marvi%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Liping Wang</t>
+          <t>Houlong Zhuang</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -873,39 +880,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Liping.Wang@asu.edu</t>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>zhuanghl@asu.edu</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>heat transfer</t>
+          <t>computational physics</t>
         </is>
       </c>
       <c r="G11" t="b">
         <v>1</v>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/lwang78</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University</t>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/hzhuang7</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Houlong%20Zhuang%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Qiong Nian</t>
+          <t>Huan Wu</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Faculty</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -918,30 +925,34 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Qiong.Nian@asu.edu</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>huanwu@asu.edu</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>computational physics</t>
+        </is>
+      </c>
       <c r="G12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/qnian</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/huanwu</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huan%20Wu%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hyunglae Lee</t>
+          <t>Huei-Ping Huang</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -959,35 +970,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Hyunglae.Lee@asu.edu</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Huei-Ping.Huang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>fluid dynamics, numerical simulation</t>
+        </is>
+      </c>
       <c r="G13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/hlee234</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/hhuang38</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Patrick Phelan</t>
+          <t>Hyunglae Lee</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1000,35 +1015,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>phelan@asu.edu</t>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Hyunglae.Lee@asu.edu</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="b">
         <v>0</v>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/pphelan</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University</t>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/hlee234</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Beomjin Kwon</t>
+          <t>Ivy Chang</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Teaching Professor</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1041,27 +1056,23 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>kwon@asu.edu</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>data-driven modeling, heat transfer, transport phenomena</t>
-        </is>
-      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Ivy.Chang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/bkwon2</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Beomjin%20Kwon%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/iychang</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ivy%20Chang%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1097,7 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Jagannathan.Rajagopalan@asu.edu</t>
         </is>
@@ -1099,12 +1110,12 @@
       <c r="G16" t="b">
         <v>1</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="1" t="inlineStr">
         <is>
           <t>https://search.asu.edu/profile/jrajago1</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="1" t="inlineStr">
         <is>
           <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jagannathan%20Rajagopalan%20Arizona%20State%20University</t>
         </is>
@@ -1113,12 +1124,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>T.-W. Lee</t>
+          <t>James Middleton</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1131,27 +1142,23 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>ATTWL@asu.edu</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>aerospace propulsion, propulsion</t>
-        </is>
-      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>jimbo@asu.edu</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/attwl</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/jimbo</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1183,7 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>joswald1@asu.edu</t>
         </is>
@@ -1189,12 +1196,12 @@
       <c r="G18" t="b">
         <v>1</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="1" t="inlineStr">
         <is>
           <t>https://search.asu.edu/profile/joswald1</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="1" t="inlineStr">
         <is>
           <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University</t>
         </is>
@@ -1203,12 +1210,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Raghavendra Murthy</t>
+          <t>Jeonglae Kim</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Associate Teaching Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1221,39 +1228,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>rnmurthy@asu.edu</t>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>jeokim@asu.edu</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>optimization, reduced-order modeling</t>
+          <t>aeroacoustics, flow control, optimization, turbulence, turbulent flows</t>
         </is>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/rnmurthy</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Raghavendra%20Murthy%20Arizona%20State%20University</t>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/jkim520</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Srinivas Chakravarthi Kosaraju</t>
+          <t>Jiefeng Sun</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Teaching Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1266,35 +1273,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Srinivas.Kosaraju@asu.edu</t>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Jiefeng.Sun@asu.edu</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="b">
         <v>0</v>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/skosara2</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Srinivas%20Chakravarthi%20Kosaraju%20Arizona%20State%20University</t>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/jsun165</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jiefeng%20Sun%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Huei-Ping Huang</t>
+          <t>Joshua Wilbur</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Associate Teaching Professor</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1307,39 +1314,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Huei-Ping.Huang@asu.edu</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>fluid dynamics, numerical simulation</t>
-        </is>
-      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Joshua.Wilbur@asu.edu</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/hhuang38</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/jdwilbu1</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Joshua%20Wilbur%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Erik Andersen</t>
+          <t>Kangping Chen</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Faculty Associate</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1352,35 +1355,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Erik.J.Andersen@asu.edu</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>k.p.chen@asu.edu</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>computational fluid dynamics, drag reduction, fluid dynamics, fluid mechanics, multiphase flow</t>
+        </is>
+      </c>
       <c r="G22" t="b">
-        <v>0</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/ejande22</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Erik%20Andersen%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/asuchen</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kangping%20Chen%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sridhar Seetharaman</t>
+          <t>Kiran Ramesh</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1393,35 +1400,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>seetharaman@asu.edu</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Kiran.Ramesh@asu.edu</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>aerodynamics, flow control, fluid dynamics, turbulence, vortex dynamics</t>
+        </is>
+      </c>
       <c r="G23" t="b">
-        <v>0</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/sseeth11</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Sridhar%20Seetharaman%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/kramesh2</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kiran%20Ramesh%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aditi Chattopadhyay</t>
+          <t>Konrad Rykaczewski</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Regents Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1434,39 +1445,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>aditi@asu.edu</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>inverse problems, multiscale modeling, optimization, transition</t>
-        </is>
-      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>konradr@asu.edu</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="b">
-        <v>1</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/chattopa</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Aditi%20Chattopadhyay%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/krykacze</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Konrad%20Rykaczewski%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mohamed Houssem Kasbaoui</t>
+          <t>Kunal Garg</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1479,39 +1486,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>houssem.kasbaoui@asu.edu</t>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>kgarg24@asu.edu</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>cfd, computational fluid dynamics, dns, fluid dynamics, multiphase flow</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="G25" t="b">
         <v>1</v>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/mkasbaou</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University</t>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/kgarg24</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kunal%20Garg%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jiefeng Sun</t>
+          <t>Leila Ladani</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1524,35 +1531,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Jiefeng.Sun@asu.edu</t>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>ladani@asu.edu</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="b">
         <v>0</v>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/jsun165</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jiefeng%20Sun%20Arizona%20State%20University</t>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/ljannesa</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Yi Ren</t>
+          <t>Leixin Ma</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1565,39 +1572,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>yiren@asu.edu</t>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Leixin.Ma@asu.edu</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>aerodynamics, fluid-structure interaction, physics-informed machine learning</t>
         </is>
       </c>
       <c r="G27" t="b">
         <v>1</v>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/yren32</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University</t>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/leixinma</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leixin%20Ma%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Derrick Speaks</t>
+          <t>Lin Li</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Assistant Teaching Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1610,35 +1617,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Derrick.Speaks@asu.edu</t>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Lin.Li.10@asu.edu</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="b">
         <v>0</v>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/dspeaks2</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Derrick%20Speaks%20Arizona%20State%20University</t>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/linli25</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Werner Dahm</t>
+          <t>Liping Wang</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SUM/WTR Faculty Research</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1651,39 +1658,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Werner.Dahm@asu.edu</t>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>Liping.Wang@asu.edu</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>combustion, computational physics, fluid dynamics, heat transfer, propulsion, turbulence</t>
+          <t>heat transfer</t>
         </is>
       </c>
       <c r="G29" t="b">
         <v>1</v>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/wdahm</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University</t>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/lwang78</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Leixin Ma</t>
+          <t>Marc Mignolet</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1696,34 +1703,30 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Leixin.Ma@asu.edu</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>aerodynamics, fluid-structure interaction, physics-informed machine learning</t>
-        </is>
-      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>marc.mignolet@asu.edu</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="b">
-        <v>1</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/leixinma</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leixin%20Ma%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/marc03</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leila Ladani</t>
+          <t>Marcus Herrmann</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1741,35 +1744,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>ladani@asu.edu</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Marcus.Herrmann@asu.edu</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>fluid mechanics, multiphase flow, numerical simulation, turbulence</t>
+        </is>
+      </c>
       <c r="G31" t="b">
-        <v>0</v>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/ljannesa</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mherrma1</t>
+        </is>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marcus%20Herrmann%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Spring Berman</t>
+          <t>Matthew Peet</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1782,9 +1789,9 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Spring.Berman@asu.edu</t>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>mpeet@asu.edu</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1795,26 +1802,26 @@
       <c r="G32" t="b">
         <v>1</v>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/smberma2</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Spring%20Berman%20Arizona%20State%20University</t>
+      <c r="H32" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mpeet</t>
+        </is>
+      </c>
+      <c r="I32" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Huan Wu</t>
+          <t>Minglei Qu</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Faculty</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1827,34 +1834,34 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>huanwu@asu.edu</t>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>minglei.qu@asu.edu</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>computational physics</t>
+          <t>instability</t>
         </is>
       </c>
       <c r="G33" t="b">
         <v>1</v>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/huanwu</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huan%20Wu%20Arizona%20State%20University</t>
+      <c r="H33" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mingleiq</t>
+        </is>
+      </c>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Minglei%20Qu%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Matthew Peet</t>
+          <t>Mohamed Houssem Kasbaoui</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1872,39 +1879,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>mpeet@asu.edu</t>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>houssem.kasbaoui@asu.edu</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>cfd, computational fluid dynamics, dns, fluid dynamics, multiphase flow</t>
         </is>
       </c>
       <c r="G34" t="b">
         <v>1</v>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/mpeet</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University</t>
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mkasbaou</t>
+        </is>
+      </c>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Wanxin Jin</t>
+          <t>Patrick Phelan</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1917,23 +1924,23 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>wjin@asu.edu</t>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>phelan@asu.edu</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="b">
         <v>0</v>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/wjin34</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Wanxin%20Jin%20Arizona%20State%20University</t>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/pphelan</t>
+        </is>
+      </c>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1965,7 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="1" t="inlineStr">
         <is>
           <t>pperalta@asu.edu</t>
         </is>
@@ -1967,12 +1974,12 @@
       <c r="G36" t="b">
         <v>0</v>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" s="1" t="inlineStr">
         <is>
           <t>https://search.asu.edu/profile/pperalta</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" s="1" t="inlineStr">
         <is>
           <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Pedro%20Peralta%20Arizona%20State%20University</t>
         </is>
@@ -1981,12 +1988,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ivy Chang</t>
+          <t>Qiong Nian</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Assistant Teaching Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1999,35 +2006,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Ivy.Chang@asu.edu</t>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Qiong.Nian@asu.edu</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="b">
         <v>0</v>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/iychang</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ivy%20Chang%20Arizona%20State%20University</t>
+      <c r="H37" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/qnian</t>
+        </is>
+      </c>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cindy (Xiangjia) Li</t>
+          <t>Raghavendra Murthy</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Associate Teaching Professor</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2040,35 +2047,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>xiangjia.li@asu.edu</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>rnmurthy@asu.edu</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>optimization, reduced-order modeling</t>
+        </is>
+      </c>
       <c r="G38" t="b">
-        <v>0</v>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/xiangji5</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Cindy%20%28Xiangjia%29%20Li%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rnmurthy</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Raghavendra%20Murthy%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kangping Chen</t>
+          <t>Ricardo Cruz Lozano</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Teaching Professor</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2081,34 +2092,30 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>k.p.chen@asu.edu</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>computational fluid dynamics, drag reduction, fluid dynamics, fluid mechanics, multiphase flow</t>
-        </is>
-      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>Ricardo.Cruz.Lozano@asu.edu</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="b">
-        <v>1</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/asuchen</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kangping%20Chen%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rcruzloz</t>
+        </is>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ricardo%20Cruz%20Lozano%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hamidreza Marvi</t>
+          <t>Robert Wang</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2126,35 +2133,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>hmarvi@asu.edu</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>rywang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>heat transfer</t>
+        </is>
+      </c>
       <c r="G40" t="b">
-        <v>0</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/hmarvi</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hamidreza%20Marvi%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rywang</t>
+        </is>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Robert%20Wang%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Minglei Qu</t>
+          <t>Ronald Calhoun</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2167,39 +2178,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>minglei.qu@asu.edu</t>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Ronald.Calhoun@asu.edu</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>instability</t>
+          <t>fluid dynamics</t>
         </is>
       </c>
       <c r="G41" t="b">
         <v>1</v>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/mingleiq</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Minglei%20Qu%20Arizona%20State%20University</t>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rcalhou</t>
+        </is>
+      </c>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Marcus Herrmann</t>
+          <t>Ryan Milcarek</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2212,39 +2223,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Marcus.Herrmann@asu.edu</t>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>Ryan.Milcarek@asu.edu</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>fluid mechanics, multiphase flow, numerical simulation, turbulence</t>
+          <t>combustion, transition</t>
         </is>
       </c>
       <c r="G42" t="b">
         <v>1</v>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/mherrma1</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marcus%20Herrmann%20Arizona%20State%20University</t>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rjmilcar</t>
+        </is>
+      </c>
+      <c r="I42" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ricardo Cruz Lozano</t>
+          <t>Spring Berman</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Assistant Teaching Professor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2257,35 +2268,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Ricardo.Cruz.Lozano@asu.edu</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>Spring.Berman@asu.edu</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>optimization</t>
+        </is>
+      </c>
       <c r="G43" t="b">
-        <v>0</v>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/rcruzloz</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ricardo%20Cruz%20Lozano%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/smberma2</t>
+        </is>
+      </c>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Spring%20Berman%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ryan Milcarek</t>
+          <t>Sridhar Seetharaman</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2298,39 +2313,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Ryan.Milcarek@asu.edu</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>combustion, transition</t>
-        </is>
-      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>seetharaman@asu.edu</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="b">
-        <v>1</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/rjmilcar</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/sseeth11</t>
+        </is>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Sridhar%20Seetharaman%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Konrad Rykaczewski</t>
+          <t>Srinivas Chakravarthi Kosaraju</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Teaching Professor</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2343,30 +2354,30 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>konradr@asu.edu</t>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Srinivas.Kosaraju@asu.edu</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="b">
         <v>0</v>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/krykacze</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Konrad%20Rykaczewski%20Arizona%20State%20University</t>
+      <c r="H45" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/skosara2</t>
+        </is>
+      </c>
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Srinivas%20Chakravarthi%20Kosaraju%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kiran Ramesh</t>
+          <t>T.-W. Lee</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2384,39 +2395,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Kiran.Ramesh@asu.edu</t>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>ATTWL@asu.edu</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>aerodynamics, flow control, fluid dynamics, turbulence, vortex dynamics</t>
+          <t>aerospace propulsion, propulsion</t>
         </is>
       </c>
       <c r="G46" t="b">
         <v>1</v>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/kramesh2</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kiran%20Ramesh%20Arizona%20State%20University</t>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/attwl</t>
+        </is>
+      </c>
+      <c r="I46" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Joshua Wilbur</t>
+          <t>Tianyu Yang</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Associate Teaching Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2429,35 +2440,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Joshua.Wilbur@asu.edu</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Tianyu.Yang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>heat transfer</t>
+        </is>
+      </c>
       <c r="G47" t="b">
-        <v>0</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/jdwilbu1</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Joshua%20Wilbur%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/tyang123</t>
+        </is>
+      </c>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Houlong Zhuang</t>
+          <t>Wanxin Jin</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2470,39 +2485,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>zhuanghl@asu.edu</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>computational physics</t>
-        </is>
-      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>wjin@asu.edu</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="b">
-        <v>1</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/hzhuang7</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Houlong%20Zhuang%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/wjin34</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Wanxin%20Jin%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tianyu Yang</t>
+          <t>Werner Dahm</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>SUM/WTR Faculty Research</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2515,39 +2526,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Tianyu.Yang@asu.edu</t>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>Werner.Dahm@asu.edu</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>heat transfer</t>
+          <t>combustion, computational physics, fluid dynamics, heat transfer, propulsion, turbulence</t>
         </is>
       </c>
       <c r="G49" t="b">
         <v>1</v>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/tyang123</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University</t>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/wdahm</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Yulia Peet</t>
+          <t>Wonmo Kang</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2560,39 +2571,35 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>ypeet@asu.edu</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>fluid mechanics, high-performance computing, turbulence</t>
-        </is>
-      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>Wonmo.Kang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="b">
-        <v>1</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/ypeet</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yulia%20Peet%20Arizona%20State%20University</t>
+        <v>0</v>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/wkang16</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Wonmo%20Kang%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Marc Mignolet</t>
+          <t>Yi Ren</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2605,35 +2612,39 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>marc.mignolet@asu.edu</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>yiren@asu.edu</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>optimization</t>
+        </is>
+      </c>
       <c r="G51" t="b">
-        <v>0</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/marc03</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/yren32</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Robert Wang</t>
+          <t>Yongming Liu</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2646,34 +2657,34 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>rywang@asu.edu</t>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>Yongming.Liu@asu.edu</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>heat transfer</t>
+          <t>uncertainty quantification</t>
         </is>
       </c>
       <c r="G52" t="b">
         <v>1</v>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/rywang</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Robert%20Wang%20Arizona%20State%20University</t>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/yliu35</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>James Middleton</t>
+          <t>Yulia Peet</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2691,72 +2702,1736 @@
           <t>Arizona State University</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>jimbo@asu.edu</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>ypeet@asu.edu</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>fluid mechanics, high-performance computing, turbulence</t>
+        </is>
+      </c>
       <c r="G53" t="b">
-        <v>0</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>https://search.asu.edu/profile/jimbo</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University</t>
+        <v>1</v>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/ypeet</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yulia%20Peet%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Zhe Xu</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>xzhe1@asu.edu</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="b">
+        <v>0</v>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/xzhe1</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId159"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Job Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Matched Fields</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Is Field Match</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Profile URL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Google Scholar URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aditi Chattopadhyay</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Regents Professor</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>aditi@asu.edu</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>inverse problems, multiscale modeling, optimization, transition</t>
+        </is>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/chattopa</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Aditi%20Chattopadhyay%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Alberto Scotti</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Alberto.Scotti@asu.edu</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>applied mathematics, fluid mechanics, turbulent mixing</t>
+        </is>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/adscotti</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Alberto%20Scotti%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Beomjin Kwon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>kwon@asu.edu</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>data-driven modeling, heat transfer, transport phenomena</t>
+        </is>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/bkwon2</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Beomjin%20Kwon%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gokul Pathikonda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Gokul.Pathikonda@asu.edu</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>aerodynamics, reacting flows, turbulence, turbulent mixing</t>
+        </is>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/gpathiko</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Houlong Zhuang</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>zhuanghl@asu.edu</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>computational physics</t>
+        </is>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/hzhuang7</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Houlong%20Zhuang%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Huan Wu</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Faculty</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>huanwu@asu.edu</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>computational physics</t>
+        </is>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/huanwu</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huan%20Wu%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Huei-Ping Huang</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Huei-Ping.Huang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>fluid dynamics, numerical simulation</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/hhuang38</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jagannathan Rajagopalan</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Jagannathan.Rajagopalan@asu.edu</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>optimization</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/jrajago1</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jagannathan%20Rajagopalan%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jay Oswald</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>joswald1@asu.edu</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>finite element</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/joswald1</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Jeonglae Kim</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Assistant Professor</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Aerospace &amp; Mechanical Engineering</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Arizona State University</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>jeokim@asu.edu</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>aeroacoustics, flow control, optimization, turbulence, turbulent flows</t>
         </is>
       </c>
-      <c r="G54" t="b">
-        <v>1</v>
-      </c>
-      <c r="H54" t="inlineStr">
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>https://search.asu.edu/profile/jkim520</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University</t>
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Kangping Chen</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>k.p.chen@asu.edu</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>computational fluid dynamics, drag reduction, fluid dynamics, fluid mechanics, multiphase flow</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/asuchen</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kangping%20Chen%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Kiran Ramesh</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Kiran.Ramesh@asu.edu</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>aerodynamics, flow control, fluid dynamics, turbulence, vortex dynamics</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/kramesh2</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kiran%20Ramesh%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Kunal Garg</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>kgarg24@asu.edu</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>optimization</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/kgarg24</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Kunal%20Garg%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Leixin Ma</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Leixin.Ma@asu.edu</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>aerodynamics, fluid-structure interaction, physics-informed machine learning</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/leixinma</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leixin%20Ma%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Liping Wang</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Liping.Wang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>heat transfer</t>
+        </is>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/lwang78</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Marcus Herrmann</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Marcus.Herrmann@asu.edu</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>fluid mechanics, multiphase flow, numerical simulation, turbulence</t>
+        </is>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mherrma1</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marcus%20Herrmann%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Matthew Peet</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>mpeet@asu.edu</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>optimization</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mpeet</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Minglei Qu</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>minglei.qu@asu.edu</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>instability</t>
+        </is>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mingleiq</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Minglei%20Qu%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mohamed Houssem Kasbaoui</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>houssem.kasbaoui@asu.edu</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>cfd, computational fluid dynamics, dns, fluid dynamics, multiphase flow</t>
+        </is>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/mkasbaou</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Raghavendra Murthy</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Associate Teaching Professor</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>rnmurthy@asu.edu</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>optimization, reduced-order modeling</t>
+        </is>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rnmurthy</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Raghavendra%20Murthy%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Robert Wang</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>rywang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>heat transfer</t>
+        </is>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rywang</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Robert%20Wang%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ronald Calhoun</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Ronald.Calhoun@asu.edu</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>fluid dynamics</t>
+        </is>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rcalhou</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ryan Milcarek</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Ryan.Milcarek@asu.edu</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>combustion, transition</t>
+        </is>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/rjmilcar</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Spring Berman</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>Spring.Berman@asu.edu</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>optimization</t>
+        </is>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/smberma2</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Spring%20Berman%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>T.-W. Lee</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>ATTWL@asu.edu</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>aerospace propulsion, propulsion</t>
+        </is>
+      </c>
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/attwl</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tianyu Yang</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Tianyu.Yang@asu.edu</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>heat transfer</t>
+        </is>
+      </c>
+      <c r="G27" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/tyang123</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Werner Dahm</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SUM/WTR Faculty Research</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Werner.Dahm@asu.edu</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>combustion, computational physics, fluid dynamics, heat transfer, propulsion, turbulence</t>
+        </is>
+      </c>
+      <c r="G28" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/wdahm</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Yi Ren</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>yiren@asu.edu</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>optimization</t>
+        </is>
+      </c>
+      <c r="G29" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/yren32</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Yongming Liu</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Yongming.Liu@asu.edu</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>uncertainty quantification</t>
+        </is>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/yliu35</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Yulia Peet</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Arizona State University</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>ypeet@asu.edu</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>fluid mechanics, high-performance computing, turbulence</t>
+        </is>
+      </c>
+      <c r="G31" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t>https://search.asu.edu/profile/ypeet</t>
+        </is>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yulia%20Peet%20Arizona%20State%20University</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId90"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add research interests, expertise areas, and research summary columns in ASU faculty Excel
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -465,10 +465,13 @@
     <col width="49" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="49" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="49" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,20 +512,35 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Research Interests</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Expertise Areas</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Research / Bio Summary</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Scholar ID</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Profile URL</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Google Scholar URL</t>
         </is>
@@ -531,12 +549,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Werner Dahm</t>
+          <t>Jeonglae Kim</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SUM/WTR Faculty Research</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -550,7 +568,7 @@
         </is>
       </c>
       <c r="E2" s="3">
-        <f>HYPERLINK("mailto:Werner.Dahm@asu.edu", "Werner.Dahm@asu.edu")</f>
+        <f>HYPERLINK("mailto:jeokim@asu.edu", "jeokim@asu.edu")</f>
         <v/>
       </c>
       <c r="F2" s="2" t="n">
@@ -558,31 +576,38 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>combustion, computational physics, fluid dynamics, heat transfer, propulsion, turbulence</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="b">
-        <v>1</v>
-      </c>
+          <t>aeroacoustics, flow control, high-performance computing, optimization, turbulence, turbulent flows</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/wdahm", "https://search.asu.edu/profile/wdahm")</f>
-        <v/>
-      </c>
-      <c r="K2" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University", "Google Scholar Search")</f>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Kim's research interests include large-eddy simulation of high-speed turbulent flows with multi-physics, aeroacoustics, flow control and optimization.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="3">
+        <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
+        <v/>
+      </c>
+      <c r="N2" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Jeonglae Kim</t>
+          <t>Werner Dahm</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>SUM/WTR Faculty Research</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -596,27 +621,42 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <f>HYPERLINK("mailto:jeokim@asu.edu", "jeokim@asu.edu")</f>
+        <f>HYPERLINK("mailto:Werner.Dahm@asu.edu", "Werner.Dahm@asu.edu")</f>
         <v/>
       </c>
       <c r="F3" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>aeroacoustics, flow control, optimization, turbulence, turbulent flows</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
-        <v/>
-      </c>
-      <c r="K3" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
+          <t>combustion, computational physics, fluid dynamics, heat transfer, propulsion, turbulence</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Dahm specializes in fluid dynamics, thermodynamics, combustion, heat transfer, thermal sciences, propulsion, fuel efficiency, emissions, powertrains, and other areas relevant to a broad range of automotive, aerospace, and industrial applications. He is an author of over 200 refereed technical articles, conference papers, and technical publications, a holder of six U.S. and international patents, and has given over 260 technical presentations, including over 190 invited, plenary, and keynote lectures worldwide, on topics dealing with mechanical and aerospace engineering and defense science.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace Engineering, Applied Research, Computational Modeling, Computational Physics, Mechanical Engineering, Propulsion</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Werner J.A. Dahm has since 2010 been the ASU Foundation Professor of Mechanical and Aerospace Engineering, and also Professor Emeritus of Engineering at the University of Michigan where served for the previous 25 years.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="3">
+        <f>HYPERLINK("https://search.asu.edu/profile/wdahm", "https://search.asu.edu/profile/wdahm")</f>
+        <v/>
+      </c>
+      <c r="N3" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
     </row>
@@ -653,19 +693,26 @@
           <t>computational fluid dynamics, drag reduction, fluid dynamics, fluid mechanics, multiphase flow</t>
         </is>
       </c>
-      <c r="H4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Chen’s research interests include multiphase flows, drag reduction, airplane de-icing, interfacial instabilities and flow in porous media.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>xT-lX9sAAAAJ</t>
         </is>
       </c>
-      <c r="J4" s="3">
+      <c r="M4" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="K4" s="3">
+      <c r="N4" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
@@ -703,19 +750,30 @@
           <t>aerodynamics, flow control, fluid dynamics, turbulence, vortex dynamics</t>
         </is>
       </c>
-      <c r="H5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Unsteady aerodynamics, vortex dynamics, flow control, turbulence, separated flows</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Ramesh's expertise is in unsteady fluid dynamics, vortex dynamics, turbulence and flow control.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>DKc-AgcAAAAJ</t>
         </is>
       </c>
-      <c r="J5" s="3">
+      <c r="M5" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kramesh2", "https://search.asu.edu/profile/kramesh2")</f>
         <v/>
       </c>
-      <c r="K5" s="3">
+      <c r="N5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
         <v/>
       </c>
@@ -753,15 +811,22 @@
           <t>cfd, computational fluid dynamics, dns, fluid dynamics, multiphase flow</t>
         </is>
       </c>
-      <c r="H6" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="3">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Kasbaoui's research interests include computational fluid dynamics, numerical methods, and massively parallel simulations of multiphase and particle-laden flows for environmental and aerospace applications.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
         <v/>
       </c>
-      <c r="K6" s="3">
+      <c r="N6" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -799,19 +864,26 @@
           <t>inverse problems, multiscale modeling, optimization, transition</t>
         </is>
       </c>
-      <c r="H7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Chattopadhyay is the director of Adaptive Intelligent Materials and Systems (AIMS) Center at ASU. Her research focuses on structural health monitoring and damage prognosis, and multidisciplinary design optimization.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>w3fU9E0AAAAJ</t>
         </is>
       </c>
-      <c r="J7" s="3">
+      <c r="M7" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/chattopa", "https://search.asu.edu/profile/chattopa")</f>
         <v/>
       </c>
-      <c r="K7" s="3">
+      <c r="N7" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
@@ -849,15 +921,30 @@
           <t>aerodynamics, reacting flows, turbulence, turbulent mixing</t>
         </is>
       </c>
-      <c r="H8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="3">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Pathikonda studies turbulent fluid flows to understand natural and engineering phenomena using lab experiments. His expertise is in complex (reacting) mixing, high Re-flows, laser-based &amp; spectroscopic techniques, etc.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
         <v/>
       </c>
-      <c r="K8" s="3">
+      <c r="N8" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -895,19 +982,26 @@
           <t>fluid mechanics, multiphase flow, numerical simulation, turbulence</t>
         </is>
       </c>
-      <c r="H9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Herrmann's research interests include fluid mechanics, modeling and numerical simulation of multiphase flows with a focus on turbulent atomization processes, and numerical methods for discontinuous interfaces.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>yv6aCW8AAAAJ</t>
         </is>
       </c>
-      <c r="J9" s="3">
+      <c r="M9" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mherrma1", "https://search.asu.edu/profile/mherrma1")</f>
         <v/>
       </c>
-      <c r="K9" s="3">
+      <c r="N9" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
@@ -945,19 +1039,34 @@
           <t>applied mathematics, fluid mechanics, turbulent mixing</t>
         </is>
       </c>
-      <c r="H10" s="2" t="b">
-        <v>1</v>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Modeling and Simulation, Oceanography, Earth Systems and Climate Science, Modeling, Modeling, Simulation and Cyberinfrastructure, Applied Mathematics</t>
+        </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
+          <t>Modeling and Simulation, Oceanography, Earth Systems and Climate Science, Modeling, Modeling, Simulation and Cyberinfrastructure, Applied Mathematics</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Scotti's main focus is theoretical, experimental and computational aspects of environmental fluid mechanics.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
           <t>HRx2lJQAAAAJ</t>
         </is>
       </c>
-      <c r="J10" s="3">
+      <c r="M10" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/adscotti", "https://search.asu.edu/profile/adscotti")</f>
         <v/>
       </c>
-      <c r="K10" s="3">
+      <c r="N10" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
@@ -995,19 +1104,30 @@
           <t>data-driven modeling, heat transfer, transport phenomena</t>
         </is>
       </c>
-      <c r="H11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Transport phenomena in heat transfer systems Additive manufacturing Data-driven modeling and design</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Kwon aims to improve the energy conversion and transport systems through the fundamental insights into transport physics, and by exploiting additive manufacturing and data-driven approaches.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>fs2d97sAAAAJ</t>
         </is>
       </c>
-      <c r="J11" s="3">
+      <c r="M11" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/bkwon2", "https://search.asu.edu/profile/bkwon2")</f>
         <v/>
       </c>
-      <c r="K11" s="3">
+      <c r="N11" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
@@ -1045,19 +1165,34 @@
           <t>aerodynamics, fluid-structure interaction, physics-informed machine learning</t>
         </is>
       </c>
-      <c r="H12" s="2" t="b">
-        <v>1</v>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+        </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Leixin Ma's career goal is a data-driven and physically consistent approach to modeling and designing programmable smart structures and robots, especially under complex fluid flow conditions.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
           <t>2xQTOc0AAAAJ</t>
         </is>
       </c>
-      <c r="J12" s="3">
+      <c r="M12" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
-      <c r="K12" s="3">
+      <c r="N12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
         <v/>
       </c>
@@ -1095,19 +1230,26 @@
           <t>fluid mechanics, high-performance computing, turbulence</t>
         </is>
       </c>
-      <c r="H13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Yulia Peet is an associate professor of aerospace and mechanical engineering in the School for Engineering of Matter, Transport and Energy with the Ira A. Fulton Schools of Engineering at Arizona State University. Her Ph.D. degree is in Aeronautics and Astronautics from Stanford (2006), M.S. and B.S. degrees are from Moscow Institute of Physics and Technology (1999 and 1997). Her previous appoi...</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>_6o8MrUAAAAJ</t>
         </is>
       </c>
-      <c r="J13" s="3">
+      <c r="M13" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="K13" s="3">
+      <c r="N13" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
@@ -1145,15 +1287,22 @@
           <t>fluid dynamics, numerical simulation</t>
         </is>
       </c>
-      <c r="H14" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="3">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Huang's research interests are geophysical and environmental fluid dynamics, numerical simulation of atmospheric and oceanic flows, Earth system remote sensing, and climate change.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hhuang38", "https://search.asu.edu/profile/hhuang38")</f>
         <v/>
       </c>
-      <c r="K14" s="3">
+      <c r="N14" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1191,15 +1340,22 @@
           <t>optimization, reduced-order modeling</t>
         </is>
       </c>
-      <c r="H15" s="2" t="b">
-        <v>1</v>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Structural Dynamics, Rotordynamics, Vibration Analysis, Reduced-Order Modeling, Optimization</t>
+        </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="3">
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rnmurthy", "https://search.asu.edu/profile/rnmurthy")</f>
         <v/>
       </c>
-      <c r="K15" s="3">
+      <c r="N15" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Raghavendra%20Murthy%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1237,19 +1393,34 @@
           <t>combustion, transition</t>
         </is>
       </c>
-      <c r="H16" s="2" t="b">
-        <v>1</v>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Energy management and efficiency, energy transition, energy storage, solid oxide fuel cells, partial oxidation, cogeneration, combustion, and synthesis of hydrogen</t>
+        </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
+          <t>Ceramics, Electrochemistry, Energy, Energy and Sustainability, Energy Conservation, Energy Economics, Energy Efficiency Technologies, Thin Film Materials</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Milcarek's current research focuses on energy management and efficiency, energy system modeling, energy transition, energy storage, solid oxide fuel cells fabrication and testing, partial oxidation and synthesis of hydrogen.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
           <t>m-Pb6g2pm2UC</t>
         </is>
       </c>
-      <c r="J16" s="3">
+      <c r="M16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="K16" s="3">
+      <c r="N16" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
         <v/>
       </c>
@@ -1287,15 +1458,22 @@
           <t>aerospace propulsion, propulsion</t>
         </is>
       </c>
-      <c r="H17" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="3">
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Lee's areas of expertise include energy system analysis, thermal and fluid process characterization, and fuel property measurements for energy systems.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/attwl", "https://search.asu.edu/profile/attwl")</f>
         <v/>
       </c>
-      <c r="K17" s="3">
+      <c r="N17" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1333,19 +1511,34 @@
           <t>computational physics</t>
         </is>
       </c>
-      <c r="H18" s="2" t="b">
-        <v>1</v>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Quantum simulations Machine learning Quantum computing</t>
+        </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
+          <t>Artificial Photosynthesis, Chemistry, Computational Physics, Machine Learning, Materials Science, Metals, Nanoscience, Semiconductors</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Houlong Zhuang is an associate professor in the School for Engineering of Matter, Transport and Energy at ASU. He received his doctorate in materials science and engineering at Cornell University. Prior to ASU, Dr. Zhuang was a postdoctoral researcher at Princeton University. Dr. Zhuang’s current research interests are quantum mechanical simulations, machine learning, and quantum computing.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
           <t>4yYKCpUAAAAJ</t>
         </is>
       </c>
-      <c r="J18" s="3">
+      <c r="M18" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hzhuang7", "https://search.asu.edu/profile/hzhuang7")</f>
         <v/>
       </c>
-      <c r="K18" s="3">
+      <c r="N18" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
@@ -1383,19 +1576,34 @@
           <t>computational physics</t>
         </is>
       </c>
-      <c r="H19" s="2" t="b">
-        <v>1</v>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace Engineering, Computational Physics, Energy, Material Physics, Materials Science, Mechanical Engineering, Modeling and Simulation, Theoretical Solid State Physics</t>
+        </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
+          <t>Aerospace Engineering, Computational Physics, Energy, Material Physics, Materials Science, Mechanical Engineering, Modeling and Simulation, Theoretical Solid State Physics</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Wu’s research focuses on electron, phonon, and magnon transport, exploring nanoscale energy transport and conversion through first-principles approaches, as well as material thermal and electrical transport properties.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
           <t>8CS4X9IAAAAJ</t>
         </is>
       </c>
-      <c r="J19" s="3">
+      <c r="M19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/huanwu", "https://search.asu.edu/profile/huanwu")</f>
         <v/>
       </c>
-      <c r="K19" s="3">
+      <c r="N19" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=8CS4X9IAAAAJ", "Scholar (8CS4X9IAAAAJ)")</f>
         <v/>
       </c>
@@ -1433,19 +1641,34 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H20" s="2" t="b">
-        <v>1</v>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Synthesis of nanocrystalline materials with tailored microstructures, Mechanics of nanostructured metal and alloy films, MEMS for in situ materials testing, Polymer based micro devices for cell mechanics and biohybrid platforms</t>
+        </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
+          <t>Thin Film Materials, Materials Science, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Rajagopalan's research focuses on the mechanics of nanoscale materials, cells and biological systems.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
           <t>ClqRIhIAAAAJ</t>
         </is>
       </c>
-      <c r="J20" s="3">
+      <c r="M20" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jrajago1", "https://search.asu.edu/profile/jrajago1")</f>
         <v/>
       </c>
-      <c r="K20" s="3">
+      <c r="N20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
         <v/>
       </c>
@@ -1483,15 +1706,26 @@
           <t>finite element</t>
         </is>
       </c>
-      <c r="H21" s="2" t="b">
-        <v>1</v>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Development of computational mechanics: finite element methods, molecular dynamics, multiscale methods, failure analysis, and material design.</t>
+        </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="3">
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Oswald develops computational and AI-driven methods for advanced manufacturing, including laser welding, automated inspection, robotics, and computational mechanics.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/joswald1", "https://search.asu.edu/profile/joswald1")</f>
         <v/>
       </c>
-      <c r="K21" s="3">
+      <c r="N21" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1529,19 +1763,34 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H22" s="2" t="b">
-        <v>1</v>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Distributed multi-agent motion planning and control, Provably safe control design using machine learning-based certificates, Foundation models in complex robotic tasks, Failure prediction from limited demonstrations, Human-robot interaction.</t>
+        </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
+          <t>Control Systems, Dynamical Systems, Machine Learning, Nonlinear Dynamical Systems, Robotics</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Garg's research interests include control synthesis for multi-agent coordination using control theory and machine learning.</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
           <t>vs3pl-8AAAAJ</t>
         </is>
       </c>
-      <c r="J22" s="3">
+      <c r="M22" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
         <v/>
       </c>
-      <c r="K22" s="3">
+      <c r="N22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
         <v/>
       </c>
@@ -1579,15 +1828,26 @@
           <t>heat transfer</t>
         </is>
       </c>
-      <c r="H23" s="2" t="b">
-        <v>1</v>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
+        </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="3">
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Wang research interests include selective control of thermal emission/absorption using meta-materials for energy harvesting and near-field radiation heat transfer enhancement between meta-materials for thermophotovoltaics.</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
         <v/>
       </c>
-      <c r="K23" s="3">
+      <c r="N23" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1625,15 +1885,30 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="3">
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>The intersection of computer science and control including convex optimization, artificial intelligence, and manipulation of delayed and PDE systems. The understanding and regulation of complex dynamical systems such as the motion of plasma in nuclear fusion reactors, autoregulation in the human immune response, and the motion of spacecraft in orbit.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Control Systems, Dynamical Systems Theory, Aerospace Engineering, Algorithm Development, Dynamical Systems, Nonlinear Dynamical Systems, Mathematical and System Dynamics Modeling, Immunology</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Peet's current research interests are in the role of computation as it is applied to the understanding and control of complex and large-scale systems.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mpeet", "https://search.asu.edu/profile/mpeet")</f>
         <v/>
       </c>
-      <c r="K24" s="3">
+      <c r="N24" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1671,19 +1946,30 @@
           <t>instability</t>
         </is>
       </c>
-      <c r="H25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Metal additive manufacturing, in-situ synchrotron X-ray and neutron characterization, non-equilibrium phase transformation, metal matrix composites. Selected Publications M. Qu , J. Yuan, Q. Guo, A. Nabaa, L. I. Escano, J. Huang, Q. Li, L. Chen. Achieving uniformly refined grain structure in metal additive manufacturing: Experimental demonstration and analytical model development. Additive Manufacturing 108 (2025) 104805. M. Qu , D. Yu, J. Yuan, L. Chen, K. An, Y. Chen. Multi-stage load partitioning in additively manufactured Al6061+TiC nanocomposite characterized by in-situ neutron diffraction. Additive Manufacturing, 96 (2024) 104584. M. Qu , J. Yuan, A. Nabaa, J. Huang, C. A. Chuang, L. Chen. Melting and solidification dynamics during laser additive manufacturing of reaction-based metal matrix composites uncovered by in-situ synchrotron X-ray diffraction. Acta Materialia , 271 (2024) 119875. M. Qu , Q. Guo, L. I. Escano, A. Nabaa, S. M. H. Hojjatzadeh, Z. A. Young, L. Chen. Controlling process instability for defect lean metal additive manufacturing. Nature Communications , 13 (2022) 1079. M. Qu , Q. Guo, L. I. Escano, A. Nabaa, K. Fezzaa, L. Chen. Nanoparticle-enabled increase of energy efficiency during laser metal additive manufacturing. Additive Manufacturing , 60 (2022) 103242. M. Qu , Q.Guo, L. I. Escano, J. Yuan, S. J. Clark, K. Fezzaa, L. Chen. Controlling melt flow by nanoparticles to eliminate surface wave induced surface fluctuation. Additive Manufacturing , 59 (2022) 103081.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Minglei Qu is an Assistant Professor of Mechanical Engineering and a graduate faculty of Materials Science and Engineering in the School for Engineering of Matter, Transport and Energy at ASU. His research lies at the intersection of metal additive manufacturing, in-situ characterization, and materials science. By utilizing advanced in-situ characterization tools, including synchrotron X-ray im...</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>9LWNC50AAAAJ</t>
         </is>
       </c>
-      <c r="J25" s="3">
+      <c r="M25" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mingleiq", "https://search.asu.edu/profile/mingleiq")</f>
         <v/>
       </c>
-      <c r="K25" s="3">
+      <c r="N25" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
@@ -1721,19 +2007,34 @@
           <t>heat transfer</t>
         </is>
       </c>
-      <c r="H26" s="2" t="b">
-        <v>1</v>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>My research group is an interdisciplinary nanoengineering team that focuses on manipulating material properties for thermal energy applications. Some of our focus areas are thermoelectric power generation, thermal storage media, heat transfer, and phonon optics. To achieve our objectives, we custom-design materials using colloidal nanoparticles, chemical precursors, and nanocomposites.</t>
+        </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
+          <t>Mechanical Engineering, Energy, Renewable Energy, Energy and Sustainability, Clean Energy, Energy Efficiency Technologies, Materials Science and Engineering, Chemical Engineering, Nanoengineering, Nanoscience, Nanotechnology, Solid State Physics, Thin Film Materials, Semiconductors, Chemistry, Physics</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Wang's research interests include thermal energy conversion, storage, and transport in nanostructured materials; thermoelectric power generation; thermal storage media; heat transfer, and phonon optics</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
           <t>LaUdx9gAAAAJ</t>
         </is>
       </c>
-      <c r="J26" s="3">
+      <c r="M26" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rywang", "https://search.asu.edu/profile/rywang")</f>
         <v/>
       </c>
-      <c r="K26" s="3">
+      <c r="N26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
         <v/>
       </c>
@@ -1771,15 +2072,22 @@
           <t>fluid dynamics</t>
         </is>
       </c>
-      <c r="H27" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="3">
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Calhoun’s research interests are in fluid dynamics; atmospheric sciences; boundary layer; wind energy and remote sensing.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcalhou", "https://search.asu.edu/profile/rcalhou")</f>
         <v/>
       </c>
-      <c r="K27" s="3">
+      <c r="N27" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1817,19 +2125,34 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H28" s="2" t="b">
-        <v>1</v>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Modeling, analysis, control, and optimization of multi-robot systems including robotic swarms; analysis of collective behaviors in biology and biologically-inspired control of distributed systems</t>
+        </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
+          <t>Systems and Control Theory, Mechanical Engineering, Autonomous Technologies, Robotics</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Berman directs the Autonomous Collective Systems Laboratory at ASU, which models and analyzes behaviors in biological and engineered collectives and designs control strategies for multi-robot systems.</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
           <t>KKup0OgAAAAJ</t>
         </is>
       </c>
-      <c r="J28" s="3">
+      <c r="M28" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="K28" s="3">
+      <c r="N28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
         <v/>
       </c>
@@ -1867,20 +2190,23 @@
           <t>heat transfer</t>
         </is>
       </c>
-      <c r="H29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>OmBV67MAAAAJ</t>
-        </is>
-      </c>
-      <c r="J29" s="3">
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Yang studies heat transfer, thermal management of electronics, and biomedical devices. She has published multiple research papers in major scientific journals.</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="K29" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
+      <c r="N29" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
     </row>
@@ -1917,15 +2243,22 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H30" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="3">
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Ren’s current research interests include optimization, product/configuration design, human-computer interaction and machine learning.</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yren32", "https://search.asu.edu/profile/yren32")</f>
         <v/>
       </c>
-      <c r="K30" s="3">
+      <c r="N30" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1963,15 +2296,26 @@
           <t>uncertainty quantification</t>
         </is>
       </c>
-      <c r="H31" s="2" t="b">
-        <v>1</v>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Yongming Liu is a professor of aerospace and mechanical engineering with the School for Engineering of Matter, Transport and Energy at Arizona State University. Fatigue and fracture of engineering materials and structures, probabilistic computational mechanics, risk assessment and management, multi-physics damage modeling and structural durability, multi-scale uncertainty quantification and propagation, imaging-based experimental testing, diagnostics and prognostics</t>
+        </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="3">
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Liu heads the Prognostic Analysis and Reliability Assessment Laboratory (PARA). He joined ASU in 2012.</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yliu35", "https://search.asu.edu/profile/yliu35")</f>
         <v/>
       </c>
-      <c r="K31" s="3">
+      <c r="N31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -1979,95 +2323,95 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2079,7 +2423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2089,10 +2433,13 @@
     <col width="49" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="49" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="49" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2133,20 +2480,35 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Research Interests</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Expertise Areas</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Research / Bio Summary</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Scholar ID</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Profile URL</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Google Scholar URL</t>
         </is>
@@ -2155,12 +2517,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Werner Dahm</t>
+          <t>Jeonglae Kim</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SUM/WTR Faculty Research</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2174,7 +2536,7 @@
         </is>
       </c>
       <c r="E2" s="3">
-        <f>HYPERLINK("mailto:Werner.Dahm@asu.edu", "Werner.Dahm@asu.edu")</f>
+        <f>HYPERLINK("mailto:jeokim@asu.edu", "jeokim@asu.edu")</f>
         <v/>
       </c>
       <c r="F2" s="2" t="n">
@@ -2182,31 +2544,38 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>combustion, computational physics, fluid dynamics, heat transfer, propulsion, turbulence</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="b">
-        <v>1</v>
-      </c>
+          <t>aeroacoustics, flow control, high-performance computing, optimization, turbulence, turbulent flows</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/wdahm", "https://search.asu.edu/profile/wdahm")</f>
-        <v/>
-      </c>
-      <c r="K2" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University", "Google Scholar Search")</f>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Kim's research interests include large-eddy simulation of high-speed turbulent flows with multi-physics, aeroacoustics, flow control and optimization.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="3">
+        <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
+        <v/>
+      </c>
+      <c r="N2" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Jeonglae Kim</t>
+          <t>Werner Dahm</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>SUM/WTR Faculty Research</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2220,27 +2589,42 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <f>HYPERLINK("mailto:jeokim@asu.edu", "jeokim@asu.edu")</f>
+        <f>HYPERLINK("mailto:Werner.Dahm@asu.edu", "Werner.Dahm@asu.edu")</f>
         <v/>
       </c>
       <c r="F3" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>aeroacoustics, flow control, optimization, turbulence, turbulent flows</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
-        <v/>
-      </c>
-      <c r="K3" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
+          <t>combustion, computational physics, fluid dynamics, heat transfer, propulsion, turbulence</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Dahm specializes in fluid dynamics, thermodynamics, combustion, heat transfer, thermal sciences, propulsion, fuel efficiency, emissions, powertrains, and other areas relevant to a broad range of automotive, aerospace, and industrial applications. He is an author of over 200 refereed technical articles, conference papers, and technical publications, a holder of six U.S. and international patents, and has given over 260 technical presentations, including over 190 invited, plenary, and keynote lectures worldwide, on topics dealing with mechanical and aerospace engineering and defense science.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace Engineering, Applied Research, Computational Modeling, Computational Physics, Mechanical Engineering, Propulsion</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Werner J.A. Dahm has since 2010 been the ASU Foundation Professor of Mechanical and Aerospace Engineering, and also Professor Emeritus of Engineering at the University of Michigan where served for the previous 25 years.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="3">
+        <f>HYPERLINK("https://search.asu.edu/profile/wdahm", "https://search.asu.edu/profile/wdahm")</f>
+        <v/>
+      </c>
+      <c r="N3" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
     </row>
@@ -2277,19 +2661,26 @@
           <t>computational fluid dynamics, drag reduction, fluid dynamics, fluid mechanics, multiphase flow</t>
         </is>
       </c>
-      <c r="H4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Chen’s research interests include multiphase flows, drag reduction, airplane de-icing, interfacial instabilities and flow in porous media.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>xT-lX9sAAAAJ</t>
         </is>
       </c>
-      <c r="J4" s="3">
+      <c r="M4" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="K4" s="3">
+      <c r="N4" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
@@ -2327,19 +2718,30 @@
           <t>aerodynamics, flow control, fluid dynamics, turbulence, vortex dynamics</t>
         </is>
       </c>
-      <c r="H5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Unsteady aerodynamics, vortex dynamics, flow control, turbulence, separated flows</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Ramesh's expertise is in unsteady fluid dynamics, vortex dynamics, turbulence and flow control.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>DKc-AgcAAAAJ</t>
         </is>
       </c>
-      <c r="J5" s="3">
+      <c r="M5" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kramesh2", "https://search.asu.edu/profile/kramesh2")</f>
         <v/>
       </c>
-      <c r="K5" s="3">
+      <c r="N5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
         <v/>
       </c>
@@ -2377,15 +2779,22 @@
           <t>cfd, computational fluid dynamics, dns, fluid dynamics, multiphase flow</t>
         </is>
       </c>
-      <c r="H6" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="3">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Kasbaoui's research interests include computational fluid dynamics, numerical methods, and massively parallel simulations of multiphase and particle-laden flows for environmental and aerospace applications.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
         <v/>
       </c>
-      <c r="K6" s="3">
+      <c r="N6" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -2423,19 +2832,26 @@
           <t>inverse problems, multiscale modeling, optimization, transition</t>
         </is>
       </c>
-      <c r="H7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Chattopadhyay is the director of Adaptive Intelligent Materials and Systems (AIMS) Center at ASU. Her research focuses on structural health monitoring and damage prognosis, and multidisciplinary design optimization.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>w3fU9E0AAAAJ</t>
         </is>
       </c>
-      <c r="J7" s="3">
+      <c r="M7" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/chattopa", "https://search.asu.edu/profile/chattopa")</f>
         <v/>
       </c>
-      <c r="K7" s="3">
+      <c r="N7" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
@@ -2473,15 +2889,30 @@
           <t>aerodynamics, reacting flows, turbulence, turbulent mixing</t>
         </is>
       </c>
-      <c r="H8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="3">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Pathikonda studies turbulent fluid flows to understand natural and engineering phenomena using lab experiments. His expertise is in complex (reacting) mixing, high Re-flows, laser-based &amp; spectroscopic techniques, etc.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
         <v/>
       </c>
-      <c r="K8" s="3">
+      <c r="N8" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -2519,19 +2950,26 @@
           <t>fluid mechanics, multiphase flow, numerical simulation, turbulence</t>
         </is>
       </c>
-      <c r="H9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Herrmann's research interests include fluid mechanics, modeling and numerical simulation of multiphase flows with a focus on turbulent atomization processes, and numerical methods for discontinuous interfaces.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>yv6aCW8AAAAJ</t>
         </is>
       </c>
-      <c r="J9" s="3">
+      <c r="M9" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mherrma1", "https://search.asu.edu/profile/mherrma1")</f>
         <v/>
       </c>
-      <c r="K9" s="3">
+      <c r="N9" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
@@ -2569,19 +3007,34 @@
           <t>applied mathematics, fluid mechanics, turbulent mixing</t>
         </is>
       </c>
-      <c r="H10" s="2" t="b">
-        <v>1</v>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Modeling and Simulation, Oceanography, Earth Systems and Climate Science, Modeling, Modeling, Simulation and Cyberinfrastructure, Applied Mathematics</t>
+        </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
+          <t>Modeling and Simulation, Oceanography, Earth Systems and Climate Science, Modeling, Modeling, Simulation and Cyberinfrastructure, Applied Mathematics</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Scotti's main focus is theoretical, experimental and computational aspects of environmental fluid mechanics.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
           <t>HRx2lJQAAAAJ</t>
         </is>
       </c>
-      <c r="J10" s="3">
+      <c r="M10" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/adscotti", "https://search.asu.edu/profile/adscotti")</f>
         <v/>
       </c>
-      <c r="K10" s="3">
+      <c r="N10" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
@@ -2619,19 +3072,30 @@
           <t>data-driven modeling, heat transfer, transport phenomena</t>
         </is>
       </c>
-      <c r="H11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Transport phenomena in heat transfer systems Additive manufacturing Data-driven modeling and design</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Kwon aims to improve the energy conversion and transport systems through the fundamental insights into transport physics, and by exploiting additive manufacturing and data-driven approaches.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>fs2d97sAAAAJ</t>
         </is>
       </c>
-      <c r="J11" s="3">
+      <c r="M11" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/bkwon2", "https://search.asu.edu/profile/bkwon2")</f>
         <v/>
       </c>
-      <c r="K11" s="3">
+      <c r="N11" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
@@ -2669,19 +3133,34 @@
           <t>aerodynamics, fluid-structure interaction, physics-informed machine learning</t>
         </is>
       </c>
-      <c r="H12" s="2" t="b">
-        <v>1</v>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+        </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Leixin Ma's career goal is a data-driven and physically consistent approach to modeling and designing programmable smart structures and robots, especially under complex fluid flow conditions.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
           <t>2xQTOc0AAAAJ</t>
         </is>
       </c>
-      <c r="J12" s="3">
+      <c r="M12" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
-      <c r="K12" s="3">
+      <c r="N12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
         <v/>
       </c>
@@ -2719,19 +3198,26 @@
           <t>fluid mechanics, high-performance computing, turbulence</t>
         </is>
       </c>
-      <c r="H13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Yulia Peet is an associate professor of aerospace and mechanical engineering in the School for Engineering of Matter, Transport and Energy with the Ira A. Fulton Schools of Engineering at Arizona State University. Her Ph.D. degree is in Aeronautics and Astronautics from Stanford (2006), M.S. and B.S. degrees are from Moscow Institute of Physics and Technology (1999 and 1997). Her previous appoi...</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>_6o8MrUAAAAJ</t>
         </is>
       </c>
-      <c r="J13" s="3">
+      <c r="M13" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="K13" s="3">
+      <c r="N13" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
@@ -2769,15 +3255,22 @@
           <t>fluid dynamics, numerical simulation</t>
         </is>
       </c>
-      <c r="H14" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="3">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Huang's research interests are geophysical and environmental fluid dynamics, numerical simulation of atmospheric and oceanic flows, Earth system remote sensing, and climate change.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hhuang38", "https://search.asu.edu/profile/hhuang38")</f>
         <v/>
       </c>
-      <c r="K14" s="3">
+      <c r="N14" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -2815,15 +3308,22 @@
           <t>optimization, reduced-order modeling</t>
         </is>
       </c>
-      <c r="H15" s="2" t="b">
-        <v>1</v>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Structural Dynamics, Rotordynamics, Vibration Analysis, Reduced-Order Modeling, Optimization</t>
+        </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="3">
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rnmurthy", "https://search.asu.edu/profile/rnmurthy")</f>
         <v/>
       </c>
-      <c r="K15" s="3">
+      <c r="N15" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Raghavendra%20Murthy%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -2861,19 +3361,34 @@
           <t>combustion, transition</t>
         </is>
       </c>
-      <c r="H16" s="2" t="b">
-        <v>1</v>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Energy management and efficiency, energy transition, energy storage, solid oxide fuel cells, partial oxidation, cogeneration, combustion, and synthesis of hydrogen</t>
+        </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
+          <t>Ceramics, Electrochemistry, Energy, Energy and Sustainability, Energy Conservation, Energy Economics, Energy Efficiency Technologies, Thin Film Materials</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Milcarek's current research focuses on energy management and efficiency, energy system modeling, energy transition, energy storage, solid oxide fuel cells fabrication and testing, partial oxidation and synthesis of hydrogen.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
           <t>m-Pb6g2pm2UC</t>
         </is>
       </c>
-      <c r="J16" s="3">
+      <c r="M16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="K16" s="3">
+      <c r="N16" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
         <v/>
       </c>
@@ -2911,15 +3426,22 @@
           <t>aerospace propulsion, propulsion</t>
         </is>
       </c>
-      <c r="H17" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="3">
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Lee's areas of expertise include energy system analysis, thermal and fluid process characterization, and fuel property measurements for energy systems.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/attwl", "https://search.asu.edu/profile/attwl")</f>
         <v/>
       </c>
-      <c r="K17" s="3">
+      <c r="N17" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -2957,19 +3479,34 @@
           <t>computational physics</t>
         </is>
       </c>
-      <c r="H18" s="2" t="b">
-        <v>1</v>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Quantum simulations Machine learning Quantum computing</t>
+        </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
+          <t>Artificial Photosynthesis, Chemistry, Computational Physics, Machine Learning, Materials Science, Metals, Nanoscience, Semiconductors</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Houlong Zhuang is an associate professor in the School for Engineering of Matter, Transport and Energy at ASU. He received his doctorate in materials science and engineering at Cornell University. Prior to ASU, Dr. Zhuang was a postdoctoral researcher at Princeton University. Dr. Zhuang’s current research interests are quantum mechanical simulations, machine learning, and quantum computing.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
           <t>4yYKCpUAAAAJ</t>
         </is>
       </c>
-      <c r="J18" s="3">
+      <c r="M18" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hzhuang7", "https://search.asu.edu/profile/hzhuang7")</f>
         <v/>
       </c>
-      <c r="K18" s="3">
+      <c r="N18" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
@@ -3007,19 +3544,34 @@
           <t>computational physics</t>
         </is>
       </c>
-      <c r="H19" s="2" t="b">
-        <v>1</v>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace Engineering, Computational Physics, Energy, Material Physics, Materials Science, Mechanical Engineering, Modeling and Simulation, Theoretical Solid State Physics</t>
+        </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
+          <t>Aerospace Engineering, Computational Physics, Energy, Material Physics, Materials Science, Mechanical Engineering, Modeling and Simulation, Theoretical Solid State Physics</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Wu’s research focuses on electron, phonon, and magnon transport, exploring nanoscale energy transport and conversion through first-principles approaches, as well as material thermal and electrical transport properties.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
           <t>8CS4X9IAAAAJ</t>
         </is>
       </c>
-      <c r="J19" s="3">
+      <c r="M19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/huanwu", "https://search.asu.edu/profile/huanwu")</f>
         <v/>
       </c>
-      <c r="K19" s="3">
+      <c r="N19" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=8CS4X9IAAAAJ", "Scholar (8CS4X9IAAAAJ)")</f>
         <v/>
       </c>
@@ -3057,19 +3609,34 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H20" s="2" t="b">
-        <v>1</v>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Synthesis of nanocrystalline materials with tailored microstructures, Mechanics of nanostructured metal and alloy films, MEMS for in situ materials testing, Polymer based micro devices for cell mechanics and biohybrid platforms</t>
+        </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
+          <t>Thin Film Materials, Materials Science, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Rajagopalan's research focuses on the mechanics of nanoscale materials, cells and biological systems.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
           <t>ClqRIhIAAAAJ</t>
         </is>
       </c>
-      <c r="J20" s="3">
+      <c r="M20" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jrajago1", "https://search.asu.edu/profile/jrajago1")</f>
         <v/>
       </c>
-      <c r="K20" s="3">
+      <c r="N20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
         <v/>
       </c>
@@ -3107,15 +3674,26 @@
           <t>finite element</t>
         </is>
       </c>
-      <c r="H21" s="2" t="b">
-        <v>1</v>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Development of computational mechanics: finite element methods, molecular dynamics, multiscale methods, failure analysis, and material design.</t>
+        </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="3">
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Oswald develops computational and AI-driven methods for advanced manufacturing, including laser welding, automated inspection, robotics, and computational mechanics.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/joswald1", "https://search.asu.edu/profile/joswald1")</f>
         <v/>
       </c>
-      <c r="K21" s="3">
+      <c r="N21" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3153,19 +3731,34 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H22" s="2" t="b">
-        <v>1</v>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Distributed multi-agent motion planning and control, Provably safe control design using machine learning-based certificates, Foundation models in complex robotic tasks, Failure prediction from limited demonstrations, Human-robot interaction.</t>
+        </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
+          <t>Control Systems, Dynamical Systems, Machine Learning, Nonlinear Dynamical Systems, Robotics</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Garg's research interests include control synthesis for multi-agent coordination using control theory and machine learning.</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
           <t>vs3pl-8AAAAJ</t>
         </is>
       </c>
-      <c r="J22" s="3">
+      <c r="M22" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
         <v/>
       </c>
-      <c r="K22" s="3">
+      <c r="N22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
         <v/>
       </c>
@@ -3203,15 +3796,26 @@
           <t>heat transfer</t>
         </is>
       </c>
-      <c r="H23" s="2" t="b">
-        <v>1</v>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
+        </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="3">
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Wang research interests include selective control of thermal emission/absorption using meta-materials for energy harvesting and near-field radiation heat transfer enhancement between meta-materials for thermophotovoltaics.</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
         <v/>
       </c>
-      <c r="K23" s="3">
+      <c r="N23" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3249,15 +3853,30 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="3">
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>The intersection of computer science and control including convex optimization, artificial intelligence, and manipulation of delayed and PDE systems. The understanding and regulation of complex dynamical systems such as the motion of plasma in nuclear fusion reactors, autoregulation in the human immune response, and the motion of spacecraft in orbit.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Control Systems, Dynamical Systems Theory, Aerospace Engineering, Algorithm Development, Dynamical Systems, Nonlinear Dynamical Systems, Mathematical and System Dynamics Modeling, Immunology</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Peet's current research interests are in the role of computation as it is applied to the understanding and control of complex and large-scale systems.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mpeet", "https://search.asu.edu/profile/mpeet")</f>
         <v/>
       </c>
-      <c r="K24" s="3">
+      <c r="N24" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3295,19 +3914,30 @@
           <t>instability</t>
         </is>
       </c>
-      <c r="H25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Metal additive manufacturing, in-situ synchrotron X-ray and neutron characterization, non-equilibrium phase transformation, metal matrix composites. Selected Publications M. Qu , J. Yuan, Q. Guo, A. Nabaa, L. I. Escano, J. Huang, Q. Li, L. Chen. Achieving uniformly refined grain structure in metal additive manufacturing: Experimental demonstration and analytical model development. Additive Manufacturing 108 (2025) 104805. M. Qu , D. Yu, J. Yuan, L. Chen, K. An, Y. Chen. Multi-stage load partitioning in additively manufactured Al6061+TiC nanocomposite characterized by in-situ neutron diffraction. Additive Manufacturing, 96 (2024) 104584. M. Qu , J. Yuan, A. Nabaa, J. Huang, C. A. Chuang, L. Chen. Melting and solidification dynamics during laser additive manufacturing of reaction-based metal matrix composites uncovered by in-situ synchrotron X-ray diffraction. Acta Materialia , 271 (2024) 119875. M. Qu , Q. Guo, L. I. Escano, A. Nabaa, S. M. H. Hojjatzadeh, Z. A. Young, L. Chen. Controlling process instability for defect lean metal additive manufacturing. Nature Communications , 13 (2022) 1079. M. Qu , Q. Guo, L. I. Escano, A. Nabaa, K. Fezzaa, L. Chen. Nanoparticle-enabled increase of energy efficiency during laser metal additive manufacturing. Additive Manufacturing , 60 (2022) 103242. M. Qu , Q.Guo, L. I. Escano, J. Yuan, S. J. Clark, K. Fezzaa, L. Chen. Controlling melt flow by nanoparticles to eliminate surface wave induced surface fluctuation. Additive Manufacturing , 59 (2022) 103081.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Minglei Qu is an Assistant Professor of Mechanical Engineering and a graduate faculty of Materials Science and Engineering in the School for Engineering of Matter, Transport and Energy at ASU. His research lies at the intersection of metal additive manufacturing, in-situ characterization, and materials science. By utilizing advanced in-situ characterization tools, including synchrotron X-ray im...</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>9LWNC50AAAAJ</t>
         </is>
       </c>
-      <c r="J25" s="3">
+      <c r="M25" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mingleiq", "https://search.asu.edu/profile/mingleiq")</f>
         <v/>
       </c>
-      <c r="K25" s="3">
+      <c r="N25" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
@@ -3345,19 +3975,34 @@
           <t>heat transfer</t>
         </is>
       </c>
-      <c r="H26" s="2" t="b">
-        <v>1</v>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>My research group is an interdisciplinary nanoengineering team that focuses on manipulating material properties for thermal energy applications. Some of our focus areas are thermoelectric power generation, thermal storage media, heat transfer, and phonon optics. To achieve our objectives, we custom-design materials using colloidal nanoparticles, chemical precursors, and nanocomposites.</t>
+        </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
+          <t>Mechanical Engineering, Energy, Renewable Energy, Energy and Sustainability, Clean Energy, Energy Efficiency Technologies, Materials Science and Engineering, Chemical Engineering, Nanoengineering, Nanoscience, Nanotechnology, Solid State Physics, Thin Film Materials, Semiconductors, Chemistry, Physics</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Wang's research interests include thermal energy conversion, storage, and transport in nanostructured materials; thermoelectric power generation; thermal storage media; heat transfer, and phonon optics</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
           <t>LaUdx9gAAAAJ</t>
         </is>
       </c>
-      <c r="J26" s="3">
+      <c r="M26" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rywang", "https://search.asu.edu/profile/rywang")</f>
         <v/>
       </c>
-      <c r="K26" s="3">
+      <c r="N26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
         <v/>
       </c>
@@ -3395,15 +4040,22 @@
           <t>fluid dynamics</t>
         </is>
       </c>
-      <c r="H27" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="3">
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Calhoun’s research interests are in fluid dynamics; atmospheric sciences; boundary layer; wind energy and remote sensing.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcalhou", "https://search.asu.edu/profile/rcalhou")</f>
         <v/>
       </c>
-      <c r="K27" s="3">
+      <c r="N27" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3441,19 +4093,34 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H28" s="2" t="b">
-        <v>1</v>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Modeling, analysis, control, and optimization of multi-robot systems including robotic swarms; analysis of collective behaviors in biology and biologically-inspired control of distributed systems</t>
+        </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
+          <t>Systems and Control Theory, Mechanical Engineering, Autonomous Technologies, Robotics</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Berman directs the Autonomous Collective Systems Laboratory at ASU, which models and analyzes behaviors in biological and engineered collectives and designs control strategies for multi-robot systems.</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
           <t>KKup0OgAAAAJ</t>
         </is>
       </c>
-      <c r="J28" s="3">
+      <c r="M28" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="K28" s="3">
+      <c r="N28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
         <v/>
       </c>
@@ -3491,20 +4158,23 @@
           <t>heat transfer</t>
         </is>
       </c>
-      <c r="H29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>OmBV67MAAAAJ</t>
-        </is>
-      </c>
-      <c r="J29" s="3">
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Yang studies heat transfer, thermal management of electronics, and biomedical devices. She has published multiple research papers in major scientific journals.</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="K29" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
+      <c r="N29" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
     </row>
@@ -3541,15 +4211,22 @@
           <t>optimization</t>
         </is>
       </c>
-      <c r="H30" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="3">
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Ren’s current research interests include optimization, product/configuration design, human-computer interaction and machine learning.</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yren32", "https://search.asu.edu/profile/yren32")</f>
         <v/>
       </c>
-      <c r="K30" s="3">
+      <c r="N30" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3587,15 +4264,26 @@
           <t>uncertainty quantification</t>
         </is>
       </c>
-      <c r="H31" s="2" t="b">
-        <v>1</v>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Yongming Liu is a professor of aerospace and mechanical engineering with the School for Engineering of Matter, Transport and Energy at Arizona State University. Fatigue and fracture of engineering materials and structures, probabilistic computational mechanics, risk assessment and management, multi-physics damage modeling and structural durability, multi-scale uncertainty quantification and propagation, imaging-based experimental testing, diagnostics and prognostics</t>
+        </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="3">
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Liu heads the Prognostic Analysis and Reliability Assessment Laboratory (PARA). He joined ASU in 2012.</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yliu35", "https://search.asu.edu/profile/yliu35")</f>
         <v/>
       </c>
-      <c r="K31" s="3">
+      <c r="N31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3629,15 +4317,18 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="b">
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="3">
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/astefan9", "https://search.asu.edu/profile/astefan9")</f>
         <v/>
       </c>
-      <c r="K32" s="3">
+      <c r="N32" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Aikaterini%20Stefanaki%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3671,19 +4362,34 @@
         <v>0</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="b">
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Biomimetic Additive Manufacturing (3D Printing); Bioinspired Material and Structure Design; Stereolithography; Photopolymerization based 3D Printing; Multi-material and Multi-scale 3D printing; Biofabrication; Biomaterial; Ceramic Printing; Nanocomposite Printing; Physical Field Assisted Printing; 4D Printing; Flexible Sensor; Biomedical Device; Tissue Repair and Regeneration.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Ceramic Technology, Mechanics of Composite Materials, Mechanical Engineering, Biomimicry, 3D Printing, Additive Manufacturing, Manufacturing Engineering</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Xiangjia (Cindy) Li is an Associate Professor at Arizona State University. Her research focuses on multiscale, multimaterial additive manufacturing and bioinspired design for functional materials and devices.</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>tGQzHJIAAAAJ</t>
         </is>
       </c>
-      <c r="J33" s="3">
+      <c r="M33" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xiangji5", "https://search.asu.edu/profile/xiangji5")</f>
         <v/>
       </c>
-      <c r="K33" s="3">
+      <c r="N33" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=tGQzHJIAAAAJ", "Scholar (tGQzHJIAAAAJ)")</f>
         <v/>
       </c>
@@ -3717,15 +4423,18 @@
         <v>0</v>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="b">
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="3">
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/dspeaks2", "https://search.asu.edu/profile/dspeaks2")</f>
         <v/>
       </c>
-      <c r="K34" s="3">
+      <c r="N34" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Derrick%20Speaks%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3759,15 +4468,18 @@
         <v>0</v>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="b">
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="3">
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ejande22", "https://search.asu.edu/profile/ejande22")</f>
         <v/>
       </c>
-      <c r="K35" s="3">
+      <c r="N35" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Erik%20Andersen%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3801,19 +4513,30 @@
         <v>0</v>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="b">
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Bio-inspired robotics Soft robotics Magnetic micro-robotics Mechanics of animal locomotion</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Marvi would like to develop bio-inspired robotic systems and programmable interfacial structures for search and rescue, exploratory and medical applications.</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>00Fepb0AAAAJ</t>
         </is>
       </c>
-      <c r="J36" s="3">
+      <c r="M36" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hmarvi", "https://search.asu.edu/profile/hmarvi")</f>
         <v/>
       </c>
-      <c r="K36" s="3">
+      <c r="N36" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=00Fepb0AAAAJ", "Scholar (00Fepb0AAAAJ)")</f>
         <v/>
       </c>
@@ -3847,15 +4570,22 @@
         <v>0</v>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="b">
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Lee's research interests include physical human-robot interaction, neuromuscular control of human movement, robot-aided neurorehabilitation, bio-inspired robotics and system identification for physiological systems.</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="3">
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hlee234", "https://search.asu.edu/profile/hlee234")</f>
         <v/>
       </c>
-      <c r="K37" s="3">
+      <c r="N37" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3889,15 +4619,18 @@
         <v>0</v>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="b">
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="3">
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/iychang", "https://search.asu.edu/profile/iychang")</f>
         <v/>
       </c>
-      <c r="K38" s="3">
+      <c r="N38" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ivy%20Chang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3931,15 +4664,26 @@
         <v>0</v>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="b">
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Student learning of mathematical concepts. Motivation and mathematics learning. Teacher change. Applications of technology to mathematics teaching and learning.</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Middleton’s research interests focus in the following areas where he has published extensively: children’s mathematical thinking; teacher and student motivation in mathematics; and teacher change in mathematics.</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="3">
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jimbo", "https://search.asu.edu/profile/jimbo")</f>
         <v/>
       </c>
-      <c r="K39" s="3">
+      <c r="N39" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -3973,19 +4717,34 @@
         <v>0</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="b">
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Hire students to conduct research https://sunroboticslab.github.io</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous Technologies, Control Systems, Mechanical Engineering, Robotics</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Sun's research focuses on the design, dynamics, and control of soft robots and artificial muscles</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>fjUoHOsAAAAJ</t>
         </is>
       </c>
-      <c r="J40" s="3">
+      <c r="M40" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jsun165", "https://search.asu.edu/profile/jsun165")</f>
         <v/>
       </c>
-      <c r="K40" s="3">
+      <c r="N40" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fjUoHOsAAAAJ", "Scholar (fjUoHOsAAAAJ)")</f>
         <v/>
       </c>
@@ -4019,15 +4778,18 @@
         <v>0</v>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="b">
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="3">
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jdwilbu1", "https://search.asu.edu/profile/jdwilbu1")</f>
         <v/>
       </c>
-      <c r="K41" s="3">
+      <c r="N41" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Joshua%20Wilbur%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4061,19 +4823,26 @@
         <v>0</v>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="b">
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Rykaczewski's research focuses on development of soft thermal materials and system as well as studying human thermal exposure in extreme heat.</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>SWeAf4UAAAAJ</t>
         </is>
       </c>
-      <c r="J42" s="3">
+      <c r="M42" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/krykacze", "https://search.asu.edu/profile/krykacze")</f>
         <v/>
       </c>
-      <c r="K42" s="3">
+      <c r="N42" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SWeAf4UAAAAJ", "Scholar (SWeAf4UAAAAJ)")</f>
         <v/>
       </c>
@@ -4107,15 +4876,30 @@
         <v>0</v>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="b">
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing process simulation and modeling and experiments Additive manufacturing Micro/nano manufacturing Microelectronic packaging Application of AI in manufacturing Mechanic of metallic materials Materials characterization Fatigue and damage modeling and simulation</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Additive Manufacturing, Manufacturing Engineering</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Ladani is a Professor of Mechanical and Aerospace Engineering at Arizona State University.</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="3">
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ljannesa", "https://search.asu.edu/profile/ljannesa")</f>
         <v/>
       </c>
-      <c r="K43" s="3">
+      <c r="N43" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4149,15 +4933,22 @@
         <v>0</v>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="b">
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Li uses multiscale material mechanics models, computational and data tools to explore advanced materials for extreme environments.</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="3">
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/linli25", "https://search.asu.edu/profile/linli25")</f>
         <v/>
       </c>
-      <c r="K44" s="3">
+      <c r="N44" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4191,15 +4982,22 @@
         <v>0</v>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="b">
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Mignolet's research interests include structural dynamics, vibrations, modeling of uncertainty in structures and stochastic multiscale analyses.</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="3">
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/marc03", "https://search.asu.edu/profile/marc03")</f>
         <v/>
       </c>
-      <c r="K45" s="3">
+      <c r="N45" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4233,15 +5031,30 @@
         <v>0</v>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="b">
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Thermal engineering, sustainable energy systems, energy management, sustainable cooling systems.</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Building Technology, Solar Energy Systems, Energy Efficiency Technologies, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Phelan researches and teaches in the area of sustainable energy, thermal transport and thermal management.</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="3">
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pphelan", "https://search.asu.edu/profile/pphelan")</f>
         <v/>
       </c>
-      <c r="K46" s="3">
+      <c r="N46" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4275,15 +5088,22 @@
         <v>0</v>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="b">
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Peralta's research focuses on mechanics of materials, fatigue and fracture of metallic alloys, dynamic and shock loading of metallic and intermetallic materials.</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="3">
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pperalta", "https://search.asu.edu/profile/pperalta")</f>
         <v/>
       </c>
-      <c r="K47" s="3">
+      <c r="N47" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Pedro%20Peralta%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4317,15 +5137,30 @@
         <v>0</v>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="b">
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Nanomanufacturing, additive manufacturing, laser-based material processing, laser matter interaction and physics simulation; inkjet printing of functional materials; and 2D materials fabrication for energy storage and bio-sensors.</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Additive Manufacturing, Manufacturing Engineering, Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Nian's research interests include additive manufacturing, laser-based manufacturing and material processing, laser matter interaction and physics simulation, and functional materials for energy storage and bio-sensors.</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="3">
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/qnian", "https://search.asu.edu/profile/qnian")</f>
         <v/>
       </c>
-      <c r="K48" s="3">
+      <c r="N48" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4359,15 +5194,18 @@
         <v>0</v>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="b">
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I49" s="2" t="inlineStr"/>
-      <c r="J49" s="3">
+      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcruzloz", "https://search.asu.edu/profile/rcruzloz")</f>
         <v/>
       </c>
-      <c r="K49" s="3">
+      <c r="N49" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ricardo%20Cruz%20Lozano%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4401,15 +5239,22 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="b">
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Seetharaman's is the director of EPIXC. His research and teaching interests lie in metals and ceramics. He is also engaged in developing materials for harsh conditions.</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="3">
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/sseeth11", "https://search.asu.edu/profile/sseeth11")</f>
         <v/>
       </c>
-      <c r="K50" s="3">
+      <c r="N50" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Sridhar%20Seetharaman%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4443,15 +5288,18 @@
         <v>0</v>
       </c>
       <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="b">
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="3">
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/skosara2", "https://search.asu.edu/profile/skosara2")</f>
         <v/>
       </c>
-      <c r="K51" s="3">
+      <c r="N51" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Srinivas%20Chakravarthi%20Kosaraju%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4485,19 +5333,30 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="b">
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>https://irislab.tech/</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Jin's research includes robotics, control and machine learning, with a focus on the autonomy of robots interacting with humans and objects.</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>SoEC4h4AAAAJ</t>
         </is>
       </c>
-      <c r="J52" s="3">
+      <c r="M52" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wjin34", "https://search.asu.edu/profile/wjin34")</f>
         <v/>
       </c>
-      <c r="K52" s="3">
+      <c r="N52" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SoEC4h4AAAAJ", "Scholar (SoEC4h4AAAAJ)")</f>
         <v/>
       </c>
@@ -4531,19 +5390,34 @@
         <v>0</v>
       </c>
       <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="b">
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Mechanics of Composite Materials, Micro and Nanoscale Bioengineering, Nanotechnology, Thin Film Materials</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Mechanics of Composite Materials, Micro and Nanoscale Bioengineering, Nanotechnology, Thin Film Materials</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Kang's current research interests include functional materials for energy/manufacturing applications and biomaterials/biomechanics for injury and wound healing mechanisms.</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="L53" s="2" t="inlineStr">
         <is>
           <t>bHyyOTAAAAAJ</t>
         </is>
       </c>
-      <c r="J53" s="3">
+      <c r="M53" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wkang16", "https://search.asu.edu/profile/wkang16")</f>
         <v/>
       </c>
-      <c r="K53" s="3">
+      <c r="N53" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=bHyyOTAAAAAJ", "Scholar (bHyyOTAAAAAJ)")</f>
         <v/>
       </c>
@@ -4577,15 +5451,30 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="b">
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>The research interests include control theory, machine learning, formal methods and autonomous systems.</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence, Control Systems, Electric Power and Energy Systems, Machine Learning, Robotics, Systems and Control Theory</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>My research interests include control theory, formal methods, and machine learning (including reinforcement learning), with applications on autonomous systems and cyber-physical systems.</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="3">
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xzhe1", "https://search.asu.edu/profile/xzhe1")</f>
         <v/>
       </c>
-      <c r="K54" s="3">
+      <c r="N54" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
@@ -4593,164 +5482,164 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId123"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId141"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId147"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId153"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId159"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add source Directory URL column at end of ASU faculty Excel
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -472,6 +472,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="49" customWidth="1" min="13" max="13"/>
     <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="49" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -545,6 +546,11 @@
           <t>Google Scholar URL</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Directory URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -598,6 +604,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O2" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -659,6 +669,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O3" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -716,6 +730,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O4" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -775,6 +793,10 @@
       </c>
       <c r="N5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O5" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -830,6 +852,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O6" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -887,6 +913,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
+      <c r="O7" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -948,6 +978,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O8" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1005,6 +1039,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
+      <c r="O9" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1070,6 +1108,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O10" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1131,6 +1173,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O11" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1194,6 +1240,10 @@
       </c>
       <c r="N12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O12" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -1253,6 +1303,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O13" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1306,6 +1360,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O14" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1359,6 +1417,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Raghavendra%20Murthy%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O15" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1411,17 +1473,17 @@
       <c r="K16" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>m-Pb6g2pm2UC</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
       <c r="N16" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O16" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -1477,6 +1539,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O17" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1542,6 +1608,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O18" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1607,6 +1677,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=8CS4X9IAAAAJ", "Scholar (8CS4X9IAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O19" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1670,6 +1744,10 @@
       </c>
       <c r="N20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O20" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -1729,6 +1807,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O21" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1792,6 +1874,10 @@
       </c>
       <c r="N22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O22" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -1851,6 +1937,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O23" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1912,6 +2002,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O24" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1973,6 +2067,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
+      <c r="O25" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2036,6 +2134,10 @@
       </c>
       <c r="N26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O26" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -2091,6 +2193,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O27" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2154,6 +2260,10 @@
       </c>
       <c r="N28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O28" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -2209,6 +2319,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O29" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2262,6 +2376,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O30" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2317,6 +2435,10 @@
       </c>
       <c r="N31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O31" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -2325,93 +2447,123 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId120"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2423,7 +2575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2440,6 +2592,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="49" customWidth="1" min="13" max="13"/>
     <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="49" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2513,6 +2666,11 @@
           <t>Google Scholar URL</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Directory URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2566,6 +2724,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O2" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2627,6 +2789,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Werner%20Dahm%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O3" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2684,6 +2850,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O4" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2743,6 +2913,10 @@
       </c>
       <c r="N5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O5" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -2798,6 +2972,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O6" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2855,6 +3033,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
+      <c r="O7" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2916,6 +3098,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O8" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2973,6 +3159,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
+      <c r="O9" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3038,6 +3228,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O10" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3099,6 +3293,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O11" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3162,6 +3360,10 @@
       </c>
       <c r="N12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O12" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -3221,6 +3423,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O13" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3274,6 +3480,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O14" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3327,6 +3537,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Raghavendra%20Murthy%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O15" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3379,17 +3593,17 @@
       <c r="K16" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>m-Pb6g2pm2UC</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
       <c r="N16" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O16" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -3445,6 +3659,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O17" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3510,6 +3728,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O18" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3575,6 +3797,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=8CS4X9IAAAAJ", "Scholar (8CS4X9IAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O19" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3638,6 +3864,10 @@
       </c>
       <c r="N20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O20" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -3697,6 +3927,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O21" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3760,6 +3994,10 @@
       </c>
       <c r="N22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O22" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -3819,6 +4057,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O23" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3880,6 +4122,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O24" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3941,6 +4187,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
+      <c r="O25" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4004,6 +4254,10 @@
       </c>
       <c r="N26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O26" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4059,6 +4313,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O27" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4122,6 +4380,10 @@
       </c>
       <c r="N28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O28" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4177,6 +4439,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O29" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4230,6 +4496,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O30" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4285,6 +4555,10 @@
       </c>
       <c r="N31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O31" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4332,6 +4606,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Aikaterini%20Stefanaki%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O32" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4391,6 +4669,10 @@
       </c>
       <c r="N33" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=tGQzHJIAAAAJ", "Scholar (tGQzHJIAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O33" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4438,6 +4720,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Derrick%20Speaks%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O34" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4483,6 +4769,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Erik%20Andersen%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O35" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4538,6 +4828,10 @@
       </c>
       <c r="N36" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=00Fepb0AAAAJ", "Scholar (00Fepb0AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O36" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4587,6 +4881,10 @@
       </c>
       <c r="N37" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O37" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4634,6 +4932,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ivy%20Chang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O38" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4687,6 +4989,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O39" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4746,6 +5052,10 @@
       </c>
       <c r="N40" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fjUoHOsAAAAJ", "Scholar (fjUoHOsAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O40" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4793,6 +5103,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Joshua%20Wilbur%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O41" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4846,6 +5160,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SWeAf4UAAAAJ", "Scholar (SWeAf4UAAAAJ)")</f>
         <v/>
       </c>
+      <c r="O42" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4901,6 +5219,10 @@
       </c>
       <c r="N43" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O43" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -4952,6 +5274,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O44" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -5001,6 +5327,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O45" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -5056,6 +5386,10 @@
       </c>
       <c r="N46" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O46" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -5107,6 +5441,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Pedro%20Peralta%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O47" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5162,6 +5500,10 @@
       </c>
       <c r="N48" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O48" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -5209,6 +5551,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ricardo%20Cruz%20Lozano%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O49" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5256,6 +5602,10 @@
       </c>
       <c r="N50" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Sridhar%20Seetharaman%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O50" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -5303,6 +5653,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Srinivas%20Chakravarthi%20Kosaraju%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
+      <c r="O51" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5360,6 +5714,10 @@
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SoEC4h4AAAAJ", "Scholar (SoEC4h4AAAAJ)")</f>
         <v/>
       </c>
+      <c r="O52" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5419,6 +5777,10 @@
       </c>
       <c r="N53" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=bHyyOTAAAAAJ", "Scholar (bHyyOTAAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="O53" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -5476,6 +5838,10 @@
       </c>
       <c r="N54" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="O54" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
     </row>
@@ -5484,162 +5850,215 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N36" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N38" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N40" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N44" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N45" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N47" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N48" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N49" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N51" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N52" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N54" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId212"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Lab / Research Group Name column to ASU faculty scraper and Excel export
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -469,13 +469,14 @@
     <col width="65" customWidth="1" min="9" max="9"/>
     <col width="65" customWidth="1" min="10" max="10"/>
     <col width="65" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="49" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="49" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="49" customWidth="1" min="18" max="18"/>
+    <col width="65" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="49" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="49" customWidth="1" min="17" max="17"/>
+    <col width="32" customWidth="1" min="18" max="18"/>
+    <col width="49" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,35 +537,40 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Lab / Research Group Name</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Office Location</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Lab / Personal Website</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Scholar ID</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Profile URL</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Google Scholar URL</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Directory URL</t>
         </is>
@@ -573,7 +579,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Liping Wang</t>
+          <t>Mohamed Houssem Kasbaoui</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -592,55 +598,52 @@
         </is>
       </c>
       <c r="E2" s="3">
-        <f>HYPERLINK("mailto:Liping.Wang@asu.edu", "Liping.Wang@asu.edu")</f>
+        <f>HYPERLINK("mailto:houssem.kasbaoui@asu.edu", "houssem.kasbaoui@asu.edu")</f>
         <v/>
       </c>
       <c r="F2" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>aerospace, guidance, heat transfer, materials, metamaterials, radiation, thermal</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
-        </is>
-      </c>
+          <t>aerospace, cfd, computational fluid dynamics, dns, fluid dynamics, fluid-structure interaction, multiphase flow, turbulent</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Wang research interests include selective control of thermal emission/absorption using meta-materials for energy harvesting and near-field radiation heat transfer enhancement between meta-materials for thermophotovoltaics.</t>
+          <t>Kasbaoui's research interests include computational fluid dynamics, numerical methods, and massively parallel simulations of multiphase and particle-laden flows for environmental and aerospace applications.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology 2011 | M.S. Refrigeration and Cryogenic Engineering, Shanghai Institute of Technical Physics, Chinese  Academy of Sciences 2007 | B.E. Thermal Science and Energy Engineering, University of Science and Technology of China 2004</t>
+          <t>Ph.D.  Aerospace Engineering, Cornell University, 2017 | M.Sc.  Aerospace Engineering, Cornell University, 2015 | M.Sc.  Theoretical Physics, Université Paris-Sud, 2014 | Diplôme d'Ingénieur , Ecole Centrale Paris, 2013 | B.Sc.  Theoretical Physics, Université Paris-Sud, 2011</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="M2" s="3">
-        <f>HYPERLINK("http://faculty.engineering.asu.edu/lpwang", "http://faculty.engineering.asu.edu/lpwang")</f>
-        <v/>
-      </c>
-      <c r="N2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
-        <v/>
-      </c>
+          <t>Multiphase Flow and Fluid-Structure Interaction Group</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="3">
+        <f>HYPERLINK("https://kasbaoui.bitbucket.io", "https://kasbaoui.bitbucket.io")</f>
+        <v/>
+      </c>
+      <c r="O2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
         <v/>
       </c>
       <c r="R2" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="S2" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -648,7 +651,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Mohamed Houssem Kasbaoui</t>
+          <t>Liping Wang</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -667,7 +670,7 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <f>HYPERLINK("mailto:houssem.kasbaoui@asu.edu", "houssem.kasbaoui@asu.edu")</f>
+        <f>HYPERLINK("mailto:Liping.Wang@asu.edu", "Liping.Wang@asu.edu")</f>
         <v/>
       </c>
       <c r="F3" s="2" t="n">
@@ -675,43 +678,52 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>aerospace, cfd, computational fluid dynamics, dns, fluid dynamics, multiphase flow, turbulent</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>aerospace, guidance, heat transfer, materials, metamaterials, radiation, thermal</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Kasbaoui's research interests include computational fluid dynamics, numerical methods, and massively parallel simulations of multiphase and particle-laden flows for environmental and aerospace applications.</t>
+          <t>Wang research interests include selective control of thermal emission/absorption using meta-materials for energy harvesting and near-field radiation heat transfer enhancement between meta-materials for thermophotovoltaics.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Ph.D.  Aerospace Engineering, Cornell University, 2017 | M.Sc.  Aerospace Engineering, Cornell University, 2015 | M.Sc.  Theoretical Physics, Université Paris-Sud, 2014 | Diplôme d'Ingénieur , Ecole Centrale Paris, 2013 | B.Sc.  Theoretical Physics, Université Paris-Sud, 2011</t>
+          <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology 2011 | M.S. Refrigeration and Cryogenic Engineering, Shanghai Institute of Technical Physics, Chinese  Academy of Sciences 2007 | B.E. Thermal Science and Energy Engineering, University of Science and Technology of China 2004</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
-      <c r="M3" s="3">
-        <f>HYPERLINK("https://kasbaoui.bitbucket.io", "https://kasbaoui.bitbucket.io")</f>
-        <v/>
-      </c>
-      <c r="N3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
-        <v/>
-      </c>
+          <t>Nanoscale Thermal Radiation Lab</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="N3" s="3">
+        <f>HYPERLINK("http://faculty.engineering.asu.edu/lpwang", "http://faculty.engineering.asu.edu/lpwang")</f>
+        <v/>
+      </c>
+      <c r="O3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
         <v/>
       </c>
       <c r="R3" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="S3" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -767,26 +779,31 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
+          <t>Computational Mechanics Lab</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 353 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M4" s="3">
+      <c r="N4" s="3">
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="N4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="3">
+      <c r="O4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/joswald1", "https://search.asu.edu/profile/joswald1")</f>
         <v/>
       </c>
-      <c r="Q4" s="3">
+      <c r="R4" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R4" s="3">
+      <c r="S4" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -846,30 +863,31 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
-      <c r="M5" s="3">
+          <t>Sun Robotics Lab</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="3">
         <f>HYPERLINK("https://sunroboticslab.github.io", "https://sunroboticslab.github.io")</f>
         <v/>
       </c>
-      <c r="N5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>fjUoHOsAAAAJ</t>
         </is>
       </c>
-      <c r="P5" s="3">
+      <c r="Q5" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jsun165", "https://search.asu.edu/profile/jsun165")</f>
         <v/>
       </c>
-      <c r="Q5" s="3">
+      <c r="R5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fjUoHOsAAAAJ", "Scholar (fjUoHOsAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R5" s="3">
+      <c r="S5" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -921,23 +939,24 @@
       </c>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>xT-lX9sAAAAJ</t>
         </is>
       </c>
-      <c r="P6" s="3">
+      <c r="Q6" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="Q6" s="3">
+      <c r="R6" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R6" s="3">
+      <c r="S6" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -993,23 +1012,24 @@
       </c>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>DKc-AgcAAAAJ</t>
         </is>
       </c>
-      <c r="P7" s="3">
+      <c r="Q7" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kramesh2", "https://search.asu.edu/profile/kramesh2")</f>
         <v/>
       </c>
-      <c r="Q7" s="3">
+      <c r="R7" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R7" s="3">
+      <c r="S7" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1017,7 +1037,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Leixin Ma</t>
+          <t>Kunal Garg</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1036,7 +1056,7 @@
         </is>
       </c>
       <c r="E8" s="3">
-        <f>HYPERLINK("mailto:Leixin.Ma@asu.edu", "Leixin.Ma@asu.edu")</f>
+        <f>HYPERLINK("mailto:kgarg24@asu.edu", "kgarg24@asu.edu")</f>
         <v/>
       </c>
       <c r="F8" s="2" t="n">
@@ -1044,51 +1064,60 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>aerodynamics, aerospace, fluid-structure interaction, fluids, materials, robot</t>
+          <t>aerospace, autonomous, control theory, motion planning, robot, robotics</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+          <t>Distributed multi-agent motion planning and control, Provably safe control design using machine learning-based certificates, Foundation models in complex robotic tasks, Failure prediction from limited demonstrations, Human-robot interaction.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+          <t>Control Systems, Dynamical Systems, Machine Learning, Nonlinear Dynamical Systems, Robotics</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Leixin Ma's career goal is a data-driven and physically consistent approach to modeling and designing programmable smart structures and robots, especially under complex fluid flow conditions.</t>
+          <t>Garg's research interests include control synthesis for multi-agent coordination using control theory and machine learning.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Ph.D. in Mechanical Engineering, Massachusetts Institute of Technology, 2021 S.M. in Mechanical Engineering, Massachusetts Institute of Technology, 2017 B.S.E. in Naval Architecture and Ocean Engineering, Shanghai Jiao Tong University, 2015</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="3">
-        <f>HYPERLINK("https://sites.google.com/view/oasislabasu", "https://sites.google.com/view/oasislabasu")</f>
-        <v/>
-      </c>
-      <c r="N8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>2xQTOc0AAAAJ</t>
-        </is>
-      </c>
-      <c r="P8" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
-        <v/>
+          <t>PhD. Aerospace Engineering, University of Michigan, Ann Arbor, 2021 MS. Aerospace Engineering, University of Michigan, Ann Arbor, 2019 BTech. Aerospace Engineering, Indian Institute of Technology, Bombay, 2016</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Safe and Autonomous Robotics (STAR) Lab</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
+        </is>
+      </c>
+      <c r="N8" s="3">
+        <f>HYPERLINK("https://sites.google.com/asu.edu/kunalgarg/", "https://sites.google.com/asu.edu/kunalgarg/")</f>
+        <v/>
+      </c>
+      <c r="O8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>vs3pl-8AAAAJ</t>
+        </is>
       </c>
       <c r="Q8" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
         <v/>
       </c>
       <c r="R8" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="S8" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1096,7 +1125,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Gokul Pathikonda</t>
+          <t>Leixin Ma</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1115,59 +1144,64 @@
         </is>
       </c>
       <c r="E9" s="3">
-        <f>HYPERLINK("mailto:Gokul.Pathikonda@asu.edu", "Gokul.Pathikonda@asu.edu")</f>
+        <f>HYPERLINK("mailto:Leixin.Ma@asu.edu", "Leixin.Ma@asu.edu")</f>
         <v/>
       </c>
       <c r="F9" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>aerodynamics, aerospace, reacting flow, turbulence, turbulent</t>
+          <t>aerodynamics, aerospace, fluid-structure interaction, fluids, materials, robot</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Dr. Pathikonda studies turbulent fluid flows to understand natural and engineering phenomena using lab experiments. His expertise is in complex (reacting) mixing, high Re-flows, laser-based &amp; spectroscopic techniques, etc.</t>
+          <t>Leixin Ma's career goal is a data-driven and physically consistent approach to modeling and designing programmable smart structures and robots, especially under complex fluid flow conditions.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Ph. D. Theoretical and Applied Mechanics, University of Illinois, Urbana Champaign, 2017 | MS Aerospace Engineering, University of Illinois, Urbana Champaign, 2013 | B. Tech. Mechanical Engineering, National Institute of Technology, Warangal, 2009</t>
+          <t>Ph.D. in Mechanical Engineering, Massachusetts Institute of Technology, 2021 S.M. in Mechanical Engineering, Massachusetts Institute of Technology, 2017 B.S.E. in Naval Architecture and Ocean Engineering, Shanghai Jiao Tong University, 2015</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
-        </is>
-      </c>
-      <c r="M9" s="3">
-        <f>HYPERLINK("https://faculty.engineering.asu.edu/cmat/", "https://faculty.engineering.asu.edu/cmat/")</f>
-        <v/>
-      </c>
-      <c r="N9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
-        <v/>
+          <t>Optimization, Autonomy, and Soft Intelligence Systems (OASIS) Lab</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="3">
+        <f>HYPERLINK("https://sites.google.com/view/oasislabasu", "https://sites.google.com/view/oasislabasu")</f>
+        <v/>
+      </c>
+      <c r="O9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2xQTOc0AAAAJ</t>
+        </is>
       </c>
       <c r="Q9" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
       <c r="R9" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="S9" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1175,7 +1209,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kunal Garg</t>
+          <t>Gokul Pathikonda</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1194,7 +1228,7 @@
         </is>
       </c>
       <c r="E10" s="3">
-        <f>HYPERLINK("mailto:kgarg24@asu.edu", "kgarg24@asu.edu")</f>
+        <f>HYPERLINK("mailto:Gokul.Pathikonda@asu.edu", "Gokul.Pathikonda@asu.edu")</f>
         <v/>
       </c>
       <c r="F10" s="2" t="n">
@@ -1202,55 +1236,52 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>aerospace, control theory, motion planning, robot, robotics</t>
+          <t>aerodynamics, aerospace, reacting flow, turbulence, turbulent</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Distributed multi-agent motion planning and control, Provably safe control design using machine learning-based certificates, Foundation models in complex robotic tasks, Failure prediction from limited demonstrations, Human-robot interaction.</t>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Control Systems, Dynamical Systems, Machine Learning, Nonlinear Dynamical Systems, Robotics</t>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Garg's research interests include control synthesis for multi-agent coordination using control theory and machine learning.</t>
+          <t>Dr. Pathikonda studies turbulent fluid flows to understand natural and engineering phenomena using lab experiments. His expertise is in complex (reacting) mixing, high Re-flows, laser-based &amp; spectroscopic techniques, etc.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>PhD. Aerospace Engineering, University of Michigan, Ann Arbor, 2021 MS. Aerospace Engineering, University of Michigan, Ann Arbor, 2019 BTech. Aerospace Engineering, Indian Institute of Technology, Bombay, 2016</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
-        </is>
-      </c>
-      <c r="M10" s="3">
-        <f>HYPERLINK("https://sites.google.com/asu.edu/kunalgarg/", "https://sites.google.com/asu.edu/kunalgarg/")</f>
-        <v/>
-      </c>
-      <c r="N10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>vs3pl-8AAAAJ</t>
-        </is>
-      </c>
-      <c r="P10" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
-        <v/>
-      </c>
+          <t>Ph. D. Theoretical and Applied Mechanics, University of Illinois, Urbana Champaign, 2017 | MS Aerospace Engineering, University of Illinois, Urbana Champaign, 2013 | B. Tech. Mechanical Engineering, National Institute of Technology, Warangal, 2009</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
+        </is>
+      </c>
+      <c r="N10" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/cmat/", "https://faculty.engineering.asu.edu/cmat/")</f>
+        <v/>
+      </c>
+      <c r="O10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
         <v/>
       </c>
       <c r="R10" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="S10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1300,25 +1331,30 @@
           <t>PhD in Mechanical Engineering, University of Technology (RWTH) Aachen, Germany 2001 | Diploma. Mechanical and Aerospace Engineering, University of Technology (RWTH) Aachen, Germany 1995</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Computational Multiphase Physics Laboratory</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>yv6aCW8AAAAJ</t>
         </is>
       </c>
-      <c r="P11" s="3">
+      <c r="Q11" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mherrma1", "https://search.asu.edu/profile/mherrma1")</f>
         <v/>
       </c>
-      <c r="Q11" s="3">
+      <c r="R11" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R11" s="3">
+      <c r="S11" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1376,28 +1412,33 @@
           <t>Ph.D. Mechanical Engineering and Applied Mechanics, University of Pennsylvania 2010 | M.S.E. Mechanical Engineering and Applied Mechanics, University of Pennsylvania 2008 | B.S.E. Mechanical and Aerospace Engineering, Princeton University 2005 | Certificate. Robotics and Intelligent Systems, Princeton University 2005</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="3">
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous Collective Systems (ACS) Laboratory</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/acs/", "http://faculty.engineering.asu.edu/acs/")</f>
         <v/>
       </c>
-      <c r="N12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>KKup0OgAAAAJ</t>
         </is>
       </c>
-      <c r="P12" s="3">
+      <c r="Q12" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="Q12" s="3">
+      <c r="R12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R12" s="3">
+      <c r="S12" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1455,28 +1496,29 @@
           <t>Ph.D Degree at the  Department of Electrical, Computer, and Systems Engineering  at  Rensselaer Polytechnic Institute  in 2018 | Master's Degree at the  School of electrical and information engineering  at  Tianjin University  in 2014 | Bachelor's Degree at the  School of electrical and information engineering  at  Tianjin University  in 2011</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M13" s="3">
+      <c r="N13" s="3">
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="N13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="3">
+      <c r="O13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xzhe1", "https://search.asu.edu/profile/xzhe1")</f>
         <v/>
       </c>
-      <c r="Q13" s="3">
+      <c r="R13" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R13" s="3">
+      <c r="S13" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1528,19 +1570,20 @@
       </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="3">
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
         <v/>
       </c>
-      <c r="Q14" s="3">
+      <c r="R14" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R14" s="3">
+      <c r="S14" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1598,24 +1641,29 @@
           <t>Ph.D. Aeronautics and Astronautics, Stanford University 2006 | Bachelor's degree. Physics, University of Texas-Austin 1999 | Bachelor's degree. Aerospace Engineering, University of Texas-Austin 1999</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="3">
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Cybernetic Systems and Controls Laboratory (CSCL)</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="3">
         <f>HYPERLINK("http://control.asu.edu/", "http://control.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="3">
+      <c r="O15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mpeet", "https://search.asu.edu/profile/mpeet")</f>
         <v/>
       </c>
-      <c r="Q15" s="3">
+      <c r="R15" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R15" s="3">
+      <c r="S15" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1674,27 +1722,28 @@
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="3">
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="3">
         <f>HYPERLINK("http://wang.faculty.asu.edu/", "http://wang.faculty.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>LaUdx9gAAAAJ</t>
         </is>
       </c>
-      <c r="P16" s="3">
+      <c r="Q16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rywang", "https://search.asu.edu/profile/rywang")</f>
         <v/>
       </c>
-      <c r="Q16" s="3">
+      <c r="R16" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R16" s="3">
+      <c r="S16" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1753,23 +1802,24 @@
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="3">
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="3">
         <f>HYPERLINK("http://RESEARCHGATE.net/profile/Ryan_Milcarek", "http://RESEARCHGATE.net/profile/Ryan_Milcarek")</f>
         <v/>
       </c>
-      <c r="N17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O17" s="2" t="inlineStr"/>
-      <c r="P17" s="3">
+      <c r="O17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="Q17" s="3">
+      <c r="R17" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R17" s="3">
+      <c r="S17" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1819,25 +1869,26 @@
           <t>Ph.D. Aerospace Engineering, University of Michigan-Ann Arbor | M.S.E. Aerospace Engineering, University of Michigan-Ann Arbor | B.S. Aeronautical and Astronautical Engineering, The Ohio State University-Columbus</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>ENGRC 377 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O18" s="2" t="inlineStr"/>
-      <c r="P18" s="3">
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/attwl", "https://search.asu.edu/profile/attwl")</f>
         <v/>
       </c>
-      <c r="Q18" s="3">
+      <c r="R18" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R18" s="3">
+      <c r="S18" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1889,19 +1940,20 @@
       </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O19" s="2" t="inlineStr"/>
-      <c r="P19" s="3">
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="Q19" s="3">
+      <c r="R19" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R19" s="3">
+      <c r="S19" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1953,27 +2005,28 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
+          <t>Adaptive Intelligent Materials &amp; Systems (AIMS) Center</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>w3fU9E0AAAAJ</t>
         </is>
       </c>
-      <c r="P20" s="3">
+      <c r="Q20" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/chattopa", "https://search.asu.edu/profile/chattopa")</f>
         <v/>
       </c>
-      <c r="Q20" s="3">
+      <c r="R20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R20" s="3">
+      <c r="S20" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2031,29 +2084,30 @@
           <t>PhD Johns Hopkins University</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>HRx2lJQAAAAJ</t>
         </is>
       </c>
-      <c r="P21" s="3">
+      <c r="Q21" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/adscotti", "https://search.asu.edu/profile/adscotti")</f>
         <v/>
       </c>
-      <c r="Q21" s="3">
+      <c r="R21" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R21" s="3">
+      <c r="S21" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2109,30 +2163,35 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
+          <t>3D Energy Lab</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
           <t>551 E Tyler Mall ERC 363 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="M22" s="3">
+      <c r="N22" s="3">
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="N22" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="O22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>fs2d97sAAAAJ</t>
         </is>
       </c>
-      <c r="P22" s="3">
+      <c r="Q22" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/bkwon2", "https://search.asu.edu/profile/bkwon2")</f>
         <v/>
       </c>
-      <c r="Q22" s="3">
+      <c r="R22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R22" s="3">
+      <c r="S22" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2186,28 +2245,33 @@
           <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology, Atlanta 2013 | M.S. Mechanical Engineering, Clemson University, SC 2009 | M.S. Biomedical Engineering, Sharif University of Technology, Tehran, Iran 2007 | B.S. Mechanical Engineering, Iran University of Science and Technology, Tehran 2004</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="3">
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Bio-Inspired Robotics, Technology, and Healthcare Laboratory (BIRTH Lab)</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="3">
         <f>HYPERLINK("http://birth.asu.edu", "http://birth.asu.edu")</f>
         <v/>
       </c>
-      <c r="N23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>00Fepb0AAAAJ</t>
         </is>
       </c>
-      <c r="P23" s="3">
+      <c r="Q23" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hmarvi", "https://search.asu.edu/profile/hmarvi")</f>
         <v/>
       </c>
-      <c r="Q23" s="3">
+      <c r="R23" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=00Fepb0AAAAJ", "Scholar (00Fepb0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R23" s="3">
+      <c r="S23" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2257,28 +2321,29 @@
           <t>B.S. Mechanical and Aerospace Engineering, Seoul National University (2002) M.S. Mechanical and Aerospace Engineering, Seoul National University (2004) Ph.D Mechanical Engineering, Massachusetts Institute of Technology (2013)</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M24" s="3">
+      <c r="N24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/hlee", "https://faculty.engineering.asu.edu/hlee")</f>
         <v/>
       </c>
-      <c r="N24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O24" s="2" t="inlineStr"/>
-      <c r="P24" s="3">
+      <c r="O24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hlee234", "https://search.asu.edu/profile/hlee234")</f>
         <v/>
       </c>
-      <c r="Q24" s="3">
+      <c r="R24" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R24" s="3">
+      <c r="S24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2336,24 +2401,29 @@
           <t>PhD. Mechanical Engineering, University of Maryland-College Park 2007 | M.S. Mechanical Engineering, University of Maryland-College Park 2005 | PhD. Student, Mechanical Engineering, Isfahan University of Technology, Iran 2001-2002 | M.S. Mechanical Engineering, Isfahan University of Technology, Iran 2001 | B.S. Mechanical Engineering, Isfahan University of Technology, Iran 1999</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="3">
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing and Advanced Materials Characterization (MAGIC) Lab</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="3">
         <f>HYPERLINK("https://magic.asu.edu/", "https://magic.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O25" s="2" t="inlineStr"/>
-      <c r="P25" s="3">
+      <c r="O25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ljannesa", "https://search.asu.edu/profile/ljannesa")</f>
         <v/>
       </c>
-      <c r="Q25" s="3">
+      <c r="R25" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R25" s="3">
+      <c r="S25" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2411,25 +2481,26 @@
           <t>Postdoctoral Fellow, Tokyo Institute of Technology, Japan 1990-1992 | Ph.D. Mechanical Engineering, University of California, Berkeley 1990 | M.S. Mechanical Engineering, Massachusetts Institute of Technology 1987 | B. S. Mechanical Engineering, Tulane University, New Orleans, LA 1985</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>ENGRC 463 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O26" s="2" t="inlineStr"/>
-      <c r="P26" s="3">
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pphelan", "https://search.asu.edu/profile/pphelan")</f>
         <v/>
       </c>
-      <c r="Q26" s="3">
+      <c r="R26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R26" s="3">
+      <c r="S26" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2479,28 +2550,33 @@
           <t>Ph.D. Aeronautics and Astronautics, Stanford University 2006 | M.S. Management, State University Higher School of Economics, Moscow, Russia 2000 | M.S. Aeromechanics and Flight Engineering, Moscow Institute of Physics and Technology, Russia 1999 | B.S. Applied Mathematics and Physics, Moscow Institute of Physics and Technology, Russia 1997</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="3">
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Interdisciplinary Simulation and Modeling (ISiM) Lab</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="3">
         <f>HYPERLINK("https://isim.asu.edu", "https://isim.asu.edu")</f>
         <v/>
       </c>
-      <c r="N27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="O27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>_6o8MrUAAAAJ</t>
         </is>
       </c>
-      <c r="P27" s="3">
+      <c r="Q27" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="Q27" s="3">
+      <c r="R27" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R27" s="3">
+      <c r="S27" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2558,25 +2634,34 @@
           <t>Postdoc, Department of Mechanical and Aerospace Engineering, Princeton University Postdoc, Center for Nanophase Materials Sciences, Oak Ridge National Laboratory Ph.D., Major: Materials Science and Engineering; Minor: Applied Engineering Physics, Cornell University M.S., Major: Materials Science and Engineering; Minor: Applied Engineering Physics, Cornell University M.Phil., Mechanical Engineering, The University of Hong Kong B.Eng., Materials Science and Engineering, Hunan University</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Computational Materials Science and Design Lab</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
         <is>
           <t>4yYKCpUAAAAJ</t>
         </is>
       </c>
-      <c r="P28" s="3">
+      <c r="Q28" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hzhuang7", "https://search.asu.edu/profile/hzhuang7")</f>
         <v/>
       </c>
-      <c r="Q28" s="3">
+      <c r="R28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R28" s="3">
+      <c r="S28" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2626,28 +2711,29 @@
           <t>Ph.D. University of Illinois-Urbana-Champaign 1997 | M.S. National Taiwan University 1989 | B.S. National Central University,Taiwan 1987</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M29" s="3">
+      <c r="N29" s="3">
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="N29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O29" s="2" t="inlineStr"/>
-      <c r="P29" s="3">
+      <c r="O29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hhuang38", "https://search.asu.edu/profile/hhuang38")</f>
         <v/>
       </c>
-      <c r="Q29" s="3">
+      <c r="R29" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R29" s="3">
+      <c r="S29" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2707,30 +2793,35 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
+          <t>Nanomechanics Laboratory</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 355 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M30" s="3">
+      <c r="N30" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/jagan/", "http://faculty.engineering.asu.edu/jagan/")</f>
         <v/>
       </c>
-      <c r="N30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="O30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>ClqRIhIAAAAJ</t>
         </is>
       </c>
-      <c r="P30" s="3">
+      <c r="Q30" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jrajago1", "https://search.asu.edu/profile/jrajago1")</f>
         <v/>
       </c>
-      <c r="Q30" s="3">
+      <c r="R30" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R30" s="3">
+      <c r="S30" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2780,28 +2871,33 @@
           <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology 2009 | M.S. Mechanical Engineering, Georgia Institute of Technology 2007 | B.S. Mechanical Engineering, Georgia Institute of Technology 2005</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="3">
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Nano-Bio-Thermal Engineering Laboratory</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/konrad/", "http://faculty.engineering.asu.edu/konrad/")</f>
         <v/>
       </c>
-      <c r="N31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
+      <c r="O31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>SWeAf4UAAAAJ</t>
         </is>
       </c>
-      <c r="P31" s="3">
+      <c r="Q31" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/krykacze", "https://search.asu.edu/profile/krykacze")</f>
         <v/>
       </c>
-      <c r="Q31" s="3">
+      <c r="R31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SWeAf4UAAAAJ", "Scholar (SWeAf4UAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R31" s="3">
+      <c r="S31" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2857,23 +2953,24 @@
       </c>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>9LWNC50AAAAJ</t>
         </is>
       </c>
-      <c r="P32" s="3">
+      <c r="Q32" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mingleiq", "https://search.asu.edu/profile/mingleiq")</f>
         <v/>
       </c>
-      <c r="Q32" s="3">
+      <c r="R32" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R32" s="3">
+      <c r="S32" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2931,28 +3028,29 @@
           <t>Ph.D. Manufacturing, Industrial Engineering, Purdue University 2015 | B.Sc. Materials Science and Engineering, University of Science and Technology of China 2009</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M33" s="3">
+      <c r="N33" s="3">
         <f>HYPERLINK("https://mmmplab.engineering.asu.edu/", "https://mmmplab.engineering.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="3">
+      <c r="O33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/qnian", "https://search.asu.edu/profile/qnian")</f>
         <v/>
       </c>
-      <c r="Q33" s="3">
+      <c r="R33" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R33" s="3">
+      <c r="S33" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3004,26 +3102,31 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
+          <t>Wind Energy and Atmospheric Boundary Layer Lab</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M34" s="3">
+      <c r="N34" s="3">
         <f>HYPERLINK("https://windlab.engineering.asu.edu/ronald-calhoun/", "https://windlab.engineering.asu.edu/ronald-calhoun/")</f>
         <v/>
       </c>
-      <c r="N34" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="3">
+      <c r="O34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcalhou", "https://search.asu.edu/profile/rcalhou")</f>
         <v/>
       </c>
-      <c r="Q34" s="3">
+      <c r="R34" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R34" s="3">
+      <c r="S34" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3077,28 +3180,33 @@
           <t>Ph.D., Purdue University 2021 | Master of Science, Harbin Institute of Technology, 2016 | Bachelor of Engineering, Harbin Institute of Technology, 2014</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="3">
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Intelligent Robotics and Interactive Systems Lab (IRIS Lab)</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="3">
         <f>HYPERLINK("https://irislab.tech/", "https://irislab.tech/")</f>
         <v/>
       </c>
-      <c r="N35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O35" s="2" t="inlineStr">
+      <c r="O35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>SoEC4h4AAAAJ</t>
         </is>
       </c>
-      <c r="P35" s="3">
+      <c r="Q35" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wjin34", "https://search.asu.edu/profile/wjin34")</f>
         <v/>
       </c>
-      <c r="Q35" s="3">
+      <c r="R35" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SoEC4h4AAAAJ", "Scholar (SoEC4h4AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R35" s="3">
+      <c r="S35" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3154,23 +3262,28 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
+          <t>Prognostics and Health Management (PHM) Lab</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 409 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O36" s="2" t="inlineStr"/>
-      <c r="P36" s="3">
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yliu35", "https://search.asu.edu/profile/yliu35")</f>
         <v/>
       </c>
-      <c r="Q36" s="3">
+      <c r="R36" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R36" s="3">
+      <c r="S36" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3228,28 +3341,33 @@
           <t>Ph.D. in Industrial and Systems Engineering, University of Southern California, 2019 M.S. in Computer Science, University of Southern California, 2019 M.S. in Manufacturing Engineering, Nanjing University of Aeronautics and Astronautics, 2014 B.E. in Mechanical Engineering and Automation, Nanjing University of Aeronautics and Astronautics, 2011</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="3">
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Advanced Manufacturing and Bio-inspired Design Lab</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="3">
         <f>HYPERLINK("https://www.cindyxjli.com/", "https://www.cindyxjli.com/")</f>
         <v/>
       </c>
-      <c r="N37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="O37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>tGQzHJIAAAAJ</t>
         </is>
       </c>
-      <c r="P37" s="3">
+      <c r="Q37" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xiangji5", "https://search.asu.edu/profile/xiangji5")</f>
         <v/>
       </c>
-      <c r="Q37" s="3">
+      <c r="R37" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=tGQzHJIAAAAJ", "Scholar (tGQzHJIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R37" s="3">
+      <c r="S37" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3304,20 +3422,25 @@
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O38" s="2" t="inlineStr"/>
-      <c r="P38" s="3">
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jimbo", "https://search.asu.edu/profile/jimbo")</f>
         <v/>
       </c>
-      <c r="Q38" s="3">
+      <c r="R38" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R38" s="3">
+      <c r="S38" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3367,25 +3490,26 @@
           <t>PhD The Ohio State University</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O39" s="2" t="inlineStr"/>
-      <c r="P39" s="3">
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/linli25", "https://search.asu.edu/profile/linli25")</f>
         <v/>
       </c>
-      <c r="Q39" s="3">
+      <c r="R39" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R39" s="3">
+      <c r="S39" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3436,20 +3560,25 @@
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O40" s="2" t="inlineStr"/>
-      <c r="P40" s="3">
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/marc03", "https://search.asu.edu/profile/marc03")</f>
         <v/>
       </c>
-      <c r="Q40" s="3">
+      <c r="R40" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R40" s="3">
+      <c r="S40" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3500,23 +3629,24 @@
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="3">
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/pperalta/", "https://faculty.engineering.asu.edu/pperalta/")</f>
         <v/>
       </c>
-      <c r="N41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O41" s="2" t="inlineStr"/>
-      <c r="P41" s="3">
+      <c r="O41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pperalta", "https://search.asu.edu/profile/pperalta")</f>
         <v/>
       </c>
-      <c r="Q41" s="3">
+      <c r="R41" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Pedro%20Peralta%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R41" s="3">
+      <c r="S41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3574,32 +3704,33 @@
           <t>Ph.D. Mechanical Science and Engineering, University of Illinois at Urbana-Champaign 2012</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M42" s="3">
+      <c r="N42" s="3">
         <f>HYPERLINK("https://wonmokang3.wixsite.com/website", "https://wonmokang3.wixsite.com/website")</f>
         <v/>
       </c>
-      <c r="N42" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
+      <c r="O42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
         <is>
           <t>bHyyOTAAAAAJ</t>
         </is>
       </c>
-      <c r="P42" s="3">
+      <c r="Q42" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wkang16", "https://search.asu.edu/profile/wkang16")</f>
         <v/>
       </c>
-      <c r="Q42" s="3">
+      <c r="R42" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=bHyyOTAAAAAJ", "Scholar (bHyyOTAAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R42" s="3">
+      <c r="S42" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3649,25 +3780,22 @@
           <t>Ph.D. Mechanical Engineering, University of Michigan 2011 | M.S. Mechanical Engineering, University of Michigan 2009 | B.S. Automative Engineering, Tsinghua University, China 2007</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>GWC 464 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr"/>
-      <c r="N43" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O43" s="2" t="inlineStr"/>
-      <c r="P43" s="3">
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P43" s="2" t="inlineStr"/>
+      <c r="Q43" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yren32", "https://search.asu.edu/profile/yren32")</f>
         <v/>
       </c>
-      <c r="Q43" s="3">
+      <c r="R43" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R43" s="3">
+      <c r="S43" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3675,199 +3803,199 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId149"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId154"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId159"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId194"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3879,7 +4007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:S49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3893,13 +4021,14 @@
     <col width="65" customWidth="1" min="9" max="9"/>
     <col width="65" customWidth="1" min="10" max="10"/>
     <col width="65" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="49" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="49" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="49" customWidth="1" min="18" max="18"/>
+    <col width="65" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="49" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="49" customWidth="1" min="17" max="17"/>
+    <col width="32" customWidth="1" min="18" max="18"/>
+    <col width="49" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3960,35 +4089,40 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Lab / Research Group Name</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Office Location</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Lab / Personal Website</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Scholar ID</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Profile URL</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Google Scholar URL</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Directory URL</t>
         </is>
@@ -3997,7 +4131,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Liping Wang</t>
+          <t>Mohamed Houssem Kasbaoui</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -4016,55 +4150,52 @@
         </is>
       </c>
       <c r="E2" s="3">
-        <f>HYPERLINK("mailto:Liping.Wang@asu.edu", "Liping.Wang@asu.edu")</f>
+        <f>HYPERLINK("mailto:houssem.kasbaoui@asu.edu", "houssem.kasbaoui@asu.edu")</f>
         <v/>
       </c>
       <c r="F2" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>aerospace, guidance, heat transfer, materials, metamaterials, radiation, thermal</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
-        </is>
-      </c>
+          <t>aerospace, cfd, computational fluid dynamics, dns, fluid dynamics, fluid-structure interaction, multiphase flow, turbulent</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Wang research interests include selective control of thermal emission/absorption using meta-materials for energy harvesting and near-field radiation heat transfer enhancement between meta-materials for thermophotovoltaics.</t>
+          <t>Kasbaoui's research interests include computational fluid dynamics, numerical methods, and massively parallel simulations of multiphase and particle-laden flows for environmental and aerospace applications.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology 2011 | M.S. Refrigeration and Cryogenic Engineering, Shanghai Institute of Technical Physics, Chinese  Academy of Sciences 2007 | B.E. Thermal Science and Energy Engineering, University of Science and Technology of China 2004</t>
+          <t>Ph.D.  Aerospace Engineering, Cornell University, 2017 | M.Sc.  Aerospace Engineering, Cornell University, 2015 | M.Sc.  Theoretical Physics, Université Paris-Sud, 2014 | Diplôme d'Ingénieur , Ecole Centrale Paris, 2013 | B.Sc.  Theoretical Physics, Université Paris-Sud, 2011</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="M2" s="3">
-        <f>HYPERLINK("http://faculty.engineering.asu.edu/lpwang", "http://faculty.engineering.asu.edu/lpwang")</f>
-        <v/>
-      </c>
-      <c r="N2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
-        <v/>
-      </c>
+          <t>Multiphase Flow and Fluid-Structure Interaction Group</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="3">
+        <f>HYPERLINK("https://kasbaoui.bitbucket.io", "https://kasbaoui.bitbucket.io")</f>
+        <v/>
+      </c>
+      <c r="O2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
         <v/>
       </c>
       <c r="R2" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="S2" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4072,7 +4203,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Mohamed Houssem Kasbaoui</t>
+          <t>Liping Wang</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -4091,7 +4222,7 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <f>HYPERLINK("mailto:houssem.kasbaoui@asu.edu", "houssem.kasbaoui@asu.edu")</f>
+        <f>HYPERLINK("mailto:Liping.Wang@asu.edu", "Liping.Wang@asu.edu")</f>
         <v/>
       </c>
       <c r="F3" s="2" t="n">
@@ -4099,43 +4230,52 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>aerospace, cfd, computational fluid dynamics, dns, fluid dynamics, multiphase flow, turbulent</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>aerospace, guidance, heat transfer, materials, metamaterials, radiation, thermal</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Kasbaoui's research interests include computational fluid dynamics, numerical methods, and massively parallel simulations of multiphase and particle-laden flows for environmental and aerospace applications.</t>
+          <t>Wang research interests include selective control of thermal emission/absorption using meta-materials for energy harvesting and near-field radiation heat transfer enhancement between meta-materials for thermophotovoltaics.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Ph.D.  Aerospace Engineering, Cornell University, 2017 | M.Sc.  Aerospace Engineering, Cornell University, 2015 | M.Sc.  Theoretical Physics, Université Paris-Sud, 2014 | Diplôme d'Ingénieur , Ecole Centrale Paris, 2013 | B.Sc.  Theoretical Physics, Université Paris-Sud, 2011</t>
+          <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology 2011 | M.S. Refrigeration and Cryogenic Engineering, Shanghai Institute of Technical Physics, Chinese  Academy of Sciences 2007 | B.E. Thermal Science and Energy Engineering, University of Science and Technology of China 2004</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
-      <c r="M3" s="3">
-        <f>HYPERLINK("https://kasbaoui.bitbucket.io", "https://kasbaoui.bitbucket.io")</f>
-        <v/>
-      </c>
-      <c r="N3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
-        <v/>
-      </c>
+          <t>Nanoscale Thermal Radiation Lab</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="N3" s="3">
+        <f>HYPERLINK("http://faculty.engineering.asu.edu/lpwang", "http://faculty.engineering.asu.edu/lpwang")</f>
+        <v/>
+      </c>
+      <c r="O3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
         <v/>
       </c>
       <c r="R3" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="S3" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4191,26 +4331,31 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
+          <t>Computational Mechanics Lab</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 353 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M4" s="3">
+      <c r="N4" s="3">
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="N4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="3">
+      <c r="O4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/joswald1", "https://search.asu.edu/profile/joswald1")</f>
         <v/>
       </c>
-      <c r="Q4" s="3">
+      <c r="R4" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R4" s="3">
+      <c r="S4" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4270,30 +4415,31 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
-      <c r="M5" s="3">
+          <t>Sun Robotics Lab</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="3">
         <f>HYPERLINK("https://sunroboticslab.github.io", "https://sunroboticslab.github.io")</f>
         <v/>
       </c>
-      <c r="N5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>fjUoHOsAAAAJ</t>
         </is>
       </c>
-      <c r="P5" s="3">
+      <c r="Q5" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jsun165", "https://search.asu.edu/profile/jsun165")</f>
         <v/>
       </c>
-      <c r="Q5" s="3">
+      <c r="R5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fjUoHOsAAAAJ", "Scholar (fjUoHOsAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R5" s="3">
+      <c r="S5" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4345,23 +4491,24 @@
       </c>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>xT-lX9sAAAAJ</t>
         </is>
       </c>
-      <c r="P6" s="3">
+      <c r="Q6" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="Q6" s="3">
+      <c r="R6" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R6" s="3">
+      <c r="S6" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4417,23 +4564,24 @@
       </c>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>DKc-AgcAAAAJ</t>
         </is>
       </c>
-      <c r="P7" s="3">
+      <c r="Q7" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kramesh2", "https://search.asu.edu/profile/kramesh2")</f>
         <v/>
       </c>
-      <c r="Q7" s="3">
+      <c r="R7" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R7" s="3">
+      <c r="S7" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4441,7 +4589,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Leixin Ma</t>
+          <t>Kunal Garg</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -4460,7 +4608,7 @@
         </is>
       </c>
       <c r="E8" s="3">
-        <f>HYPERLINK("mailto:Leixin.Ma@asu.edu", "Leixin.Ma@asu.edu")</f>
+        <f>HYPERLINK("mailto:kgarg24@asu.edu", "kgarg24@asu.edu")</f>
         <v/>
       </c>
       <c r="F8" s="2" t="n">
@@ -4468,51 +4616,60 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>aerodynamics, aerospace, fluid-structure interaction, fluids, materials, robot</t>
+          <t>aerospace, autonomous, control theory, motion planning, robot, robotics</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+          <t>Distributed multi-agent motion planning and control, Provably safe control design using machine learning-based certificates, Foundation models in complex robotic tasks, Failure prediction from limited demonstrations, Human-robot interaction.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
+          <t>Control Systems, Dynamical Systems, Machine Learning, Nonlinear Dynamical Systems, Robotics</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Leixin Ma's career goal is a data-driven and physically consistent approach to modeling and designing programmable smart structures and robots, especially under complex fluid flow conditions.</t>
+          <t>Garg's research interests include control synthesis for multi-agent coordination using control theory and machine learning.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Ph.D. in Mechanical Engineering, Massachusetts Institute of Technology, 2021 S.M. in Mechanical Engineering, Massachusetts Institute of Technology, 2017 B.S.E. in Naval Architecture and Ocean Engineering, Shanghai Jiao Tong University, 2015</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="3">
-        <f>HYPERLINK("https://sites.google.com/view/oasislabasu", "https://sites.google.com/view/oasislabasu")</f>
-        <v/>
-      </c>
-      <c r="N8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>2xQTOc0AAAAJ</t>
-        </is>
-      </c>
-      <c r="P8" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
-        <v/>
+          <t>PhD. Aerospace Engineering, University of Michigan, Ann Arbor, 2021 MS. Aerospace Engineering, University of Michigan, Ann Arbor, 2019 BTech. Aerospace Engineering, Indian Institute of Technology, Bombay, 2016</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Safe and Autonomous Robotics (STAR) Lab</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
+        </is>
+      </c>
+      <c r="N8" s="3">
+        <f>HYPERLINK("https://sites.google.com/asu.edu/kunalgarg/", "https://sites.google.com/asu.edu/kunalgarg/")</f>
+        <v/>
+      </c>
+      <c r="O8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>vs3pl-8AAAAJ</t>
+        </is>
       </c>
       <c r="Q8" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
         <v/>
       </c>
       <c r="R8" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="S8" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4520,7 +4677,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Gokul Pathikonda</t>
+          <t>Leixin Ma</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -4539,59 +4696,64 @@
         </is>
       </c>
       <c r="E9" s="3">
-        <f>HYPERLINK("mailto:Gokul.Pathikonda@asu.edu", "Gokul.Pathikonda@asu.edu")</f>
+        <f>HYPERLINK("mailto:Leixin.Ma@asu.edu", "Leixin.Ma@asu.edu")</f>
         <v/>
       </c>
       <c r="F9" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>aerodynamics, aerospace, reacting flow, turbulence, turbulent</t>
+          <t>aerodynamics, aerospace, fluid-structure interaction, fluids, materials, robot</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
+          <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Dr. Pathikonda studies turbulent fluid flows to understand natural and engineering phenomena using lab experiments. His expertise is in complex (reacting) mixing, high Re-flows, laser-based &amp; spectroscopic techniques, etc.</t>
+          <t>Leixin Ma's career goal is a data-driven and physically consistent approach to modeling and designing programmable smart structures and robots, especially under complex fluid flow conditions.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Ph. D. Theoretical and Applied Mechanics, University of Illinois, Urbana Champaign, 2017 | MS Aerospace Engineering, University of Illinois, Urbana Champaign, 2013 | B. Tech. Mechanical Engineering, National Institute of Technology, Warangal, 2009</t>
+          <t>Ph.D. in Mechanical Engineering, Massachusetts Institute of Technology, 2021 S.M. in Mechanical Engineering, Massachusetts Institute of Technology, 2017 B.S.E. in Naval Architecture and Ocean Engineering, Shanghai Jiao Tong University, 2015</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
-        </is>
-      </c>
-      <c r="M9" s="3">
-        <f>HYPERLINK("https://faculty.engineering.asu.edu/cmat/", "https://faculty.engineering.asu.edu/cmat/")</f>
-        <v/>
-      </c>
-      <c r="N9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
-        <v/>
+          <t>Optimization, Autonomy, and Soft Intelligence Systems (OASIS) Lab</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="3">
+        <f>HYPERLINK("https://sites.google.com/view/oasislabasu", "https://sites.google.com/view/oasislabasu")</f>
+        <v/>
+      </c>
+      <c r="O9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2xQTOc0AAAAJ</t>
+        </is>
       </c>
       <c r="Q9" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
       <c r="R9" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="S9" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4599,7 +4761,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kunal Garg</t>
+          <t>Gokul Pathikonda</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -4618,7 +4780,7 @@
         </is>
       </c>
       <c r="E10" s="3">
-        <f>HYPERLINK("mailto:kgarg24@asu.edu", "kgarg24@asu.edu")</f>
+        <f>HYPERLINK("mailto:Gokul.Pathikonda@asu.edu", "Gokul.Pathikonda@asu.edu")</f>
         <v/>
       </c>
       <c r="F10" s="2" t="n">
@@ -4626,55 +4788,52 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>aerospace, control theory, motion planning, robot, robotics</t>
+          <t>aerodynamics, aerospace, reacting flow, turbulence, turbulent</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Distributed multi-agent motion planning and control, Provably safe control design using machine learning-based certificates, Foundation models in complex robotic tasks, Failure prediction from limited demonstrations, Human-robot interaction.</t>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Control Systems, Dynamical Systems, Machine Learning, Nonlinear Dynamical Systems, Robotics</t>
+          <t>Aerodynamics, Aerospace Engineering, Mechanical Engineering</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Garg's research interests include control synthesis for multi-agent coordination using control theory and machine learning.</t>
+          <t>Dr. Pathikonda studies turbulent fluid flows to understand natural and engineering phenomena using lab experiments. His expertise is in complex (reacting) mixing, high Re-flows, laser-based &amp; spectroscopic techniques, etc.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>PhD. Aerospace Engineering, University of Michigan, Ann Arbor, 2021 MS. Aerospace Engineering, University of Michigan, Ann Arbor, 2019 BTech. Aerospace Engineering, Indian Institute of Technology, Bombay, 2016</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
-        </is>
-      </c>
-      <c r="M10" s="3">
-        <f>HYPERLINK("https://sites.google.com/asu.edu/kunalgarg/", "https://sites.google.com/asu.edu/kunalgarg/")</f>
-        <v/>
-      </c>
-      <c r="N10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>vs3pl-8AAAAJ</t>
-        </is>
-      </c>
-      <c r="P10" s="3">
-        <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
-        <v/>
-      </c>
+          <t>Ph. D. Theoretical and Applied Mechanics, University of Illinois, Urbana Champaign, 2017 | MS Aerospace Engineering, University of Illinois, Urbana Champaign, 2013 | B. Tech. Mechanical Engineering, National Institute of Technology, Warangal, 2009</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
+        </is>
+      </c>
+      <c r="N10" s="3">
+        <f>HYPERLINK("https://faculty.engineering.asu.edu/cmat/", "https://faculty.engineering.asu.edu/cmat/")</f>
+        <v/>
+      </c>
+      <c r="O10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
+        <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
         <v/>
       </c>
       <c r="R10" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="S10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4724,25 +4883,30 @@
           <t>PhD in Mechanical Engineering, University of Technology (RWTH) Aachen, Germany 2001 | Diploma. Mechanical and Aerospace Engineering, University of Technology (RWTH) Aachen, Germany 1995</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Computational Multiphase Physics Laboratory</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>yv6aCW8AAAAJ</t>
         </is>
       </c>
-      <c r="P11" s="3">
+      <c r="Q11" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mherrma1", "https://search.asu.edu/profile/mherrma1")</f>
         <v/>
       </c>
-      <c r="Q11" s="3">
+      <c r="R11" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R11" s="3">
+      <c r="S11" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4800,28 +4964,33 @@
           <t>Ph.D. Mechanical Engineering and Applied Mechanics, University of Pennsylvania 2010 | M.S.E. Mechanical Engineering and Applied Mechanics, University of Pennsylvania 2008 | B.S.E. Mechanical and Aerospace Engineering, Princeton University 2005 | Certificate. Robotics and Intelligent Systems, Princeton University 2005</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="3">
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous Collective Systems (ACS) Laboratory</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/acs/", "http://faculty.engineering.asu.edu/acs/")</f>
         <v/>
       </c>
-      <c r="N12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>KKup0OgAAAAJ</t>
         </is>
       </c>
-      <c r="P12" s="3">
+      <c r="Q12" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="Q12" s="3">
+      <c r="R12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R12" s="3">
+      <c r="S12" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4879,28 +5048,29 @@
           <t>Ph.D Degree at the  Department of Electrical, Computer, and Systems Engineering  at  Rensselaer Polytechnic Institute  in 2018 | Master's Degree at the  School of electrical and information engineering  at  Tianjin University  in 2014 | Bachelor's Degree at the  School of electrical and information engineering  at  Tianjin University  in 2011</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M13" s="3">
+      <c r="N13" s="3">
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="N13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="3">
+      <c r="O13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xzhe1", "https://search.asu.edu/profile/xzhe1")</f>
         <v/>
       </c>
-      <c r="Q13" s="3">
+      <c r="R13" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R13" s="3">
+      <c r="S13" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4952,19 +5122,20 @@
       </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="3">
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
         <v/>
       </c>
-      <c r="Q14" s="3">
+      <c r="R14" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R14" s="3">
+      <c r="S14" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5022,24 +5193,29 @@
           <t>Ph.D. Aeronautics and Astronautics, Stanford University 2006 | Bachelor's degree. Physics, University of Texas-Austin 1999 | Bachelor's degree. Aerospace Engineering, University of Texas-Austin 1999</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="3">
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Cybernetic Systems and Controls Laboratory (CSCL)</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="3">
         <f>HYPERLINK("http://control.asu.edu/", "http://control.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="3">
+      <c r="O15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mpeet", "https://search.asu.edu/profile/mpeet")</f>
         <v/>
       </c>
-      <c r="Q15" s="3">
+      <c r="R15" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R15" s="3">
+      <c r="S15" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5098,27 +5274,28 @@
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="3">
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="3">
         <f>HYPERLINK("http://wang.faculty.asu.edu/", "http://wang.faculty.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>LaUdx9gAAAAJ</t>
         </is>
       </c>
-      <c r="P16" s="3">
+      <c r="Q16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rywang", "https://search.asu.edu/profile/rywang")</f>
         <v/>
       </c>
-      <c r="Q16" s="3">
+      <c r="R16" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R16" s="3">
+      <c r="S16" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5177,23 +5354,24 @@
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="3">
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="3">
         <f>HYPERLINK("http://RESEARCHGATE.net/profile/Ryan_Milcarek", "http://RESEARCHGATE.net/profile/Ryan_Milcarek")</f>
         <v/>
       </c>
-      <c r="N17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O17" s="2" t="inlineStr"/>
-      <c r="P17" s="3">
+      <c r="O17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="Q17" s="3">
+      <c r="R17" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R17" s="3">
+      <c r="S17" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5243,25 +5421,26 @@
           <t>Ph.D. Aerospace Engineering, University of Michigan-Ann Arbor | M.S.E. Aerospace Engineering, University of Michigan-Ann Arbor | B.S. Aeronautical and Astronautical Engineering, The Ohio State University-Columbus</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>ENGRC 377 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O18" s="2" t="inlineStr"/>
-      <c r="P18" s="3">
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/attwl", "https://search.asu.edu/profile/attwl")</f>
         <v/>
       </c>
-      <c r="Q18" s="3">
+      <c r="R18" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R18" s="3">
+      <c r="S18" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5313,19 +5492,20 @@
       </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O19" s="2" t="inlineStr"/>
-      <c r="P19" s="3">
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="Q19" s="3">
+      <c r="R19" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R19" s="3">
+      <c r="S19" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5377,27 +5557,28 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
+          <t>Adaptive Intelligent Materials &amp; Systems (AIMS) Center</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>w3fU9E0AAAAJ</t>
         </is>
       </c>
-      <c r="P20" s="3">
+      <c r="Q20" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/chattopa", "https://search.asu.edu/profile/chattopa")</f>
         <v/>
       </c>
-      <c r="Q20" s="3">
+      <c r="R20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R20" s="3">
+      <c r="S20" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5455,29 +5636,30 @@
           <t>PhD Johns Hopkins University</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>HRx2lJQAAAAJ</t>
         </is>
       </c>
-      <c r="P21" s="3">
+      <c r="Q21" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/adscotti", "https://search.asu.edu/profile/adscotti")</f>
         <v/>
       </c>
-      <c r="Q21" s="3">
+      <c r="R21" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R21" s="3">
+      <c r="S21" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5533,30 +5715,35 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
+          <t>3D Energy Lab</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
           <t>551 E Tyler Mall ERC 363 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="M22" s="3">
+      <c r="N22" s="3">
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="N22" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="O22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>fs2d97sAAAAJ</t>
         </is>
       </c>
-      <c r="P22" s="3">
+      <c r="Q22" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/bkwon2", "https://search.asu.edu/profile/bkwon2")</f>
         <v/>
       </c>
-      <c r="Q22" s="3">
+      <c r="R22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R22" s="3">
+      <c r="S22" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5610,28 +5797,33 @@
           <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology, Atlanta 2013 | M.S. Mechanical Engineering, Clemson University, SC 2009 | M.S. Biomedical Engineering, Sharif University of Technology, Tehran, Iran 2007 | B.S. Mechanical Engineering, Iran University of Science and Technology, Tehran 2004</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="3">
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Bio-Inspired Robotics, Technology, and Healthcare Laboratory (BIRTH Lab)</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="3">
         <f>HYPERLINK("http://birth.asu.edu", "http://birth.asu.edu")</f>
         <v/>
       </c>
-      <c r="N23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>00Fepb0AAAAJ</t>
         </is>
       </c>
-      <c r="P23" s="3">
+      <c r="Q23" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hmarvi", "https://search.asu.edu/profile/hmarvi")</f>
         <v/>
       </c>
-      <c r="Q23" s="3">
+      <c r="R23" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=00Fepb0AAAAJ", "Scholar (00Fepb0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R23" s="3">
+      <c r="S23" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5681,28 +5873,29 @@
           <t>B.S. Mechanical and Aerospace Engineering, Seoul National University (2002) M.S. Mechanical and Aerospace Engineering, Seoul National University (2004) Ph.D Mechanical Engineering, Massachusetts Institute of Technology (2013)</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M24" s="3">
+      <c r="N24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/hlee", "https://faculty.engineering.asu.edu/hlee")</f>
         <v/>
       </c>
-      <c r="N24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O24" s="2" t="inlineStr"/>
-      <c r="P24" s="3">
+      <c r="O24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hlee234", "https://search.asu.edu/profile/hlee234")</f>
         <v/>
       </c>
-      <c r="Q24" s="3">
+      <c r="R24" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R24" s="3">
+      <c r="S24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5760,24 +5953,29 @@
           <t>PhD. Mechanical Engineering, University of Maryland-College Park 2007 | M.S. Mechanical Engineering, University of Maryland-College Park 2005 | PhD. Student, Mechanical Engineering, Isfahan University of Technology, Iran 2001-2002 | M.S. Mechanical Engineering, Isfahan University of Technology, Iran 2001 | B.S. Mechanical Engineering, Isfahan University of Technology, Iran 1999</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="3">
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing and Advanced Materials Characterization (MAGIC) Lab</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="3">
         <f>HYPERLINK("https://magic.asu.edu/", "https://magic.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O25" s="2" t="inlineStr"/>
-      <c r="P25" s="3">
+      <c r="O25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ljannesa", "https://search.asu.edu/profile/ljannesa")</f>
         <v/>
       </c>
-      <c r="Q25" s="3">
+      <c r="R25" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R25" s="3">
+      <c r="S25" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5835,25 +6033,26 @@
           <t>Postdoctoral Fellow, Tokyo Institute of Technology, Japan 1990-1992 | Ph.D. Mechanical Engineering, University of California, Berkeley 1990 | M.S. Mechanical Engineering, Massachusetts Institute of Technology 1987 | B. S. Mechanical Engineering, Tulane University, New Orleans, LA 1985</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>ENGRC 463 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O26" s="2" t="inlineStr"/>
-      <c r="P26" s="3">
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pphelan", "https://search.asu.edu/profile/pphelan")</f>
         <v/>
       </c>
-      <c r="Q26" s="3">
+      <c r="R26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R26" s="3">
+      <c r="S26" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5903,28 +6102,33 @@
           <t>Ph.D. Aeronautics and Astronautics, Stanford University 2006 | M.S. Management, State University Higher School of Economics, Moscow, Russia 2000 | M.S. Aeromechanics and Flight Engineering, Moscow Institute of Physics and Technology, Russia 1999 | B.S. Applied Mathematics and Physics, Moscow Institute of Physics and Technology, Russia 1997</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="3">
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Interdisciplinary Simulation and Modeling (ISiM) Lab</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="3">
         <f>HYPERLINK("https://isim.asu.edu", "https://isim.asu.edu")</f>
         <v/>
       </c>
-      <c r="N27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="O27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>_6o8MrUAAAAJ</t>
         </is>
       </c>
-      <c r="P27" s="3">
+      <c r="Q27" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="Q27" s="3">
+      <c r="R27" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R27" s="3">
+      <c r="S27" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5982,25 +6186,34 @@
           <t>Postdoc, Department of Mechanical and Aerospace Engineering, Princeton University Postdoc, Center for Nanophase Materials Sciences, Oak Ridge National Laboratory Ph.D., Major: Materials Science and Engineering; Minor: Applied Engineering Physics, Cornell University M.S., Major: Materials Science and Engineering; Minor: Applied Engineering Physics, Cornell University M.Phil., Mechanical Engineering, The University of Hong Kong B.Eng., Materials Science and Engineering, Hunan University</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Computational Materials Science and Design Lab</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
         <is>
           <t>4yYKCpUAAAAJ</t>
         </is>
       </c>
-      <c r="P28" s="3">
+      <c r="Q28" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hzhuang7", "https://search.asu.edu/profile/hzhuang7")</f>
         <v/>
       </c>
-      <c r="Q28" s="3">
+      <c r="R28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R28" s="3">
+      <c r="S28" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6050,28 +6263,29 @@
           <t>Ph.D. University of Illinois-Urbana-Champaign 1997 | M.S. National Taiwan University 1989 | B.S. National Central University,Taiwan 1987</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M29" s="3">
+      <c r="N29" s="3">
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="N29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O29" s="2" t="inlineStr"/>
-      <c r="P29" s="3">
+      <c r="O29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hhuang38", "https://search.asu.edu/profile/hhuang38")</f>
         <v/>
       </c>
-      <c r="Q29" s="3">
+      <c r="R29" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R29" s="3">
+      <c r="S29" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6131,30 +6345,35 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
+          <t>Nanomechanics Laboratory</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 355 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M30" s="3">
+      <c r="N30" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/jagan/", "http://faculty.engineering.asu.edu/jagan/")</f>
         <v/>
       </c>
-      <c r="N30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="O30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>ClqRIhIAAAAJ</t>
         </is>
       </c>
-      <c r="P30" s="3">
+      <c r="Q30" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jrajago1", "https://search.asu.edu/profile/jrajago1")</f>
         <v/>
       </c>
-      <c r="Q30" s="3">
+      <c r="R30" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R30" s="3">
+      <c r="S30" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6204,28 +6423,33 @@
           <t>Ph.D. Mechanical Engineering, Georgia Institute of Technology 2009 | M.S. Mechanical Engineering, Georgia Institute of Technology 2007 | B.S. Mechanical Engineering, Georgia Institute of Technology 2005</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="3">
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Nano-Bio-Thermal Engineering Laboratory</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/konrad/", "http://faculty.engineering.asu.edu/konrad/")</f>
         <v/>
       </c>
-      <c r="N31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
+      <c r="O31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>SWeAf4UAAAAJ</t>
         </is>
       </c>
-      <c r="P31" s="3">
+      <c r="Q31" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/krykacze", "https://search.asu.edu/profile/krykacze")</f>
         <v/>
       </c>
-      <c r="Q31" s="3">
+      <c r="R31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SWeAf4UAAAAJ", "Scholar (SWeAf4UAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R31" s="3">
+      <c r="S31" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6281,23 +6505,24 @@
       </c>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>9LWNC50AAAAJ</t>
         </is>
       </c>
-      <c r="P32" s="3">
+      <c r="Q32" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mingleiq", "https://search.asu.edu/profile/mingleiq")</f>
         <v/>
       </c>
-      <c r="Q32" s="3">
+      <c r="R32" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R32" s="3">
+      <c r="S32" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6355,28 +6580,29 @@
           <t>Ph.D. Manufacturing, Industrial Engineering, Purdue University 2015 | B.Sc. Materials Science and Engineering, University of Science and Technology of China 2009</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M33" s="3">
+      <c r="N33" s="3">
         <f>HYPERLINK("https://mmmplab.engineering.asu.edu/", "https://mmmplab.engineering.asu.edu/")</f>
         <v/>
       </c>
-      <c r="N33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="3">
+      <c r="O33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/qnian", "https://search.asu.edu/profile/qnian")</f>
         <v/>
       </c>
-      <c r="Q33" s="3">
+      <c r="R33" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R33" s="3">
+      <c r="S33" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6428,26 +6654,31 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
+          <t>Wind Energy and Atmospheric Boundary Layer Lab</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M34" s="3">
+      <c r="N34" s="3">
         <f>HYPERLINK("https://windlab.engineering.asu.edu/ronald-calhoun/", "https://windlab.engineering.asu.edu/ronald-calhoun/")</f>
         <v/>
       </c>
-      <c r="N34" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="3">
+      <c r="O34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcalhou", "https://search.asu.edu/profile/rcalhou")</f>
         <v/>
       </c>
-      <c r="Q34" s="3">
+      <c r="R34" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R34" s="3">
+      <c r="S34" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6501,28 +6732,33 @@
           <t>Ph.D., Purdue University 2021 | Master of Science, Harbin Institute of Technology, 2016 | Bachelor of Engineering, Harbin Institute of Technology, 2014</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="3">
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Intelligent Robotics and Interactive Systems Lab (IRIS Lab)</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="3">
         <f>HYPERLINK("https://irislab.tech/", "https://irislab.tech/")</f>
         <v/>
       </c>
-      <c r="N35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O35" s="2" t="inlineStr">
+      <c r="O35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>SoEC4h4AAAAJ</t>
         </is>
       </c>
-      <c r="P35" s="3">
+      <c r="Q35" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wjin34", "https://search.asu.edu/profile/wjin34")</f>
         <v/>
       </c>
-      <c r="Q35" s="3">
+      <c r="R35" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SoEC4h4AAAAJ", "Scholar (SoEC4h4AAAAJ)")</f>
         <v/>
       </c>
-      <c r="R35" s="3">
+      <c r="S35" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6578,23 +6814,28 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
+          <t>Prognostics and Health Management (PHM) Lab</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 409 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O36" s="2" t="inlineStr"/>
-      <c r="P36" s="3">
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yliu35", "https://search.asu.edu/profile/yliu35")</f>
         <v/>
       </c>
-      <c r="Q36" s="3">
+      <c r="R36" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R36" s="3">
+      <c r="S36" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6652,28 +6893,33 @@
           <t>Ph.D. in Industrial and Systems Engineering, University of Southern California, 2019 M.S. in Computer Science, University of Southern California, 2019 M.S. in Manufacturing Engineering, Nanjing University of Aeronautics and Astronautics, 2014 B.E. in Mechanical Engineering and Automation, Nanjing University of Aeronautics and Astronautics, 2011</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="3">
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Advanced Manufacturing and Bio-inspired Design Lab</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="3">
         <f>HYPERLINK("https://www.cindyxjli.com/", "https://www.cindyxjli.com/")</f>
         <v/>
       </c>
-      <c r="N37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O37" s="2" t="inlineStr">
+      <c r="O37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>tGQzHJIAAAAJ</t>
         </is>
       </c>
-      <c r="P37" s="3">
+      <c r="Q37" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xiangji5", "https://search.asu.edu/profile/xiangji5")</f>
         <v/>
       </c>
-      <c r="Q37" s="3">
+      <c r="R37" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=tGQzHJIAAAAJ", "Scholar (tGQzHJIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R37" s="3">
+      <c r="S37" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6728,20 +6974,25 @@
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O38" s="2" t="inlineStr"/>
-      <c r="P38" s="3">
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jimbo", "https://search.asu.edu/profile/jimbo")</f>
         <v/>
       </c>
-      <c r="Q38" s="3">
+      <c r="R38" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R38" s="3">
+      <c r="S38" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6791,25 +7042,26 @@
           <t>PhD The Ohio State University</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O39" s="2" t="inlineStr"/>
-      <c r="P39" s="3">
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/linli25", "https://search.asu.edu/profile/linli25")</f>
         <v/>
       </c>
-      <c r="Q39" s="3">
+      <c r="R39" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R39" s="3">
+      <c r="S39" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6860,20 +7112,25 @@
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O40" s="2" t="inlineStr"/>
-      <c r="P40" s="3">
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/marc03", "https://search.asu.edu/profile/marc03")</f>
         <v/>
       </c>
-      <c r="Q40" s="3">
+      <c r="R40" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R40" s="3">
+      <c r="S40" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6924,23 +7181,24 @@
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="3">
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/pperalta/", "https://faculty.engineering.asu.edu/pperalta/")</f>
         <v/>
       </c>
-      <c r="N41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O41" s="2" t="inlineStr"/>
-      <c r="P41" s="3">
+      <c r="O41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pperalta", "https://search.asu.edu/profile/pperalta")</f>
         <v/>
       </c>
-      <c r="Q41" s="3">
+      <c r="R41" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Pedro%20Peralta%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R41" s="3">
+      <c r="S41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6998,32 +7256,33 @@
           <t>Ph.D. Mechanical Science and Engineering, University of Illinois at Urbana-Champaign 2012</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M42" s="3">
+      <c r="N42" s="3">
         <f>HYPERLINK("https://wonmokang3.wixsite.com/website", "https://wonmokang3.wixsite.com/website")</f>
         <v/>
       </c>
-      <c r="N42" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
+      <c r="O42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
         <is>
           <t>bHyyOTAAAAAJ</t>
         </is>
       </c>
-      <c r="P42" s="3">
+      <c r="Q42" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wkang16", "https://search.asu.edu/profile/wkang16")</f>
         <v/>
       </c>
-      <c r="Q42" s="3">
+      <c r="R42" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=bHyyOTAAAAAJ", "Scholar (bHyyOTAAAAAJ)")</f>
         <v/>
       </c>
-      <c r="R42" s="3">
+      <c r="S42" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7073,25 +7332,22 @@
           <t>Ph.D. Mechanical Engineering, University of Michigan 2011 | M.S. Mechanical Engineering, University of Michigan 2009 | B.S. Automative Engineering, Tsinghua University, China 2007</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>GWC 464 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr"/>
-      <c r="N43" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O43" s="2" t="inlineStr"/>
-      <c r="P43" s="3">
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P43" s="2" t="inlineStr"/>
+      <c r="Q43" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yren32", "https://search.asu.edu/profile/yren32")</f>
         <v/>
       </c>
-      <c r="Q43" s="3">
+      <c r="R43" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R43" s="3">
+      <c r="S43" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7131,19 +7387,20 @@
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="b">
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="O44" s="2" t="inlineStr"/>
-      <c r="P44" s="3">
+      <c r="P44" s="2" t="inlineStr"/>
+      <c r="Q44" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/dspeaks2", "https://search.asu.edu/profile/dspeaks2")</f>
         <v/>
       </c>
-      <c r="Q44" s="3">
+      <c r="R44" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Derrick%20Speaks%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R44" s="3">
+      <c r="S44" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7185,25 +7442,26 @@
           <t>Ph.D. in Mechanical Engineering 2022 - University of Utah B.S./M.S.in Mechanical Engineering 2018 - University of Utah</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>Campus: Otherus</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr"/>
-      <c r="N45" s="2" t="b">
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="O45" s="2" t="inlineStr"/>
-      <c r="P45" s="3">
+      <c r="P45" s="2" t="inlineStr"/>
+      <c r="Q45" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ejande22", "https://search.asu.edu/profile/ejande22")</f>
         <v/>
       </c>
-      <c r="Q45" s="3">
+      <c r="R45" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Erik%20Andersen%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R45" s="3">
+      <c r="S45" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7243,19 +7501,20 @@
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="b">
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="O46" s="2" t="inlineStr"/>
-      <c r="P46" s="3">
+      <c r="P46" s="2" t="inlineStr"/>
+      <c r="Q46" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/iychang", "https://search.asu.edu/profile/iychang")</f>
         <v/>
       </c>
-      <c r="Q46" s="3">
+      <c r="R46" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ivy%20Chang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R46" s="3">
+      <c r="S46" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7295,19 +7554,20 @@
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
-      <c r="N47" s="2" t="b">
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="O47" s="2" t="inlineStr"/>
-      <c r="P47" s="3">
+      <c r="P47" s="2" t="inlineStr"/>
+      <c r="Q47" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jdwilbu1", "https://search.asu.edu/profile/jdwilbu1")</f>
         <v/>
       </c>
-      <c r="Q47" s="3">
+      <c r="R47" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Joshua%20Wilbur%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R47" s="3">
+      <c r="S47" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7347,19 +7607,20 @@
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="b">
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="O48" s="2" t="inlineStr"/>
-      <c r="P48" s="3">
+      <c r="P48" s="2" t="inlineStr"/>
+      <c r="Q48" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcruzloz", "https://search.asu.edu/profile/rcruzloz")</f>
         <v/>
       </c>
-      <c r="Q48" s="3">
+      <c r="R48" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ricardo%20Cruz%20Lozano%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R48" s="3">
+      <c r="S48" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7397,25 +7658,26 @@
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="M49" s="2" t="inlineStr"/>
-      <c r="N49" s="2" t="b">
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="O49" s="2" t="inlineStr"/>
-      <c r="P49" s="3">
+      <c r="P49" s="2" t="inlineStr"/>
+      <c r="Q49" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/skosara2", "https://search.asu.edu/profile/skosara2")</f>
         <v/>
       </c>
-      <c r="Q49" s="3">
+      <c r="R49" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Srinivas%20Chakravarthi%20Kosaraju%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="R49" s="3">
+      <c r="S49" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7423,223 +7685,223 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId149"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId154"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId159"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S44" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P45" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P47" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId210"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId214"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId218"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scrape deep lab site intelligence: hiring status, required prerequisites, funding sponsors, and code repositories
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S43"/>
+  <dimension ref="A1:X43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -470,13 +470,18 @@
     <col width="65" customWidth="1" min="10" max="10"/>
     <col width="65" customWidth="1" min="11" max="11"/>
     <col width="65" customWidth="1" min="12" max="12"/>
-    <col width="46" customWidth="1" min="13" max="13"/>
-    <col width="49" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="49" customWidth="1" min="17" max="17"/>
-    <col width="32" customWidth="1" min="18" max="18"/>
+    <col width="65" customWidth="1" min="13" max="13"/>
+    <col width="53" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="65" customWidth="1" min="16" max="16"/>
+    <col width="56" customWidth="1" min="17" max="17"/>
+    <col width="46" customWidth="1" min="18" max="18"/>
     <col width="49" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="49" customWidth="1" min="22" max="22"/>
+    <col width="32" customWidth="1" min="23" max="23"/>
+    <col width="49" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,35 +547,60 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Actively Hiring / Openings</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Target Skills / Prerequisites</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Funding Sponsors</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Software / Code Repo</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Latest Project / Highlight</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Office Location</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Lab / Personal Website</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Scholar ID</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Profile URL</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Google Scholar URL</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Directory URL</t>
         </is>
@@ -627,23 +657,44 @@
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="3">
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>CFD</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>AFOSR</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>School for Engineering of Matter, Transport &amp; Energy</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="3">
         <f>HYPERLINK("https://kasbaoui.bitbucket.io", "https://kasbaoui.bitbucket.io")</f>
         <v/>
       </c>
-      <c r="O2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="3">
+      <c r="T2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
         <v/>
       </c>
-      <c r="R2" s="3">
+      <c r="W2" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S2" s="3">
+      <c r="X2" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -704,26 +755,43 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
+          <t>Multiple UG/MS research positions available for Fall 2024 (volunteer) and Spring/Summer 2025 (possible FURI / MORE support)</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>NASA, NSF</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>News&amp;Awards</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N3" s="3">
+      <c r="S3" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/lpwang", "http://faculty.engineering.asu.edu/lpwang")</f>
         <v/>
       </c>
-      <c r="O3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="3">
+      <c r="T3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
         <v/>
       </c>
-      <c r="R3" s="3">
+      <c r="W3" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S3" s="3">
+      <c r="X3" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -782,28 +850,33 @@
           <t>Computational Mechanics Lab</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 353 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="N4" s="3">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Multiscale polymer analysis</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="3">
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="O4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="3">
+      <c r="T4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/joswald1", "https://search.asu.edu/profile/joswald1")</f>
         <v/>
       </c>
-      <c r="R4" s="3">
+      <c r="W4" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S4" s="3">
+      <c r="X4" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -866,28 +939,45 @@
           <t>Sun Robotics Lab</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="3">
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Dec 19, 2025 We have two openings for fully supported summer interns through SURI program at ASU</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Mission and Core Values</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S5" s="3">
         <f>HYPERLINK("https://sunroboticslab.github.io", "https://sunroboticslab.github.io")</f>
         <v/>
       </c>
-      <c r="O5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
         <is>
           <t>fjUoHOsAAAAJ</t>
         </is>
       </c>
-      <c r="Q5" s="3">
+      <c r="V5" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jsun165", "https://search.asu.edu/profile/jsun165")</f>
         <v/>
       </c>
-      <c r="R5" s="3">
+      <c r="W5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fjUoHOsAAAAJ", "Scholar (fjUoHOsAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S5" s="3">
+      <c r="X5" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -940,23 +1030,32 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 361 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
         <is>
           <t>xT-lX9sAAAAJ</t>
         </is>
       </c>
-      <c r="Q6" s="3">
+      <c r="V6" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="R6" s="3">
+      <c r="W6" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S6" s="3">
+      <c r="X6" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1013,23 +1112,28 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
         <is>
           <t>DKc-AgcAAAAJ</t>
         </is>
       </c>
-      <c r="Q7" s="3">
+      <c r="V7" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kramesh2", "https://search.asu.edu/profile/kramesh2")</f>
         <v/>
       </c>
-      <c r="R7" s="3">
+      <c r="W7" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S7" s="3">
+      <c r="X7" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1094,30 +1198,43 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t>Actively seeking graduate students (see bio/lab link)</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Python, PyTorch, ROS, ROS2, C/C++, Linear Algebra</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
           <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="N8" s="3">
+      <c r="S8" s="3">
         <f>HYPERLINK("https://sites.google.com/asu.edu/kunalgarg/", "https://sites.google.com/asu.edu/kunalgarg/")</f>
         <v/>
       </c>
-      <c r="O8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="T8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>vs3pl-8AAAAJ</t>
         </is>
       </c>
-      <c r="Q8" s="3">
+      <c r="V8" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
         <v/>
       </c>
-      <c r="R8" s="3">
+      <c r="W8" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S8" s="3">
+      <c r="X8" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1180,28 +1297,45 @@
           <t>Optimization, Autonomy, and Soft Intelligence Systems (OASIS) Lab</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="3">
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>Ocean and Soft Intelligent Structure Interaction Lab</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>ERC 485 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
+      <c r="S9" s="3">
         <f>HYPERLINK("https://sites.google.com/view/oasislabasu", "https://sites.google.com/view/oasislabasu")</f>
         <v/>
       </c>
-      <c r="O9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="T9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t>2xQTOc0AAAAJ</t>
         </is>
       </c>
-      <c r="Q9" s="3">
+      <c r="V9" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
-      <c r="R9" s="3">
+      <c r="W9" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S9" s="3">
+      <c r="X9" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1260,28 +1394,37 @@
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Want to be part of CMAT Lab?</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="N10" s="3">
+      <c r="S10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/cmat/", "https://faculty.engineering.asu.edu/cmat/")</f>
         <v/>
       </c>
-      <c r="O10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P10" s="2" t="inlineStr"/>
-      <c r="Q10" s="3">
+      <c r="T10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
         <v/>
       </c>
-      <c r="R10" s="3">
+      <c r="W10" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S10" s="3">
+      <c r="X10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1338,23 +1481,28 @@
       </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
         <is>
           <t>yv6aCW8AAAAJ</t>
         </is>
       </c>
-      <c r="Q11" s="3">
+      <c r="V11" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mherrma1", "https://search.asu.edu/profile/mherrma1")</f>
         <v/>
       </c>
-      <c r="R11" s="3">
+      <c r="W11" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S11" s="3">
+      <c r="X11" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1418,27 +1566,36 @@
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="3">
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S12" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/acs/", "http://faculty.engineering.asu.edu/acs/")</f>
         <v/>
       </c>
-      <c r="O12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="T12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
         <is>
           <t>KKup0OgAAAAJ</t>
         </is>
       </c>
-      <c r="Q12" s="3">
+      <c r="V12" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="R12" s="3">
+      <c r="W12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S12" s="3">
+      <c r="X12" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1497,28 +1654,33 @@
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N13" s="3">
+      <c r="S13" s="3">
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="O13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="3">
+      <c r="T13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xzhe1", "https://search.asu.edu/profile/xzhe1")</f>
         <v/>
       </c>
-      <c r="R13" s="3">
+      <c r="W13" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S13" s="3">
+      <c r="X13" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1571,19 +1733,24 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="3">
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
         <v/>
       </c>
-      <c r="R14" s="3">
+      <c r="W14" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S14" s="3">
+      <c r="X14" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1647,23 +1814,28 @@
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="3">
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="3">
         <f>HYPERLINK("http://control.asu.edu/", "http://control.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="3">
+      <c r="T15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mpeet", "https://search.asu.edu/profile/mpeet")</f>
         <v/>
       </c>
-      <c r="R15" s="3">
+      <c r="W15" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S15" s="3">
+      <c r="X15" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1723,27 +1895,32 @@
       </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="3">
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="3">
         <f>HYPERLINK("http://wang.faculty.asu.edu/", "http://wang.faculty.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
+      <c r="T16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
         <is>
           <t>LaUdx9gAAAAJ</t>
         </is>
       </c>
-      <c r="Q16" s="3">
+      <c r="V16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rywang", "https://search.asu.edu/profile/rywang")</f>
         <v/>
       </c>
-      <c r="R16" s="3">
+      <c r="W16" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S16" s="3">
+      <c r="X16" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1803,23 +1980,36 @@
       </c>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="3">
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 465 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
+      <c r="S17" s="3">
         <f>HYPERLINK("http://RESEARCHGATE.net/profile/Ryan_Milcarek", "http://RESEARCHGATE.net/profile/Ryan_Milcarek")</f>
         <v/>
       </c>
-      <c r="O17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="3">
+      <c r="T17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>m-Pb6g2pm2UC</t>
+        </is>
+      </c>
+      <c r="V17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="R17" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
-        <v/>
-      </c>
-      <c r="S17" s="3">
+      <c r="W17" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
+        <v/>
+      </c>
+      <c r="X17" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1870,25 +2060,30 @@
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
         <is>
           <t>ENGRC 377 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="3">
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/attwl", "https://search.asu.edu/profile/attwl")</f>
         <v/>
       </c>
-      <c r="R18" s="3">
+      <c r="W18" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S18" s="3">
+      <c r="X18" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1941,19 +2136,32 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="3">
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>OmBV67MAAAAJ</t>
+        </is>
+      </c>
+      <c r="V19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="R19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
-        <v/>
-      </c>
-      <c r="S19" s="3">
+      <c r="W19" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="X19" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2010,23 +2218,28 @@
       </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
         <is>
           <t>w3fU9E0AAAAJ</t>
         </is>
       </c>
-      <c r="Q20" s="3">
+      <c r="V20" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/chattopa", "https://search.asu.edu/profile/chattopa")</f>
         <v/>
       </c>
-      <c r="R20" s="3">
+      <c r="W20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S20" s="3">
+      <c r="X20" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2085,29 +2298,34 @@
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
         <is>
           <t>HRx2lJQAAAAJ</t>
         </is>
       </c>
-      <c r="Q21" s="3">
+      <c r="V21" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/adscotti", "https://search.asu.edu/profile/adscotti")</f>
         <v/>
       </c>
-      <c r="R21" s="3">
+      <c r="W21" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S21" s="3">
+      <c r="X21" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2166,32 +2384,45 @@
           <t>3D Energy Lab</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>3D Energy Device Laboratory</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 363 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="N22" s="3">
+      <c r="S22" s="3">
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="O22" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
+      <c r="T22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
         <is>
           <t>fs2d97sAAAAJ</t>
         </is>
       </c>
-      <c r="Q22" s="3">
+      <c r="V22" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/bkwon2", "https://search.asu.edu/profile/bkwon2")</f>
         <v/>
       </c>
-      <c r="R22" s="3">
+      <c r="W22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S22" s="3">
+      <c r="X22" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2251,27 +2482,36 @@
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="3">
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S23" s="3">
         <f>HYPERLINK("http://birth.asu.edu", "http://birth.asu.edu")</f>
         <v/>
       </c>
-      <c r="O23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
+      <c r="T23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
         <is>
           <t>00Fepb0AAAAJ</t>
         </is>
       </c>
-      <c r="Q23" s="3">
+      <c r="V23" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hmarvi", "https://search.asu.edu/profile/hmarvi")</f>
         <v/>
       </c>
-      <c r="R23" s="3">
+      <c r="W23" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=00Fepb0AAAAJ", "Scholar (00Fepb0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S23" s="3">
+      <c r="X23" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2322,28 +2562,33 @@
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N24" s="3">
+      <c r="S24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/hlee", "https://faculty.engineering.asu.edu/hlee")</f>
         <v/>
       </c>
-      <c r="O24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P24" s="2" t="inlineStr"/>
-      <c r="Q24" s="3">
+      <c r="T24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U24" s="2" t="inlineStr"/>
+      <c r="V24" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hlee234", "https://search.asu.edu/profile/hlee234")</f>
         <v/>
       </c>
-      <c r="R24" s="3">
+      <c r="W24" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S24" s="3">
+      <c r="X24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2407,23 +2652,28 @@
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="3">
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="3">
         <f>HYPERLINK("https://magic.asu.edu/", "https://magic.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="inlineStr"/>
-      <c r="Q25" s="3">
+      <c r="T25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U25" s="2" t="inlineStr"/>
+      <c r="V25" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ljannesa", "https://search.asu.edu/profile/ljannesa")</f>
         <v/>
       </c>
-      <c r="R25" s="3">
+      <c r="W25" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S25" s="3">
+      <c r="X25" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2482,25 +2732,30 @@
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
         <is>
           <t>ENGRC 463 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="3">
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U26" s="2" t="inlineStr"/>
+      <c r="V26" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pphelan", "https://search.asu.edu/profile/pphelan")</f>
         <v/>
       </c>
-      <c r="R26" s="3">
+      <c r="W26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S26" s="3">
+      <c r="X26" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2556,27 +2811,32 @@
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="3">
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="3">
         <f>HYPERLINK("https://isim.asu.edu", "https://isim.asu.edu")</f>
         <v/>
       </c>
-      <c r="O27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
+      <c r="T27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
         <is>
           <t>_6o8MrUAAAAJ</t>
         </is>
       </c>
-      <c r="Q27" s="3">
+      <c r="V27" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="R27" s="3">
+      <c r="W27" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S27" s="3">
+      <c r="X27" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2639,29 +2899,30 @@
           <t>Computational Materials Science and Design Lab</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
         <is>
           <t>4yYKCpUAAAAJ</t>
         </is>
       </c>
-      <c r="Q28" s="3">
+      <c r="V28" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hzhuang7", "https://search.asu.edu/profile/hzhuang7")</f>
         <v/>
       </c>
-      <c r="R28" s="3">
+      <c r="W28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S28" s="3">
+      <c r="X28" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2712,28 +2973,33 @@
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="N29" s="3">
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>Log in to www_public</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="3">
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="O29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P29" s="2" t="inlineStr"/>
-      <c r="Q29" s="3">
+      <c r="T29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U29" s="2" t="inlineStr"/>
+      <c r="V29" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hhuang38", "https://search.asu.edu/profile/hhuang38")</f>
         <v/>
       </c>
-      <c r="R29" s="3">
+      <c r="W29" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S29" s="3">
+      <c r="X29" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2796,32 +3062,41 @@
           <t>Nanomechanics Laboratory</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr"/>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>Nanostructured Materials</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
         <is>
           <t>ENGRC 355 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N30" s="3">
+      <c r="S30" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/jagan/", "http://faculty.engineering.asu.edu/jagan/")</f>
         <v/>
       </c>
-      <c r="O30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
+      <c r="T30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
         <is>
           <t>ClqRIhIAAAAJ</t>
         </is>
       </c>
-      <c r="Q30" s="3">
+      <c r="V30" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jrajago1", "https://search.asu.edu/profile/jrajago1")</f>
         <v/>
       </c>
-      <c r="R30" s="3">
+      <c r="W30" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S30" s="3">
+      <c r="X30" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2877,27 +3152,36 @@
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="3">
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 309 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
+      <c r="S31" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/konrad/", "http://faculty.engineering.asu.edu/konrad/")</f>
         <v/>
       </c>
-      <c r="O31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
+      <c r="T31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
         <is>
           <t>SWeAf4UAAAAJ</t>
         </is>
       </c>
-      <c r="Q31" s="3">
+      <c r="V31" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/krykacze", "https://search.asu.edu/profile/krykacze")</f>
         <v/>
       </c>
-      <c r="R31" s="3">
+      <c r="W31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SWeAf4UAAAAJ", "Scholar (SWeAf4UAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S31" s="3">
+      <c r="X31" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2954,23 +3238,32 @@
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
         <is>
           <t>9LWNC50AAAAJ</t>
         </is>
       </c>
-      <c r="Q32" s="3">
+      <c r="V32" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mingleiq", "https://search.asu.edu/profile/mingleiq")</f>
         <v/>
       </c>
-      <c r="R32" s="3">
+      <c r="W32" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S32" s="3">
+      <c r="X32" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3029,28 +3322,33 @@
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N33" s="3">
+      <c r="S33" s="3">
         <f>HYPERLINK("https://mmmplab.engineering.asu.edu/", "https://mmmplab.engineering.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="3">
+      <c r="T33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U33" s="2" t="inlineStr"/>
+      <c r="V33" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/qnian", "https://search.asu.edu/profile/qnian")</f>
         <v/>
       </c>
-      <c r="R33" s="3">
+      <c r="W33" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S33" s="3">
+      <c r="X33" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3105,28 +3403,33 @@
           <t>Wind Energy and Atmospheric Boundary Layer Lab</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr">
         <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N34" s="3">
+      <c r="S34" s="3">
         <f>HYPERLINK("https://windlab.engineering.asu.edu/ronald-calhoun/", "https://windlab.engineering.asu.edu/ronald-calhoun/")</f>
         <v/>
       </c>
-      <c r="O34" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="3">
+      <c r="T34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U34" s="2" t="inlineStr"/>
+      <c r="V34" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcalhou", "https://search.asu.edu/profile/rcalhou")</f>
         <v/>
       </c>
-      <c r="R34" s="3">
+      <c r="W34" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S34" s="3">
+      <c r="X34" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3186,27 +3489,48 @@
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="3">
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/asu-iris</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>Recent Updates</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S35" s="3">
         <f>HYPERLINK("https://irislab.tech/", "https://irislab.tech/")</f>
         <v/>
       </c>
-      <c r="O35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P35" s="2" t="inlineStr">
+      <c r="T35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
         <is>
           <t>SoEC4h4AAAAJ</t>
         </is>
       </c>
-      <c r="Q35" s="3">
+      <c r="V35" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wjin34", "https://search.asu.edu/profile/wjin34")</f>
         <v/>
       </c>
-      <c r="R35" s="3">
+      <c r="W35" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SoEC4h4AAAAJ", "Scholar (SoEC4h4AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S35" s="3">
+      <c r="X35" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3265,25 +3589,30 @@
           <t>Prognostics and Health Management (PHM) Lab</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="R36" s="2" t="inlineStr">
         <is>
           <t>ENGRC 409 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P36" s="2" t="inlineStr"/>
-      <c r="Q36" s="3">
+      <c r="S36" s="2" t="inlineStr"/>
+      <c r="T36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U36" s="2" t="inlineStr"/>
+      <c r="V36" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yliu35", "https://search.asu.edu/profile/yliu35")</f>
         <v/>
       </c>
-      <c r="R36" s="3">
+      <c r="W36" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S36" s="3">
+      <c r="X36" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3347,27 +3676,40 @@
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="3">
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="3">
         <f>HYPERLINK("https://www.cindyxjli.com/", "https://www.cindyxjli.com/")</f>
         <v/>
       </c>
-      <c r="O37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P37" s="2" t="inlineStr">
+      <c r="T37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
         <is>
           <t>tGQzHJIAAAAJ</t>
         </is>
       </c>
-      <c r="Q37" s="3">
+      <c r="V37" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xiangji5", "https://search.asu.edu/profile/xiangji5")</f>
         <v/>
       </c>
-      <c r="R37" s="3">
+      <c r="W37" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=tGQzHJIAAAAJ", "Scholar (tGQzHJIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S37" s="3">
+      <c r="X37" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3422,25 +3764,30 @@
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr">
         <is>
           <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr"/>
-      <c r="O38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P38" s="2" t="inlineStr"/>
-      <c r="Q38" s="3">
+      <c r="S38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U38" s="2" t="inlineStr"/>
+      <c r="V38" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jimbo", "https://search.asu.edu/profile/jimbo")</f>
         <v/>
       </c>
-      <c r="R38" s="3">
+      <c r="W38" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S38" s="3">
+      <c r="X38" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3491,25 +3838,30 @@
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N39" s="2" t="inlineStr"/>
-      <c r="O39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P39" s="2" t="inlineStr"/>
-      <c r="Q39" s="3">
+      <c r="S39" s="2" t="inlineStr"/>
+      <c r="T39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U39" s="2" t="inlineStr"/>
+      <c r="V39" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/linli25", "https://search.asu.edu/profile/linli25")</f>
         <v/>
       </c>
-      <c r="R39" s="3">
+      <c r="W39" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S39" s="3">
+      <c r="X39" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3560,25 +3912,30 @@
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr">
         <is>
           <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr"/>
-      <c r="O40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="3">
+      <c r="S40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U40" s="2" t="inlineStr"/>
+      <c r="V40" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/marc03", "https://search.asu.edu/profile/marc03")</f>
         <v/>
       </c>
-      <c r="R40" s="3">
+      <c r="W40" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S40" s="3">
+      <c r="X40" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3630,23 +3987,32 @@
       </c>
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="3">
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 352 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/pperalta/", "https://faculty.engineering.asu.edu/pperalta/")</f>
         <v/>
       </c>
-      <c r="O41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P41" s="2" t="inlineStr"/>
-      <c r="Q41" s="3">
+      <c r="T41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pperalta", "https://search.asu.edu/profile/pperalta")</f>
         <v/>
       </c>
-      <c r="R41" s="3">
+      <c r="W41" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Pedro%20Peralta%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S41" s="3">
+      <c r="X41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3707,30 +4073,47 @@
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr">
         <is>
+          <t>Welcome and we are looking forward to working with Dr</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>NSF, ONR</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>Highlighted as a cover in Small</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N42" s="3">
+      <c r="S42" s="3">
         <f>HYPERLINK("https://wonmokang3.wixsite.com/website", "https://wonmokang3.wixsite.com/website")</f>
         <v/>
       </c>
-      <c r="O42" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
+      <c r="T42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
         <is>
           <t>bHyyOTAAAAAJ</t>
         </is>
       </c>
-      <c r="Q42" s="3">
+      <c r="V42" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wkang16", "https://search.asu.edu/profile/wkang16")</f>
         <v/>
       </c>
-      <c r="R42" s="3">
+      <c r="W42" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=bHyyOTAAAAAJ", "Scholar (bHyyOTAAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S42" s="3">
+      <c r="X42" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3783,19 +4166,28 @@
       <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr"/>
-      <c r="O43" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="O43" s="2" t="inlineStr"/>
       <c r="P43" s="2" t="inlineStr"/>
-      <c r="Q43" s="3">
+      <c r="Q43" s="2" t="inlineStr"/>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>GWC 464 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="inlineStr"/>
+      <c r="T43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U43" s="2" t="inlineStr"/>
+      <c r="V43" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yren32", "https://search.asu.edu/profile/yren32")</f>
         <v/>
       </c>
-      <c r="R43" s="3">
+      <c r="W43" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S43" s="3">
+      <c r="X43" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3803,199 +4195,199 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W8" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W9" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W15" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V16" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W16" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V17" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W17" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V18" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W18" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V19" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W19" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V20" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W20" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V21" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W21" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V22" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W22" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V23" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W23" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V24" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W24" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V25" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W25" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V26" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W26" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V27" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W27" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V28" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W28" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V29" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W29" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V30" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W30" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V31" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W31" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V32" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W32" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X32" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V33" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W33" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId149"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V34" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W34" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X34" r:id="rId154"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V35" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W35" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId159"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V36" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W36" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X36" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V37" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W37" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V38" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W38" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X38" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V39" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W39" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V40" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W40" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V41" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W41" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V42" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W42" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X42" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V43" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W43" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X43" r:id="rId194"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4007,7 +4399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S49"/>
+  <dimension ref="A1:X49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4022,13 +4414,18 @@
     <col width="65" customWidth="1" min="10" max="10"/>
     <col width="65" customWidth="1" min="11" max="11"/>
     <col width="65" customWidth="1" min="12" max="12"/>
-    <col width="46" customWidth="1" min="13" max="13"/>
-    <col width="49" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="49" customWidth="1" min="17" max="17"/>
-    <col width="32" customWidth="1" min="18" max="18"/>
+    <col width="65" customWidth="1" min="13" max="13"/>
+    <col width="53" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="65" customWidth="1" min="16" max="16"/>
+    <col width="56" customWidth="1" min="17" max="17"/>
+    <col width="46" customWidth="1" min="18" max="18"/>
     <col width="49" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="49" customWidth="1" min="22" max="22"/>
+    <col width="32" customWidth="1" min="23" max="23"/>
+    <col width="49" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4094,35 +4491,60 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Actively Hiring / Openings</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Target Skills / Prerequisites</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Funding Sponsors</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Software / Code Repo</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Latest Project / Highlight</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Office Location</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Lab / Personal Website</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Scholar ID</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Profile URL</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Google Scholar URL</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Directory URL</t>
         </is>
@@ -4179,23 +4601,44 @@
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="3">
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>CFD</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>AFOSR</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>School for Engineering of Matter, Transport &amp; Energy</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="3">
         <f>HYPERLINK("https://kasbaoui.bitbucket.io", "https://kasbaoui.bitbucket.io")</f>
         <v/>
       </c>
-      <c r="O2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="3">
+      <c r="T2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mkasbaou", "https://search.asu.edu/profile/mkasbaou")</f>
         <v/>
       </c>
-      <c r="R2" s="3">
+      <c r="W2" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Mohamed%20Houssem%20Kasbaoui%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S2" s="3">
+      <c r="X2" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4256,26 +4699,43 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
+          <t>Multiple UG/MS research positions available for Fall 2024 (volunteer) and Spring/Summer 2025 (possible FURI / MORE support)</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>NASA, NSF</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>News&amp;Awards</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N3" s="3">
+      <c r="S3" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/lpwang", "http://faculty.engineering.asu.edu/lpwang")</f>
         <v/>
       </c>
-      <c r="O3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="3">
+      <c r="T3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/lwang78", "https://search.asu.edu/profile/lwang78")</f>
         <v/>
       </c>
-      <c r="R3" s="3">
+      <c r="W3" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Liping%20Wang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S3" s="3">
+      <c r="X3" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4334,28 +4794,33 @@
           <t>Computational Mechanics Lab</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 353 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="N4" s="3">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Multiscale polymer analysis</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="3">
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="O4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="3">
+      <c r="T4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/joswald1", "https://search.asu.edu/profile/joswald1")</f>
         <v/>
       </c>
-      <c r="R4" s="3">
+      <c r="W4" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jay%20Oswald%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S4" s="3">
+      <c r="X4" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4418,28 +4883,45 @@
           <t>Sun Robotics Lab</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="3">
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Dec 19, 2025 We have two openings for fully supported summer interns through SURI program at ASU</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Mission and Core Values</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S5" s="3">
         <f>HYPERLINK("https://sunroboticslab.github.io", "https://sunroboticslab.github.io")</f>
         <v/>
       </c>
-      <c r="O5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
         <is>
           <t>fjUoHOsAAAAJ</t>
         </is>
       </c>
-      <c r="Q5" s="3">
+      <c r="V5" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jsun165", "https://search.asu.edu/profile/jsun165")</f>
         <v/>
       </c>
-      <c r="R5" s="3">
+      <c r="W5" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fjUoHOsAAAAJ", "Scholar (fjUoHOsAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S5" s="3">
+      <c r="X5" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4492,23 +4974,32 @@
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 361 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
         <is>
           <t>xT-lX9sAAAAJ</t>
         </is>
       </c>
-      <c r="Q6" s="3">
+      <c r="V6" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="R6" s="3">
+      <c r="W6" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=xT-lX9sAAAAJ", "Scholar (xT-lX9sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S6" s="3">
+      <c r="X6" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4565,23 +5056,28 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
         <is>
           <t>DKc-AgcAAAAJ</t>
         </is>
       </c>
-      <c r="Q7" s="3">
+      <c r="V7" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kramesh2", "https://search.asu.edu/profile/kramesh2")</f>
         <v/>
       </c>
-      <c r="R7" s="3">
+      <c r="W7" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=DKc-AgcAAAAJ", "Scholar (DKc-AgcAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S7" s="3">
+      <c r="X7" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4646,30 +5142,43 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t>Actively seeking graduate students (see bio/lab link)</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Python, PyTorch, ROS, ROS2, C/C++, Linear Algebra</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
           <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="N8" s="3">
+      <c r="S8" s="3">
         <f>HYPERLINK("https://sites.google.com/asu.edu/kunalgarg/", "https://sites.google.com/asu.edu/kunalgarg/")</f>
         <v/>
       </c>
-      <c r="O8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="T8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
         <is>
           <t>vs3pl-8AAAAJ</t>
         </is>
       </c>
-      <c r="Q8" s="3">
+      <c r="V8" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/kgarg24", "https://search.asu.edu/profile/kgarg24")</f>
         <v/>
       </c>
-      <c r="R8" s="3">
+      <c r="W8" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=vs3pl-8AAAAJ", "Scholar (vs3pl-8AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S8" s="3">
+      <c r="X8" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4732,28 +5241,45 @@
           <t>Optimization, Autonomy, and Soft Intelligence Systems (OASIS) Lab</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="3">
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>Ocean and Soft Intelligent Structure Interaction Lab</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>ERC 485 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
+      <c r="S9" s="3">
         <f>HYPERLINK("https://sites.google.com/view/oasislabasu", "https://sites.google.com/view/oasislabasu")</f>
         <v/>
       </c>
-      <c r="O9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="T9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t>2xQTOc0AAAAJ</t>
         </is>
       </c>
-      <c r="Q9" s="3">
+      <c r="V9" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
-      <c r="R9" s="3">
+      <c r="W9" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=2xQTOc0AAAAJ", "Scholar (2xQTOc0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S9" s="3">
+      <c r="X9" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4812,28 +5338,37 @@
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Want to be part of CMAT Lab?</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="N10" s="3">
+      <c r="S10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/cmat/", "https://faculty.engineering.asu.edu/cmat/")</f>
         <v/>
       </c>
-      <c r="O10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P10" s="2" t="inlineStr"/>
-      <c r="Q10" s="3">
+      <c r="T10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/gpathiko", "https://search.asu.edu/profile/gpathiko")</f>
         <v/>
       </c>
-      <c r="R10" s="3">
+      <c r="W10" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Gokul%20Pathikonda%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S10" s="3">
+      <c r="X10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4890,23 +5425,28 @@
       </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr"/>
-      <c r="O11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
         <is>
           <t>yv6aCW8AAAAJ</t>
         </is>
       </c>
-      <c r="Q11" s="3">
+      <c r="V11" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mherrma1", "https://search.asu.edu/profile/mherrma1")</f>
         <v/>
       </c>
-      <c r="R11" s="3">
+      <c r="W11" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=yv6aCW8AAAAJ", "Scholar (yv6aCW8AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S11" s="3">
+      <c r="X11" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4970,27 +5510,36 @@
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="3">
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S12" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/acs/", "http://faculty.engineering.asu.edu/acs/")</f>
         <v/>
       </c>
-      <c r="O12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="T12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
         <is>
           <t>KKup0OgAAAAJ</t>
         </is>
       </c>
-      <c r="Q12" s="3">
+      <c r="V12" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="R12" s="3">
+      <c r="W12" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=KKup0OgAAAAJ", "Scholar (KKup0OgAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S12" s="3">
+      <c r="X12" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5049,28 +5598,33 @@
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N13" s="3">
+      <c r="S13" s="3">
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="O13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="3">
+      <c r="T13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xzhe1", "https://search.asu.edu/profile/xzhe1")</f>
         <v/>
       </c>
-      <c r="R13" s="3">
+      <c r="W13" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Zhe%20Xu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S13" s="3">
+      <c r="X13" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5123,19 +5677,24 @@
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
-      <c r="O14" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="3">
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jkim520", "https://search.asu.edu/profile/jkim520")</f>
         <v/>
       </c>
-      <c r="R14" s="3">
+      <c r="W14" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Jeonglae%20Kim%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S14" s="3">
+      <c r="X14" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5199,23 +5758,28 @@
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="3">
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="3">
         <f>HYPERLINK("http://control.asu.edu/", "http://control.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="3">
+      <c r="T15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mpeet", "https://search.asu.edu/profile/mpeet")</f>
         <v/>
       </c>
-      <c r="R15" s="3">
+      <c r="W15" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S15" s="3">
+      <c r="X15" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5275,27 +5839,32 @@
       </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="3">
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="3">
         <f>HYPERLINK("http://wang.faculty.asu.edu/", "http://wang.faculty.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
+      <c r="T16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
         <is>
           <t>LaUdx9gAAAAJ</t>
         </is>
       </c>
-      <c r="Q16" s="3">
+      <c r="V16" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rywang", "https://search.asu.edu/profile/rywang")</f>
         <v/>
       </c>
-      <c r="R16" s="3">
+      <c r="W16" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=LaUdx9gAAAAJ", "Scholar (LaUdx9gAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S16" s="3">
+      <c r="X16" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5355,23 +5924,36 @@
       </c>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="3">
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 465 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
+      <c r="S17" s="3">
         <f>HYPERLINK("http://RESEARCHGATE.net/profile/Ryan_Milcarek", "http://RESEARCHGATE.net/profile/Ryan_Milcarek")</f>
         <v/>
       </c>
-      <c r="O17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="3">
+      <c r="T17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>m-Pb6g2pm2UC</t>
+        </is>
+      </c>
+      <c r="V17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="R17" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
-        <v/>
-      </c>
-      <c r="S17" s="3">
+      <c r="W17" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
+        <v/>
+      </c>
+      <c r="X17" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5422,25 +6004,30 @@
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
         <is>
           <t>ENGRC 377 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="3">
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/attwl", "https://search.asu.edu/profile/attwl")</f>
         <v/>
       </c>
-      <c r="R18" s="3">
+      <c r="W18" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=T.-W.%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S18" s="3">
+      <c r="X18" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5493,19 +6080,32 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="3">
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>OmBV67MAAAAJ</t>
+        </is>
+      </c>
+      <c r="V19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="R19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
-        <v/>
-      </c>
-      <c r="S19" s="3">
+      <c r="W19" s="3">
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
+        <v/>
+      </c>
+      <c r="X19" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5562,23 +6162,28 @@
       </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
-      <c r="O20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
         <is>
           <t>w3fU9E0AAAAJ</t>
         </is>
       </c>
-      <c r="Q20" s="3">
+      <c r="V20" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/chattopa", "https://search.asu.edu/profile/chattopa")</f>
         <v/>
       </c>
-      <c r="R20" s="3">
+      <c r="W20" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=w3fU9E0AAAAJ", "Scholar (w3fU9E0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S20" s="3">
+      <c r="X20" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5637,29 +6242,34 @@
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
         <is>
           <t>HRx2lJQAAAAJ</t>
         </is>
       </c>
-      <c r="Q21" s="3">
+      <c r="V21" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/adscotti", "https://search.asu.edu/profile/adscotti")</f>
         <v/>
       </c>
-      <c r="R21" s="3">
+      <c r="W21" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=HRx2lJQAAAAJ", "Scholar (HRx2lJQAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S21" s="3">
+      <c r="X21" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5718,32 +6328,45 @@
           <t>3D Energy Lab</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>3D Energy Device Laboratory</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 363 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="N22" s="3">
+      <c r="S22" s="3">
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="O22" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
+      <c r="T22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
         <is>
           <t>fs2d97sAAAAJ</t>
         </is>
       </c>
-      <c r="Q22" s="3">
+      <c r="V22" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/bkwon2", "https://search.asu.edu/profile/bkwon2")</f>
         <v/>
       </c>
-      <c r="R22" s="3">
+      <c r="W22" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=fs2d97sAAAAJ", "Scholar (fs2d97sAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S22" s="3">
+      <c r="X22" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5803,27 +6426,36 @@
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="3">
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S23" s="3">
         <f>HYPERLINK("http://birth.asu.edu", "http://birth.asu.edu")</f>
         <v/>
       </c>
-      <c r="O23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
+      <c r="T23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
         <is>
           <t>00Fepb0AAAAJ</t>
         </is>
       </c>
-      <c r="Q23" s="3">
+      <c r="V23" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hmarvi", "https://search.asu.edu/profile/hmarvi")</f>
         <v/>
       </c>
-      <c r="R23" s="3">
+      <c r="W23" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=00Fepb0AAAAJ", "Scholar (00Fepb0AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S23" s="3">
+      <c r="X23" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5874,28 +6506,33 @@
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N24" s="3">
+      <c r="S24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/hlee", "https://faculty.engineering.asu.edu/hlee")</f>
         <v/>
       </c>
-      <c r="O24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P24" s="2" t="inlineStr"/>
-      <c r="Q24" s="3">
+      <c r="T24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U24" s="2" t="inlineStr"/>
+      <c r="V24" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hlee234", "https://search.asu.edu/profile/hlee234")</f>
         <v/>
       </c>
-      <c r="R24" s="3">
+      <c r="W24" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Hyunglae%20Lee%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S24" s="3">
+      <c r="X24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5959,23 +6596,28 @@
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="3">
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="3">
         <f>HYPERLINK("https://magic.asu.edu/", "https://magic.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="inlineStr"/>
-      <c r="Q25" s="3">
+      <c r="T25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U25" s="2" t="inlineStr"/>
+      <c r="V25" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ljannesa", "https://search.asu.edu/profile/ljannesa")</f>
         <v/>
       </c>
-      <c r="R25" s="3">
+      <c r="W25" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Leila%20Ladani%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S25" s="3">
+      <c r="X25" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6034,25 +6676,30 @@
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
         <is>
           <t>ENGRC 463 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="3">
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U26" s="2" t="inlineStr"/>
+      <c r="V26" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pphelan", "https://search.asu.edu/profile/pphelan")</f>
         <v/>
       </c>
-      <c r="R26" s="3">
+      <c r="W26" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Patrick%20Phelan%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S26" s="3">
+      <c r="X26" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6108,27 +6755,32 @@
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="3">
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="3">
         <f>HYPERLINK("https://isim.asu.edu", "https://isim.asu.edu")</f>
         <v/>
       </c>
-      <c r="O27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
+      <c r="T27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
         <is>
           <t>_6o8MrUAAAAJ</t>
         </is>
       </c>
-      <c r="Q27" s="3">
+      <c r="V27" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="R27" s="3">
+      <c r="W27" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=_6o8MrUAAAAJ", "Scholar (_6o8MrUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S27" s="3">
+      <c r="X27" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6191,29 +6843,30 @@
           <t>Computational Materials Science and Design Lab</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
+      <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
         <is>
           <t>4yYKCpUAAAAJ</t>
         </is>
       </c>
-      <c r="Q28" s="3">
+      <c r="V28" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hzhuang7", "https://search.asu.edu/profile/hzhuang7")</f>
         <v/>
       </c>
-      <c r="R28" s="3">
+      <c r="W28" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=4yYKCpUAAAAJ", "Scholar (4yYKCpUAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S28" s="3">
+      <c r="X28" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6264,28 +6917,33 @@
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="N29" s="3">
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>Log in to www_public</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr"/>
+      <c r="S29" s="3">
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="O29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P29" s="2" t="inlineStr"/>
-      <c r="Q29" s="3">
+      <c r="T29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U29" s="2" t="inlineStr"/>
+      <c r="V29" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/hhuang38", "https://search.asu.edu/profile/hhuang38")</f>
         <v/>
       </c>
-      <c r="R29" s="3">
+      <c r="W29" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Huei-Ping%20Huang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S29" s="3">
+      <c r="X29" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6348,32 +7006,41 @@
           <t>Nanomechanics Laboratory</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr"/>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>Nanostructured Materials</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
         <is>
           <t>ENGRC 355 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N30" s="3">
+      <c r="S30" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/jagan/", "http://faculty.engineering.asu.edu/jagan/")</f>
         <v/>
       </c>
-      <c r="O30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
+      <c r="T30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
         <is>
           <t>ClqRIhIAAAAJ</t>
         </is>
       </c>
-      <c r="Q30" s="3">
+      <c r="V30" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jrajago1", "https://search.asu.edu/profile/jrajago1")</f>
         <v/>
       </c>
-      <c r="R30" s="3">
+      <c r="W30" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=ClqRIhIAAAAJ", "Scholar (ClqRIhIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S30" s="3">
+      <c r="X30" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6429,27 +7096,36 @@
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="3">
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 309 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
+      <c r="S31" s="3">
         <f>HYPERLINK("http://faculty.engineering.asu.edu/konrad/", "http://faculty.engineering.asu.edu/konrad/")</f>
         <v/>
       </c>
-      <c r="O31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
+      <c r="T31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U31" s="2" t="inlineStr">
         <is>
           <t>SWeAf4UAAAAJ</t>
         </is>
       </c>
-      <c r="Q31" s="3">
+      <c r="V31" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/krykacze", "https://search.asu.edu/profile/krykacze")</f>
         <v/>
       </c>
-      <c r="R31" s="3">
+      <c r="W31" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SWeAf4UAAAAJ", "Scholar (SWeAf4UAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S31" s="3">
+      <c r="X31" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6506,23 +7182,32 @@
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
         <is>
           <t>9LWNC50AAAAJ</t>
         </is>
       </c>
-      <c r="Q32" s="3">
+      <c r="V32" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/mingleiq", "https://search.asu.edu/profile/mingleiq")</f>
         <v/>
       </c>
-      <c r="R32" s="3">
+      <c r="W32" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=9LWNC50AAAAJ", "Scholar (9LWNC50AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S32" s="3">
+      <c r="X32" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6581,28 +7266,33 @@
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N33" s="3">
+      <c r="S33" s="3">
         <f>HYPERLINK("https://mmmplab.engineering.asu.edu/", "https://mmmplab.engineering.asu.edu/")</f>
         <v/>
       </c>
-      <c r="O33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="3">
+      <c r="T33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U33" s="2" t="inlineStr"/>
+      <c r="V33" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/qnian", "https://search.asu.edu/profile/qnian")</f>
         <v/>
       </c>
-      <c r="R33" s="3">
+      <c r="W33" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Qiong%20Nian%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S33" s="3">
+      <c r="X33" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6657,28 +7347,33 @@
           <t>Wind Energy and Atmospheric Boundary Layer Lab</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr">
         <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N34" s="3">
+      <c r="S34" s="3">
         <f>HYPERLINK("https://windlab.engineering.asu.edu/ronald-calhoun/", "https://windlab.engineering.asu.edu/ronald-calhoun/")</f>
         <v/>
       </c>
-      <c r="O34" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="3">
+      <c r="T34" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U34" s="2" t="inlineStr"/>
+      <c r="V34" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcalhou", "https://search.asu.edu/profile/rcalhou")</f>
         <v/>
       </c>
-      <c r="R34" s="3">
+      <c r="W34" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ronald%20Calhoun%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S34" s="3">
+      <c r="X34" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6738,27 +7433,48 @@
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="3">
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/asu-iris</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="inlineStr">
+        <is>
+          <t>Recent Updates</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S35" s="3">
         <f>HYPERLINK("https://irislab.tech/", "https://irislab.tech/")</f>
         <v/>
       </c>
-      <c r="O35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P35" s="2" t="inlineStr">
+      <c r="T35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U35" s="2" t="inlineStr">
         <is>
           <t>SoEC4h4AAAAJ</t>
         </is>
       </c>
-      <c r="Q35" s="3">
+      <c r="V35" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wjin34", "https://search.asu.edu/profile/wjin34")</f>
         <v/>
       </c>
-      <c r="R35" s="3">
+      <c r="W35" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=SoEC4h4AAAAJ", "Scholar (SoEC4h4AAAAJ)")</f>
         <v/>
       </c>
-      <c r="S35" s="3">
+      <c r="X35" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6817,25 +7533,30 @@
           <t>Prognostics and Health Management (PHM) Lab</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="R36" s="2" t="inlineStr">
         <is>
           <t>ENGRC 409 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P36" s="2" t="inlineStr"/>
-      <c r="Q36" s="3">
+      <c r="S36" s="2" t="inlineStr"/>
+      <c r="T36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U36" s="2" t="inlineStr"/>
+      <c r="V36" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yliu35", "https://search.asu.edu/profile/yliu35")</f>
         <v/>
       </c>
-      <c r="R36" s="3">
+      <c r="W36" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yongming%20Liu%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S36" s="3">
+      <c r="X36" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6899,27 +7620,40 @@
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="3">
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>NSF</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="R37" s="2" t="inlineStr"/>
+      <c r="S37" s="3">
         <f>HYPERLINK("https://www.cindyxjli.com/", "https://www.cindyxjli.com/")</f>
         <v/>
       </c>
-      <c r="O37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P37" s="2" t="inlineStr">
+      <c r="T37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U37" s="2" t="inlineStr">
         <is>
           <t>tGQzHJIAAAAJ</t>
         </is>
       </c>
-      <c r="Q37" s="3">
+      <c r="V37" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/xiangji5", "https://search.asu.edu/profile/xiangji5")</f>
         <v/>
       </c>
-      <c r="R37" s="3">
+      <c r="W37" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=tGQzHJIAAAAJ", "Scholar (tGQzHJIAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S37" s="3">
+      <c r="X37" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6974,25 +7708,30 @@
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr">
         <is>
           <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr"/>
-      <c r="O38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P38" s="2" t="inlineStr"/>
-      <c r="Q38" s="3">
+      <c r="S38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U38" s="2" t="inlineStr"/>
+      <c r="V38" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jimbo", "https://search.asu.edu/profile/jimbo")</f>
         <v/>
       </c>
-      <c r="R38" s="3">
+      <c r="W38" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=James%20Middleton%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S38" s="3">
+      <c r="X38" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7043,25 +7782,30 @@
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N39" s="2" t="inlineStr"/>
-      <c r="O39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P39" s="2" t="inlineStr"/>
-      <c r="Q39" s="3">
+      <c r="S39" s="2" t="inlineStr"/>
+      <c r="T39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U39" s="2" t="inlineStr"/>
+      <c r="V39" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/linli25", "https://search.asu.edu/profile/linli25")</f>
         <v/>
       </c>
-      <c r="R39" s="3">
+      <c r="W39" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Lin%20Li%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S39" s="3">
+      <c r="X39" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7112,25 +7856,30 @@
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="R40" s="2" t="inlineStr">
         <is>
           <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr"/>
-      <c r="O40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="3">
+      <c r="S40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U40" s="2" t="inlineStr"/>
+      <c r="V40" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/marc03", "https://search.asu.edu/profile/marc03")</f>
         <v/>
       </c>
-      <c r="R40" s="3">
+      <c r="W40" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Marc%20Mignolet%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S40" s="3">
+      <c r="X40" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7182,23 +7931,32 @@
       </c>
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="3">
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 352 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/pperalta/", "https://faculty.engineering.asu.edu/pperalta/")</f>
         <v/>
       </c>
-      <c r="O41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P41" s="2" t="inlineStr"/>
-      <c r="Q41" s="3">
+      <c r="T41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/pperalta", "https://search.asu.edu/profile/pperalta")</f>
         <v/>
       </c>
-      <c r="R41" s="3">
+      <c r="W41" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Pedro%20Peralta%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S41" s="3">
+      <c r="X41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7259,30 +8017,47 @@
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr">
         <is>
+          <t>Welcome and we are looking forward to working with Dr</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>NSF, ONR</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>Highlighted as a cover in Small</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="N42" s="3">
+      <c r="S42" s="3">
         <f>HYPERLINK("https://wonmokang3.wixsite.com/website", "https://wonmokang3.wixsite.com/website")</f>
         <v/>
       </c>
-      <c r="O42" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
+      <c r="T42" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
         <is>
           <t>bHyyOTAAAAAJ</t>
         </is>
       </c>
-      <c r="Q42" s="3">
+      <c r="V42" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/wkang16", "https://search.asu.edu/profile/wkang16")</f>
         <v/>
       </c>
-      <c r="R42" s="3">
+      <c r="W42" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=bHyyOTAAAAAJ", "Scholar (bHyyOTAAAAAJ)")</f>
         <v/>
       </c>
-      <c r="S42" s="3">
+      <c r="X42" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7335,19 +8110,28 @@
       <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr"/>
-      <c r="O43" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="O43" s="2" t="inlineStr"/>
       <c r="P43" s="2" t="inlineStr"/>
-      <c r="Q43" s="3">
+      <c r="Q43" s="2" t="inlineStr"/>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>GWC 464 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="S43" s="2" t="inlineStr"/>
+      <c r="T43" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U43" s="2" t="inlineStr"/>
+      <c r="V43" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/yren32", "https://search.asu.edu/profile/yren32")</f>
         <v/>
       </c>
-      <c r="R43" s="3">
+      <c r="W43" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Yi%20Ren%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S43" s="3">
+      <c r="X43" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7388,19 +8172,24 @@
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="2" t="inlineStr"/>
-      <c r="O44" s="2" t="b">
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr"/>
+      <c r="Q44" s="2" t="inlineStr"/>
+      <c r="R44" s="2" t="inlineStr"/>
+      <c r="S44" s="2" t="inlineStr"/>
+      <c r="T44" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="P44" s="2" t="inlineStr"/>
-      <c r="Q44" s="3">
+      <c r="U44" s="2" t="inlineStr"/>
+      <c r="V44" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/dspeaks2", "https://search.asu.edu/profile/dspeaks2")</f>
         <v/>
       </c>
-      <c r="R44" s="3">
+      <c r="W44" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Derrick%20Speaks%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S44" s="3">
+      <c r="X44" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7443,25 +8232,26 @@
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr"/>
-      <c r="M45" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Otherus</t>
-        </is>
-      </c>
+      <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr"/>
-      <c r="O45" s="2" t="b">
+      <c r="O45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr"/>
+      <c r="Q45" s="2" t="inlineStr"/>
+      <c r="R45" s="2" t="inlineStr"/>
+      <c r="S45" s="2" t="inlineStr"/>
+      <c r="T45" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="P45" s="2" t="inlineStr"/>
-      <c r="Q45" s="3">
+      <c r="U45" s="2" t="inlineStr"/>
+      <c r="V45" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/ejande22", "https://search.asu.edu/profile/ejande22")</f>
         <v/>
       </c>
-      <c r="R45" s="3">
+      <c r="W45" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Erik%20Andersen%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S45" s="3">
+      <c r="X45" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7502,19 +8292,28 @@
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
-      <c r="O46" s="2" t="b">
+      <c r="O46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr"/>
+      <c r="Q46" s="2" t="inlineStr"/>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="inlineStr"/>
+      <c r="T46" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="P46" s="2" t="inlineStr"/>
-      <c r="Q46" s="3">
+      <c r="U46" s="2" t="inlineStr"/>
+      <c r="V46" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/iychang", "https://search.asu.edu/profile/iychang")</f>
         <v/>
       </c>
-      <c r="R46" s="3">
+      <c r="W46" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ivy%20Chang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S46" s="3">
+      <c r="X46" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7555,19 +8354,24 @@
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr"/>
-      <c r="O47" s="2" t="b">
+      <c r="O47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr"/>
+      <c r="Q47" s="2" t="inlineStr"/>
+      <c r="R47" s="2" t="inlineStr"/>
+      <c r="S47" s="2" t="inlineStr"/>
+      <c r="T47" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="P47" s="2" t="inlineStr"/>
-      <c r="Q47" s="3">
+      <c r="U47" s="2" t="inlineStr"/>
+      <c r="V47" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/jdwilbu1", "https://search.asu.edu/profile/jdwilbu1")</f>
         <v/>
       </c>
-      <c r="R47" s="3">
+      <c r="W47" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Joshua%20Wilbur%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S47" s="3">
+      <c r="X47" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7608,19 +8412,24 @@
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr"/>
       <c r="N48" s="2" t="inlineStr"/>
-      <c r="O48" s="2" t="b">
+      <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr"/>
+      <c r="Q48" s="2" t="inlineStr"/>
+      <c r="R48" s="2" t="inlineStr"/>
+      <c r="S48" s="2" t="inlineStr"/>
+      <c r="T48" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="P48" s="2" t="inlineStr"/>
-      <c r="Q48" s="3">
+      <c r="U48" s="2" t="inlineStr"/>
+      <c r="V48" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rcruzloz", "https://search.asu.edu/profile/rcruzloz")</f>
         <v/>
       </c>
-      <c r="R48" s="3">
+      <c r="W48" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ricardo%20Cruz%20Lozano%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S48" s="3">
+      <c r="X48" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7659,25 +8468,26 @@
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
-      <c r="M49" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr"/>
-      <c r="O49" s="2" t="b">
+      <c r="O49" s="2" t="inlineStr"/>
+      <c r="P49" s="2" t="inlineStr"/>
+      <c r="Q49" s="2" t="inlineStr"/>
+      <c r="R49" s="2" t="inlineStr"/>
+      <c r="S49" s="2" t="inlineStr"/>
+      <c r="T49" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="P49" s="2" t="inlineStr"/>
-      <c r="Q49" s="3">
+      <c r="U49" s="2" t="inlineStr"/>
+      <c r="V49" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/skosara2", "https://search.asu.edu/profile/skosara2")</f>
         <v/>
       </c>
-      <c r="R49" s="3">
+      <c r="W49" s="3">
         <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Srinivas%20Chakravarthi%20Kosaraju%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
-      <c r="S49" s="3">
+      <c r="X49" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7685,223 +8495,223 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W8" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W9" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W15" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V16" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W16" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V17" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W17" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V18" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W18" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V19" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W19" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V20" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W20" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V21" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W21" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V22" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W22" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V23" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W23" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V24" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W24" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V25" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W25" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V26" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W26" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V27" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W27" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V28" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W28" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V29" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W29" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V30" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W30" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V31" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W31" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R32" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V32" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W32" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X32" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N33" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R33" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V33" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W33" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId149"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N34" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R34" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V34" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W34" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X34" r:id="rId154"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N35" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R35" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V35" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W35" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId159"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R36" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V36" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W36" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X36" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N37" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R37" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V37" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W37" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R38" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V38" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W38" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X38" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R39" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V39" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W39" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R40" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V40" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W40" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N41" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R41" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V41" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W41" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R42" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V42" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W42" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X42" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R43" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V43" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W43" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X43" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R44" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S44" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V44" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W44" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X44" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R45" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V45" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W45" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X45" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R46" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V46" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W46" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X46" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R47" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V47" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W47" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X47" r:id="rId210"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R48" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V48" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W48" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X48" r:id="rId214"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R49" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V49" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W49" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X49" r:id="rId218"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor asu_profs.py with fully dynamic column configuration and column name-based referencing
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -470,8 +470,8 @@
     <col width="49" customWidth="1" min="10" max="10"/>
     <col width="53" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="65" customWidth="1" min="13" max="13"/>
-    <col width="61" customWidth="1" min="14" max="14"/>
+    <col width="49" customWidth="1" min="13" max="13"/>
+    <col width="56" customWidth="1" min="14" max="14"/>
     <col width="65" customWidth="1" min="15" max="15"/>
     <col width="65" customWidth="1" min="16" max="16"/>
     <col width="65" customWidth="1" min="17" max="17"/>
@@ -479,7 +479,7 @@
     <col width="32" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="49" customWidth="1" min="21" max="21"/>
-    <col width="46" customWidth="1" min="22" max="22"/>
+    <col width="54" customWidth="1" min="22" max="22"/>
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="49" customWidth="1" min="24" max="24"/>
   </cols>
@@ -659,10 +659,9 @@
           <t>AFOSR</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master</t>
-        </is>
+      <c r="M2" s="3">
+        <f>HYPERLINK("https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz", "https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master")</f>
+        <v/>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -1055,11 +1054,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 361 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V6" s="2" t="inlineStr"/>
       <c r="W6" s="2" t="b">
         <v>1</v>
       </c>
@@ -1335,7 +1330,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
-      <c r="V9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>ERC 485 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="W9" s="2" t="b">
         <v>1</v>
       </c>
@@ -1591,11 +1590,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V12" s="2" t="inlineStr"/>
       <c r="W12" s="2" t="b">
         <v>1</v>
       </c>
@@ -1890,11 +1885,7 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>Thermal Energy &amp; Nanomaterials Lab</t>
-        </is>
-      </c>
+      <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
           <t>My research group is an interdisciplinary nanoengineering team that focuses on manipulating material properties for thermal energy applications. Some of our focus areas are thermoelectric power generation, thermal storage media, heat transfer, and phonon optics. To achieve our objectives, we custom-design materials using colloidal nanoparticles, chemical precursors, and nanocomposites.</t>
@@ -2005,23 +1996,15 @@
         </is>
       </c>
       <c r="S17" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
-        <v/>
-      </c>
-      <c r="T17" s="2" t="inlineStr">
-        <is>
-          <t>m-Pb6g2pm2UC</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 465 (Tempe, AZ 85287)</t>
-        </is>
-      </c>
+      <c r="V17" s="2" t="inlineStr"/>
       <c r="W17" s="2" t="b">
         <v>1</v>
       </c>
@@ -2157,23 +2140,15 @@
         </is>
       </c>
       <c r="S19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
-        <v/>
-      </c>
-      <c r="T19" s="2" t="inlineStr">
-        <is>
-          <t>OmBV67MAAAAJ</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="V19" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="V19" s="2" t="inlineStr"/>
       <c r="W19" s="2" t="b">
         <v>1</v>
       </c>
@@ -2493,11 +2468,7 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>Latest News</t>
-        </is>
-      </c>
+      <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
           <t>Bio-inspired robotics Soft robotics Magnetic micro-robotics Mechanics of animal locomotion</t>
@@ -2527,11 +2498,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/hmarvi", "https://search.asu.edu/profile/hmarvi")</f>
         <v/>
       </c>
-      <c r="V23" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="V23" s="2" t="inlineStr"/>
       <c r="W23" s="2" t="b">
         <v>1</v>
       </c>
@@ -2661,17 +2628,9 @@
         <v/>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>NSF</t>
-        </is>
-      </c>
+      <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>Advancing manufacturing innovation</t>
-        </is>
-      </c>
+      <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
           <t>Manufacturing process simulation and modeling and experiments Additive manufacturing Micro/nano manufacturing Microelectronic packaging Application of AI in manufacturing Mechanic of metallic materials Materials characterization Fatigue and damage modeling and simulation</t>
@@ -2701,7 +2660,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/ljannesa", "https://search.asu.edu/profile/ljannesa")</f>
         <v/>
       </c>
-      <c r="V25" s="2" t="inlineStr"/>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>ISTB4, ROOM 379 781 S Terrace Rd (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="W25" s="2" t="b">
         <v>1</v>
       </c>
@@ -2864,7 +2827,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="V27" s="2" t="inlineStr"/>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 379 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="W27" s="2" t="b">
         <v>1</v>
       </c>
@@ -3344,17 +3311,9 @@
         <v/>
       </c>
       <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>NSF</t>
-        </is>
-      </c>
+      <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>Multi-scale Manufacturing Material Processing Lab (MMMPL)</t>
-        </is>
-      </c>
+      <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
           <t>Nanomanufacturing, additive manufacturing, laser-based material processing, laser matter interaction and physics simulation; inkjet printing of functional materials; and 2D materials fabrication for energy storage and bio-sensors.</t>
@@ -3441,17 +3400,9 @@
         <v/>
       </c>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>DOE, NASA</t>
-        </is>
-      </c>
+      <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>Environmental Remote SensingGroup</t>
-        </is>
-      </c>
+      <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr"/>
       <c r="Q34" s="2" t="inlineStr">
@@ -3535,10 +3486,9 @@
           <t>NSF</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/asu-iris</t>
-        </is>
+      <c r="M35" s="3">
+        <f>HYPERLINK("https://github.com/asu-iris", "https://github.com/asu-iris")</f>
+        <v/>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
@@ -3574,7 +3524,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/wjin34", "https://search.asu.edu/profile/wjin34")</f>
         <v/>
       </c>
-      <c r="V35" s="2" t="inlineStr"/>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="W35" s="2" t="b">
         <v>1</v>
       </c>
@@ -3753,7 +3707,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/xiangji5", "https://search.asu.edu/profile/xiangji5")</f>
         <v/>
       </c>
-      <c r="V37" s="2" t="inlineStr"/>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
+        </is>
+      </c>
       <c r="W37" s="2" t="b">
         <v>1</v>
       </c>
@@ -3827,11 +3785,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/jimbo", "https://search.asu.edu/profile/jimbo")</f>
         <v/>
       </c>
-      <c r="V38" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V38" s="2" t="inlineStr"/>
       <c r="W38" s="2" t="b">
         <v>1</v>
       </c>
@@ -3975,11 +3929,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/marc03", "https://search.asu.edu/profile/marc03")</f>
         <v/>
       </c>
-      <c r="V40" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V40" s="2" t="inlineStr"/>
       <c r="W40" s="2" t="b">
         <v>1</v>
       </c>
@@ -4240,198 +4190,200 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U13" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U16" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U17" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U20" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U21" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U22" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U23" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U24" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U25" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U26" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U29" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U30" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U31" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U32" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X32" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U34" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X34" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U35" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U36" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X36" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U37" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U38" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X38" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U40" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U42" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X42" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U43" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X43" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U13" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U15" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U16" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U17" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U20" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U21" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U22" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U23" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U25" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U26" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U29" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U30" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U31" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U32" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X32" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U34" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X34" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U35" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U36" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X36" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U37" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U38" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X38" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U40" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U42" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X42" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U43" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X43" r:id="rId196"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4458,8 +4410,8 @@
     <col width="49" customWidth="1" min="10" max="10"/>
     <col width="53" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="65" customWidth="1" min="13" max="13"/>
-    <col width="61" customWidth="1" min="14" max="14"/>
+    <col width="49" customWidth="1" min="13" max="13"/>
+    <col width="56" customWidth="1" min="14" max="14"/>
     <col width="65" customWidth="1" min="15" max="15"/>
     <col width="65" customWidth="1" min="16" max="16"/>
     <col width="65" customWidth="1" min="17" max="17"/>
@@ -4467,7 +4419,7 @@
     <col width="32" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="49" customWidth="1" min="21" max="21"/>
-    <col width="46" customWidth="1" min="22" max="22"/>
+    <col width="54" customWidth="1" min="22" max="22"/>
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="49" customWidth="1" min="24" max="24"/>
   </cols>
@@ -4647,10 +4599,9 @@
           <t>AFOSR</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master</t>
-        </is>
+      <c r="M2" s="3">
+        <f>HYPERLINK("https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz", "https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master")</f>
+        <v/>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -5043,11 +4994,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/asuchen", "https://search.asu.edu/profile/asuchen")</f>
         <v/>
       </c>
-      <c r="V6" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 361 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V6" s="2" t="inlineStr"/>
       <c r="W6" s="2" t="b">
         <v>1</v>
       </c>
@@ -5323,7 +5270,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/leixinma", "https://search.asu.edu/profile/leixinma")</f>
         <v/>
       </c>
-      <c r="V9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>ERC 485 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="W9" s="2" t="b">
         <v>1</v>
       </c>
@@ -5579,11 +5530,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/smberma2", "https://search.asu.edu/profile/smberma2")</f>
         <v/>
       </c>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V12" s="2" t="inlineStr"/>
       <c r="W12" s="2" t="b">
         <v>1</v>
       </c>
@@ -5878,11 +5825,7 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>Thermal Energy &amp; Nanomaterials Lab</t>
-        </is>
-      </c>
+      <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
           <t>My research group is an interdisciplinary nanoengineering team that focuses on manipulating material properties for thermal energy applications. Some of our focus areas are thermoelectric power generation, thermal storage media, heat transfer, and phonon optics. To achieve our objectives, we custom-design materials using colloidal nanoparticles, chemical precursors, and nanocomposites.</t>
@@ -5993,23 +5936,15 @@
         </is>
       </c>
       <c r="S17" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=m-Pb6g2pm2UC", "Scholar (m-Pb6g2pm2UC)")</f>
-        <v/>
-      </c>
-      <c r="T17" s="2" t="inlineStr">
-        <is>
-          <t>m-Pb6g2pm2UC</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Ryan%20Milcarek%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/rjmilcar", "https://search.asu.edu/profile/rjmilcar")</f>
         <v/>
       </c>
-      <c r="V17" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 465 (Tempe, AZ 85287)</t>
-        </is>
-      </c>
+      <c r="V17" s="2" t="inlineStr"/>
       <c r="W17" s="2" t="b">
         <v>1</v>
       </c>
@@ -6145,23 +6080,15 @@
         </is>
       </c>
       <c r="S19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
-        <v/>
-      </c>
-      <c r="T19" s="2" t="inlineStr">
-        <is>
-          <t>OmBV67MAAAAJ</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <v/>
+      </c>
+      <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="3">
         <f>HYPERLINK("https://search.asu.edu/profile/tyang123", "https://search.asu.edu/profile/tyang123")</f>
         <v/>
       </c>
-      <c r="V19" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="V19" s="2" t="inlineStr"/>
       <c r="W19" s="2" t="b">
         <v>1</v>
       </c>
@@ -6481,11 +6408,7 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>Latest News</t>
-        </is>
-      </c>
+      <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
           <t>Bio-inspired robotics Soft robotics Magnetic micro-robotics Mechanics of animal locomotion</t>
@@ -6515,11 +6438,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/hmarvi", "https://search.asu.edu/profile/hmarvi")</f>
         <v/>
       </c>
-      <c r="V23" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="V23" s="2" t="inlineStr"/>
       <c r="W23" s="2" t="b">
         <v>1</v>
       </c>
@@ -6649,17 +6568,9 @@
         <v/>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>NSF</t>
-        </is>
-      </c>
+      <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>Advancing manufacturing innovation</t>
-        </is>
-      </c>
+      <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
           <t>Manufacturing process simulation and modeling and experiments Additive manufacturing Micro/nano manufacturing Microelectronic packaging Application of AI in manufacturing Mechanic of metallic materials Materials characterization Fatigue and damage modeling and simulation</t>
@@ -6689,7 +6600,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/ljannesa", "https://search.asu.edu/profile/ljannesa")</f>
         <v/>
       </c>
-      <c r="V25" s="2" t="inlineStr"/>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>ISTB4, ROOM 379 781 S Terrace Rd (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="W25" s="2" t="b">
         <v>1</v>
       </c>
@@ -6852,7 +6767,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/ypeet", "https://search.asu.edu/profile/ypeet")</f>
         <v/>
       </c>
-      <c r="V27" s="2" t="inlineStr"/>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 379 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="W27" s="2" t="b">
         <v>1</v>
       </c>
@@ -7332,17 +7251,9 @@
         <v/>
       </c>
       <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>NSF</t>
-        </is>
-      </c>
+      <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>Multi-scale Manufacturing Material Processing Lab (MMMPL)</t>
-        </is>
-      </c>
+      <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
           <t>Nanomanufacturing, additive manufacturing, laser-based material processing, laser matter interaction and physics simulation; inkjet printing of functional materials; and 2D materials fabrication for energy storage and bio-sensors.</t>
@@ -7429,17 +7340,9 @@
         <v/>
       </c>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>DOE, NASA</t>
-        </is>
-      </c>
+      <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>Environmental Remote SensingGroup</t>
-        </is>
-      </c>
+      <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr"/>
       <c r="Q34" s="2" t="inlineStr">
@@ -7523,10 +7426,9 @@
           <t>NSF</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/asu-iris</t>
-        </is>
+      <c r="M35" s="3">
+        <f>HYPERLINK("https://github.com/asu-iris", "https://github.com/asu-iris")</f>
+        <v/>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
@@ -7562,7 +7464,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/wjin34", "https://search.asu.edu/profile/wjin34")</f>
         <v/>
       </c>
-      <c r="V35" s="2" t="inlineStr"/>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="W35" s="2" t="b">
         <v>1</v>
       </c>
@@ -7741,7 +7647,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/xiangji5", "https://search.asu.edu/profile/xiangji5")</f>
         <v/>
       </c>
-      <c r="V37" s="2" t="inlineStr"/>
+      <c r="V37" s="2" t="inlineStr">
+        <is>
+          <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
+        </is>
+      </c>
       <c r="W37" s="2" t="b">
         <v>1</v>
       </c>
@@ -7815,11 +7725,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/jimbo", "https://search.asu.edu/profile/jimbo")</f>
         <v/>
       </c>
-      <c r="V38" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V38" s="2" t="inlineStr"/>
       <c r="W38" s="2" t="b">
         <v>1</v>
       </c>
@@ -7963,11 +7869,7 @@
         <f>HYPERLINK("https://search.asu.edu/profile/marc03", "https://search.asu.edu/profile/marc03")</f>
         <v/>
       </c>
-      <c r="V40" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="V40" s="2" t="inlineStr"/>
       <c r="W40" s="2" t="b">
         <v>1</v>
       </c>
@@ -8273,7 +8175,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/dspeaks2", "https://search.asu.edu/profile/dspeaks2")</f>
         <v/>
       </c>
-      <c r="V44" s="2" t="inlineStr"/>
+      <c r="V44" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="W44" s="2" t="b">
         <v>0</v>
       </c>
@@ -8513,7 +8419,11 @@
         <f>HYPERLINK("https://search.asu.edu/profile/rcruzloz", "https://search.asu.edu/profile/rcruzloz")</f>
         <v/>
       </c>
-      <c r="V48" s="2" t="inlineStr"/>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="W48" s="2" t="b">
         <v>0</v>
       </c>
@@ -8588,222 +8498,224 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U13" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U16" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U17" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U20" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U21" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U22" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U23" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U24" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U25" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U26" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U29" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U30" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U31" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U32" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X32" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U34" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X34" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U35" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U36" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X36" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U37" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U38" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X38" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U40" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U42" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X42" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U43" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X43" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S44" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U44" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X44" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U45" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X45" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U46" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X46" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U47" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X47" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U48" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X48" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X49" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U13" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U15" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U16" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U17" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U20" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U21" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U22" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U23" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U25" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U26" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U29" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U30" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U31" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U32" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X32" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X33" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U34" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X34" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U35" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U36" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X36" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U37" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X37" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U38" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X38" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X39" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S40" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U40" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X40" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S41" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X41" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U42" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X42" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U43" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X43" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S44" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U44" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X44" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U45" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X45" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S46" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U46" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X46" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U47" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X47" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U48" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X48" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X49" r:id="rId220"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scrape publications, openings, and outreach instructions directly from lab websites
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -483,7 +483,7 @@
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="49" customWidth="1" min="24" max="24"/>
     <col width="56" customWidth="1" min="25" max="25"/>
-    <col width="46" customWidth="1" min="26" max="26"/>
+    <col width="54" customWidth="1" min="26" max="26"/>
     <col width="18" customWidth="1" min="27" max="27"/>
     <col width="49" customWidth="1" min="28" max="28"/>
   </cols>
@@ -672,8 +672,16 @@
           <t>aerospace, cfd, computational fluid dynamics, dns, fluid dynamics, fluid-structure interaction, multiphase flow, turbulent</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Refereed Journal Papers M. H. Kasbaoui and M. Herrmann, A high-fidelity methodology for particle-resolved direct numerical simu...</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 574: Multiphase Flow | MAE 501: Linear Algebra in Engineering</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -717,7 +725,11 @@
           <t>School for Engineering of Matter, Transport &amp; Energy</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA2" s="2" t="b">
         <v>1</v>
       </c>
@@ -768,7 +780,11 @@
           <t>aerospace, guidance, heat transfer, materials, metamaterials, radiation, thermal</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>One PhD position available for Fall 2024 on AFM based near-field thermal measurement! ($32k/year stipend + tuition + benefit)</t>
+        </is>
+      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>MAE 584: Internship | MAE 593: Applied Project | MAE 241: Intro to Thermodynamics</t>
@@ -779,7 +795,11 @@
           <t>2017         AFOSR Young Investigator (YIP) Award,  ASU | 2016         JQSRT/Elsevier Viskanta Young Scientist Award,  ASU</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Please send your CV to Prof</t>
+        </is>
+      </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
@@ -884,7 +904,11 @@
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>If you're interested in joining our group, please email</t>
+        </is>
+      </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Development of computational mechanics: finite element methods, molecular dynamics, multiscale methods, failure analysis, and material design.</t>
@@ -910,7 +934,11 @@
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="U4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>What we're looking for:</t>
+        </is>
+      </c>
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr"/>
@@ -978,10 +1006,22 @@
           <t>aerospace, autonomous, materials, robot, robotics, smart materials</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026 Versatile artificial muscles by decoupling anisotropy Eric Weissman, Rohan Khatavkar, and Jiefeng Sun Proceedings of the N...</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>MAE 547: Modeling and Control of Robots | MAE 593: Applied Project | MAE 499: Individualized Instruction</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Additionally, they should send an email titled “Prospective Ph</t>
+        </is>
+      </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Hire students to conduct research https://sunroboticslab.github.io</t>
@@ -1024,7 +1064,11 @@
           <t>Mission and Core Values</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA5" s="2" t="b">
         <v>1</v>
       </c>
@@ -1247,7 +1291,11 @@
           <t>aerospace, autonomous, control theory, motion planning, robot, robotics</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Search this site Embedded Files Skip to main content Skip to navigation Kunal Garg Home People Teaching Research Publications K...</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>MAE 417: System Dynamics and Control II | MAE 593: Applied Project | MAE 598: Special Topics</t>
@@ -1360,10 +1408,22 @@
           <t>aerodynamics, aerospace, fluid-structure interaction, fluids, materials, robot</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Search this site Embedded Files Skip to main content Skip to navigation OASIS group at ASU Home Research People Publications Ne...</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>MAE 499: Individualized Instruction | MAE 202: Mech.Particles/Rigid Bodies II | MAE 318: System Dynamics and Control I</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Potential candidates with strong backgrounds in fluid-structure interaction, soft robotics , machine learning can send their CV to leixinma@asu</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
           <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
@@ -1406,7 +1466,11 @@
           <t>Ocean and Soft Intelligent Structure Interaction Lab</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>ERC 485 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="AA9" s="2" t="b">
         <v>1</v>
       </c>
@@ -1653,7 +1717,11 @@
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>MAE 318: System Dynamics and Control I | MAE 598: Special Topics | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr">
@@ -1690,7 +1758,11 @@
       <c r="W12" s="2" t="inlineStr"/>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr"/>
-      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA12" s="2" t="b">
         <v>1</v>
       </c>
@@ -1778,7 +1850,11 @@
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="U13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V13" s="2" t="inlineStr"/>
       <c r="W13" s="2" t="inlineStr"/>
       <c r="X13" s="2" t="inlineStr"/>
@@ -1839,7 +1915,11 @@
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 593: Applied Project | MAE 598: Special Topics</t>
+        </is>
+      </c>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr"/>
@@ -1861,7 +1941,11 @@
       <c r="W14" s="2" t="inlineStr"/>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="inlineStr"/>
-      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA14" s="2" t="b">
         <v>1</v>
       </c>
@@ -2006,7 +2090,11 @@
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>MAE 241: Intro to Thermodynamics | MAE 593: Applied Project | MAE 588: Nanoscale Heat Transfer</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
@@ -2039,7 +2127,11 @@
       <c r="W16" s="2" t="inlineStr"/>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="2" t="inlineStr"/>
-      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 307 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA16" s="2" t="b">
         <v>1</v>
       </c>
@@ -2255,7 +2347,7 @@
         <v/>
       </c>
       <c r="D19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2268,11 +2360,7 @@
           <t>Aerospace &amp; Mechanical Engineering</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>OmBV67MAAAAJ</t>
-        </is>
-      </c>
+      <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="3">
         <f>HYPERLINK("mailto:Tianyu.Yang@asu.edu", "Tianyu.Yang@asu.edu")</f>
         <v/>
@@ -2286,11 +2374,7 @@
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>MAE 241: Intro to Thermodynamics</t>
-        </is>
-      </c>
+      <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
@@ -2312,11 +2396,7 @@
       <c r="W19" s="2" t="inlineStr"/>
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr"/>
-      <c r="Z19" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="Z19" s="2" t="inlineStr"/>
       <c r="AA19" s="2" t="b">
         <v>1</v>
       </c>
@@ -2372,7 +2452,11 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>MAE 557: Mechanics Composite Materials | MAE 494: Special Topics | MAE 521: Structural Optimization</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
@@ -2398,7 +2482,11 @@
       <c r="W20" s="2" t="inlineStr"/>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
-      <c r="Z20" s="2" t="inlineStr"/>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA20" s="2" t="b">
         <v>1</v>
       </c>
@@ -2547,7 +2635,11 @@
           <t>aerospace, energy systems, heat transfer</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Journal Papers 62. N. Ohashi, J. Deng, L.K. Hwang, P.K. Kang, and B. Kwon, “Physics-Informed Machine Learning for Reconstructin...</t>
+        </is>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>MAE 593: Applied Project | MAE 241: Intro to Thermodynamics | MAE 598: Special Topics</t>
@@ -2580,7 +2672,11 @@
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="U22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr">
         <is>
@@ -2652,8 +2748,16 @@
           <t>aerospace, robot, robotics</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Shape-programmable magnetic soft matter,</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>MAE 417: System Dynamics and Control II | MAE 598: Special Topics | MAE 547: Modeling and Control of Robots</t>
+        </is>
+      </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
           <t>KEEN Professorship, The Kern Family Foundation, 2017. | Peebles Award for Graduate Student Research in Adhesion Science, Adhesion Society, 2015.</t>
@@ -2690,7 +2794,11 @@
       <c r="W23" s="2" t="inlineStr"/>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="inlineStr"/>
-      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA23" s="2" t="b">
         <v>1</v>
       </c>
@@ -2827,7 +2935,11 @@
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>MAE 598: Special Topics | MAE 494: Special Topics | MAE 201: Mech. Particles/Rigid Bodies I</t>
+        </is>
+      </c>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
@@ -2864,7 +2976,11 @@
       <c r="W25" s="2" t="inlineStr"/>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="inlineStr"/>
-      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>ISTB4, ROOM 379 781 S Terrace Rd (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="AA25" s="2" t="b">
         <v>1</v>
       </c>
@@ -3014,7 +3130,11 @@
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>MAE 215: Intro to Programming in MATLAB | MAE 591: Seminar | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="inlineStr"/>
@@ -3043,7 +3163,11 @@
       <c r="W27" s="2" t="inlineStr"/>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="inlineStr"/>
-      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 379 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA27" s="2" t="b">
         <v>1</v>
       </c>
@@ -3099,7 +3223,11 @@
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>MAE 551: Appl Machine Learn Mech Engr | MAE 451: Appl Machine Learn Mech Engr | MAE 202: Mech.Particles/Rigid Bodies II</t>
+        </is>
+      </c>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
@@ -3133,7 +3261,11 @@
       <c r="W28" s="2" t="inlineStr"/>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
-      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA28" s="2" t="b">
         <v>1</v>
       </c>
@@ -3185,7 +3317,11 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>MAE 502: Partial Diff Equations Engr | MAE 460: Applied Comput Fluid Dynamics | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
@@ -3205,7 +3341,11 @@
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="U29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V29" s="2" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
@@ -3214,7 +3354,11 @@
           <t>Log in to www_public</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA29" s="2" t="b">
         <v>1</v>
       </c>
@@ -3411,11 +3555,7 @@
       <c r="V31" s="2" t="inlineStr"/>
       <c r="W31" s="2" t="inlineStr"/>
       <c r="X31" s="2" t="inlineStr"/>
-      <c r="Y31" s="2" t="inlineStr">
-        <is>
-          <t>Rykaczewski Lab</t>
-        </is>
-      </c>
+      <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr">
         <is>
           <t>ENGRC 309 (Tempe, AZ 85287)</t>
@@ -3747,10 +3887,22 @@
           <t>robot, robotics</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Below are selected papers that represent our main research threads. Please visit Publications for the full list. Contact-rich i...</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>MAE 301: Applied Experimental Statistic | MAE 593: Applied Project | MAE 547: Modeling and Control of Robots</t>
+        </is>
+      </c>
       <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>If you are interested, please email Dr</t>
+        </is>
+      </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
           <t>https://irislab.tech/</t>
@@ -3776,7 +3928,11 @@
         <f>HYPERLINK("https://irislab.tech/", "https://irislab.tech/")</f>
         <v/>
       </c>
-      <c r="U35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>Looking for ASU Undergraduate and Master Students</t>
+        </is>
+      </c>
       <c r="V35" s="2" t="inlineStr"/>
       <c r="W35" s="2" t="inlineStr">
         <is>
@@ -3792,7 +3948,11 @@
           <t>Recent Updates</t>
         </is>
       </c>
-      <c r="Z35" s="2" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA35" s="2" t="b">
         <v>1</v>
       </c>
@@ -3937,12 +4097,12 @@
           <t>materials</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>MAE 301: Applied Experimental Statistic | MAE 593: Applied Project | MAE 494: Special Topics</t>
-        </is>
-      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Dylan Joralmon~, Soham Khairnar, Xiangjia Li*, "Rapid Fabrication of Multi-Metal 3D Objects with Adjustable Gradients by Contin...</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
           <t>2026 The J. Orin Edson Entrepreneurship &amp; Innovation Seed Funding Award ASU 2025 1st place Skysong Startup Competition C</t>
@@ -3978,7 +4138,11 @@
         <f>HYPERLINK("https://www.cindyxjli.com/", "https://www.cindyxjli.com/")</f>
         <v/>
       </c>
-      <c r="U37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V37" s="2" t="inlineStr"/>
       <c r="W37" s="2" t="inlineStr">
         <is>
@@ -3991,11 +4155,7 @@
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr">
-        <is>
-          <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
-        </is>
-      </c>
+      <c r="Z37" s="2" t="inlineStr"/>
       <c r="AA37" s="2" t="b">
         <v>1</v>
       </c>
@@ -4046,16 +4206,8 @@
           <t>aerospace</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>Journal Articles Middleton, J. A. (in press). Archimedes, Euler, &amp; Nursing Cats: Rethinking the Arithmetic Mean. OnCore,</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>MAE 484: Internship | MAE 301: Applied Experimental Statistic | MAE 394: Special Topics</t>
-        </is>
-      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr">
@@ -4081,11 +4233,7 @@
       <c r="W38" s="2" t="inlineStr"/>
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="2" t="inlineStr"/>
-      <c r="Z38" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z38" s="2" t="inlineStr"/>
       <c r="AA38" s="2" t="b">
         <v>1</v>
       </c>
@@ -4219,11 +4367,7 @@
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>MAE 510: Dynamics and Vibrations | MAE 591: Seminar | MAE 394: Special Topics</t>
-        </is>
-      </c>
+      <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
@@ -4245,11 +4389,7 @@
       <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
-      <c r="Z40" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z40" s="2" t="inlineStr"/>
       <c r="AA40" s="2" t="b">
         <v>1</v>
       </c>
@@ -4301,7 +4441,11 @@
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>MAE 213: Mechanics of Materials | MAE 593: Applied Project | MAE 520: Stress Analysis</t>
+        </is>
+      </c>
       <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="2" t="inlineStr"/>
       <c r="O41" s="2" t="inlineStr"/>
@@ -4326,7 +4470,11 @@
       <c r="W41" s="2" t="inlineStr"/>
       <c r="X41" s="2" t="inlineStr"/>
       <c r="Y41" s="2" t="inlineStr"/>
-      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 352 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA41" s="2" t="b">
         <v>1</v>
       </c>
@@ -4381,7 +4529,11 @@
           <t>materials</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>top of page This website was built on Wix. Create yours today. Get Started Bio &amp; Nano Lab Home Dr. Kang Lab Members Publication...</t>
+        </is>
+      </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
           <t>MAE 598: Special Topics | MAE 494: Special Topics | MAE 202: Mech.Particles/Rigid Bodies II</t>
@@ -4491,7 +4643,11 @@
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>MAE 494: Special Topics | MAE 598: Special Topics | MAE 301: Applied Experimental Statistic</t>
+        </is>
+      </c>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr"/>
       <c r="O43" s="2" t="inlineStr"/>
@@ -4513,7 +4669,11 @@
       <c r="W43" s="2" t="inlineStr"/>
       <c r="X43" s="2" t="inlineStr"/>
       <c r="Y43" s="2" t="inlineStr"/>
-      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>GWC 464 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA43" s="2" t="b">
         <v>1</v>
       </c>
@@ -4759,7 +4919,7 @@
     <col width="20" customWidth="1" min="23" max="23"/>
     <col width="49" customWidth="1" min="24" max="24"/>
     <col width="56" customWidth="1" min="25" max="25"/>
-    <col width="46" customWidth="1" min="26" max="26"/>
+    <col width="54" customWidth="1" min="26" max="26"/>
     <col width="18" customWidth="1" min="27" max="27"/>
     <col width="49" customWidth="1" min="28" max="28"/>
   </cols>
@@ -4948,8 +5108,16 @@
           <t>aerospace, cfd, computational fluid dynamics, dns, fluid dynamics, fluid-structure interaction, multiphase flow, turbulent</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Refereed Journal Papers M. H. Kasbaoui and M. Herrmann, A high-fidelity methodology for particle-resolved direct numerical simu...</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 574: Multiphase Flow | MAE 501: Linear Algebra in Engineering</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -4993,7 +5161,11 @@
           <t>School for Engineering of Matter, Transport &amp; Energy</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA2" s="2" t="b">
         <v>1</v>
       </c>
@@ -5044,7 +5216,11 @@
           <t>aerospace, guidance, heat transfer, materials, metamaterials, radiation, thermal</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>One PhD position available for Fall 2024 on AFM based near-field thermal measurement! ($32k/year stipend + tuition + benefit)</t>
+        </is>
+      </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>MAE 584: Internship | MAE 593: Applied Project | MAE 241: Intro to Thermodynamics</t>
@@ -5055,7 +5231,11 @@
           <t>2017         AFOSR Young Investigator (YIP) Award,  ASU | 2016         JQSRT/Elsevier Viskanta Young Scientist Award,  ASU</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Please send your CV to Prof</t>
+        </is>
+      </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Nanoscale heat transfer, metamaterials, plasmonics, and nanophotonics with an emphasis on solar thermal energy harvesting using plasmonic-enhanced light trapping for photovolatics, as well as near-field enhancement and spectral control of radiation for thermophotovoltaic energy conversion. Other research interests involve electronic cooling, MEMS, and bio-sensing.</t>
@@ -5160,7 +5340,11 @@
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>If you're interested in joining our group, please email</t>
+        </is>
+      </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Development of computational mechanics: finite element methods, molecular dynamics, multiscale methods, failure analysis, and material design.</t>
@@ -5186,7 +5370,11 @@
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="U4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>What we're looking for:</t>
+        </is>
+      </c>
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr"/>
@@ -5254,10 +5442,22 @@
           <t>aerospace, autonomous, materials, robot, robotics, smart materials</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026 Versatile artificial muscles by decoupling anisotropy Eric Weissman, Rohan Khatavkar, and Jiefeng Sun Proceedings of the N...</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>MAE 547: Modeling and Control of Robots | MAE 593: Applied Project | MAE 499: Individualized Instruction</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Additionally, they should send an email titled “Prospective Ph</t>
+        </is>
+      </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Hire students to conduct research https://sunroboticslab.github.io</t>
@@ -5300,7 +5500,11 @@
           <t>Mission and Core Values</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA5" s="2" t="b">
         <v>1</v>
       </c>
@@ -5523,7 +5727,11 @@
           <t>aerospace, autonomous, control theory, motion planning, robot, robotics</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Search this site Embedded Files Skip to main content Skip to navigation Kunal Garg Home People Teaching Research Publications K...</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>MAE 417: System Dynamics and Control II | MAE 593: Applied Project | MAE 598: Special Topics</t>
@@ -5636,10 +5844,22 @@
           <t>aerodynamics, aerospace, fluid-structure interaction, fluids, materials, robot</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Search this site Embedded Files Skip to main content Skip to navigation OASIS group at ASU Home Research People Publications Ne...</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>MAE 499: Individualized Instruction | MAE 202: Mech.Particles/Rigid Bodies II | MAE 318: System Dynamics and Control I</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Potential candidates with strong backgrounds in fluid-structure interaction, soft robotics , machine learning can send their CV to leixinma@asu</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
           <t>Aerodynamics, Dynamical Systems, Machine Learning, Mechanics of Composite Materials</t>
@@ -5682,7 +5902,11 @@
           <t>Ocean and Soft Intelligent Structure Interaction Lab</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>ERC 485 (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="AA9" s="2" t="b">
         <v>1</v>
       </c>
@@ -5929,7 +6153,11 @@
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>MAE 318: System Dynamics and Control I | MAE 598: Special Topics | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr">
@@ -5966,7 +6194,11 @@
       <c r="W12" s="2" t="inlineStr"/>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr"/>
-      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA12" s="2" t="b">
         <v>1</v>
       </c>
@@ -6054,7 +6286,11 @@
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="U13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V13" s="2" t="inlineStr"/>
       <c r="W13" s="2" t="inlineStr"/>
       <c r="X13" s="2" t="inlineStr"/>
@@ -6115,7 +6351,11 @@
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 593: Applied Project | MAE 598: Special Topics</t>
+        </is>
+      </c>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr"/>
@@ -6137,7 +6377,11 @@
       <c r="W14" s="2" t="inlineStr"/>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="inlineStr"/>
-      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA14" s="2" t="b">
         <v>1</v>
       </c>
@@ -6282,7 +6526,11 @@
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>MAE 241: Intro to Thermodynamics | MAE 593: Applied Project | MAE 588: Nanoscale Heat Transfer</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
@@ -6315,7 +6563,11 @@
       <c r="W16" s="2" t="inlineStr"/>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="2" t="inlineStr"/>
-      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 307 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA16" s="2" t="b">
         <v>1</v>
       </c>
@@ -6531,7 +6783,7 @@
         <v/>
       </c>
       <c r="D19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
         <v/>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -6544,11 +6796,7 @@
           <t>Aerospace &amp; Mechanical Engineering</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>OmBV67MAAAAJ</t>
-        </is>
-      </c>
+      <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="3">
         <f>HYPERLINK("mailto:Tianyu.Yang@asu.edu", "Tianyu.Yang@asu.edu")</f>
         <v/>
@@ -6562,11 +6810,7 @@
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>MAE 241: Intro to Thermodynamics</t>
-        </is>
-      </c>
+      <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
@@ -6588,11 +6832,7 @@
       <c r="W19" s="2" t="inlineStr"/>
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr"/>
-      <c r="Z19" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="Z19" s="2" t="inlineStr"/>
       <c r="AA19" s="2" t="b">
         <v>1</v>
       </c>
@@ -6648,7 +6888,11 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>MAE 557: Mechanics Composite Materials | MAE 494: Special Topics | MAE 521: Structural Optimization</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
@@ -6674,7 +6918,11 @@
       <c r="W20" s="2" t="inlineStr"/>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
-      <c r="Z20" s="2" t="inlineStr"/>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA20" s="2" t="b">
         <v>1</v>
       </c>
@@ -6823,7 +7071,11 @@
           <t>aerospace, energy systems, heat transfer</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Journal Papers 62. N. Ohashi, J. Deng, L.K. Hwang, P.K. Kang, and B. Kwon, “Physics-Informed Machine Learning for Reconstructin...</t>
+        </is>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>MAE 593: Applied Project | MAE 241: Intro to Thermodynamics | MAE 598: Special Topics</t>
@@ -6856,7 +7108,11 @@
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="U22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr">
         <is>
@@ -6928,8 +7184,16 @@
           <t>aerospace, robot, robotics</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Shape-programmable magnetic soft matter,</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>MAE 417: System Dynamics and Control II | MAE 598: Special Topics | MAE 547: Modeling and Control of Robots</t>
+        </is>
+      </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
           <t>KEEN Professorship, The Kern Family Foundation, 2017. | Peebles Award for Graduate Student Research in Adhesion Science, Adhesion Society, 2015.</t>
@@ -6966,7 +7230,11 @@
       <c r="W23" s="2" t="inlineStr"/>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="inlineStr"/>
-      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA23" s="2" t="b">
         <v>1</v>
       </c>
@@ -7103,7 +7371,11 @@
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>MAE 598: Special Topics | MAE 494: Special Topics | MAE 201: Mech. Particles/Rigid Bodies I</t>
+        </is>
+      </c>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr">
@@ -7140,7 +7412,11 @@
       <c r="W25" s="2" t="inlineStr"/>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="inlineStr"/>
-      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>ISTB4, ROOM 379 781 S Terrace Rd (Tempe, AZ 85287)</t>
+        </is>
+      </c>
       <c r="AA25" s="2" t="b">
         <v>1</v>
       </c>
@@ -7290,7 +7566,11 @@
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>MAE 215: Intro to Programming in MATLAB | MAE 591: Seminar | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="inlineStr"/>
@@ -7319,7 +7599,11 @@
       <c r="W27" s="2" t="inlineStr"/>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="inlineStr"/>
-      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 379 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA27" s="2" t="b">
         <v>1</v>
       </c>
@@ -7375,7 +7659,11 @@
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>MAE 551: Appl Machine Learn Mech Engr | MAE 451: Appl Machine Learn Mech Engr | MAE 202: Mech.Particles/Rigid Bodies II</t>
+        </is>
+      </c>
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr">
@@ -7409,7 +7697,11 @@
       <c r="W28" s="2" t="inlineStr"/>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
-      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA28" s="2" t="b">
         <v>1</v>
       </c>
@@ -7461,7 +7753,11 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>MAE 502: Partial Diff Equations Engr | MAE 460: Applied Comput Fluid Dynamics | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
@@ -7481,7 +7777,11 @@
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="U29" s="2" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V29" s="2" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
@@ -7490,7 +7790,11 @@
           <t>Log in to www_public</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA29" s="2" t="b">
         <v>1</v>
       </c>
@@ -7687,11 +7991,7 @@
       <c r="V31" s="2" t="inlineStr"/>
       <c r="W31" s="2" t="inlineStr"/>
       <c r="X31" s="2" t="inlineStr"/>
-      <c r="Y31" s="2" t="inlineStr">
-        <is>
-          <t>Rykaczewski Lab</t>
-        </is>
-      </c>
+      <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr">
         <is>
           <t>ENGRC 309 (Tempe, AZ 85287)</t>
@@ -8023,10 +8323,22 @@
           <t>robot, robotics</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Below are selected papers that represent our main research threads. Please visit Publications for the full list. Contact-rich i...</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>MAE 301: Applied Experimental Statistic | MAE 593: Applied Project | MAE 547: Modeling and Control of Robots</t>
+        </is>
+      </c>
       <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>If you are interested, please email Dr</t>
+        </is>
+      </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
           <t>https://irislab.tech/</t>
@@ -8052,7 +8364,11 @@
         <f>HYPERLINK("https://irislab.tech/", "https://irislab.tech/")</f>
         <v/>
       </c>
-      <c r="U35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>Looking for ASU Undergraduate and Master Students</t>
+        </is>
+      </c>
       <c r="V35" s="2" t="inlineStr"/>
       <c r="W35" s="2" t="inlineStr">
         <is>
@@ -8068,7 +8384,11 @@
           <t>Recent Updates</t>
         </is>
       </c>
-      <c r="Z35" s="2" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA35" s="2" t="b">
         <v>1</v>
       </c>
@@ -8213,12 +8533,12 @@
           <t>materials</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>MAE 301: Applied Experimental Statistic | MAE 593: Applied Project | MAE 494: Special Topics</t>
-        </is>
-      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Dylan Joralmon~, Soham Khairnar, Xiangjia Li*, "Rapid Fabrication of Multi-Metal 3D Objects with Adjustable Gradients by Contin...</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
           <t>2026 The J. Orin Edson Entrepreneurship &amp; Innovation Seed Funding Award ASU 2025 1st place Skysong Startup Competition C</t>
@@ -8254,7 +8574,11 @@
         <f>HYPERLINK("https://www.cindyxjli.com/", "https://www.cindyxjli.com/")</f>
         <v/>
       </c>
-      <c r="U37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
+        </is>
+      </c>
       <c r="V37" s="2" t="inlineStr"/>
       <c r="W37" s="2" t="inlineStr">
         <is>
@@ -8267,11 +8591,7 @@
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr">
-        <is>
-          <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
-        </is>
-      </c>
+      <c r="Z37" s="2" t="inlineStr"/>
       <c r="AA37" s="2" t="b">
         <v>1</v>
       </c>
@@ -8322,16 +8642,8 @@
           <t>aerospace</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>Journal Articles Middleton, J. A. (in press). Archimedes, Euler, &amp; Nursing Cats: Rethinking the Arithmetic Mean. OnCore,</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>MAE 484: Internship | MAE 301: Applied Experimental Statistic | MAE 394: Special Topics</t>
-        </is>
-      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr">
@@ -8357,11 +8669,7 @@
       <c r="W38" s="2" t="inlineStr"/>
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="2" t="inlineStr"/>
-      <c r="Z38" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 381 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z38" s="2" t="inlineStr"/>
       <c r="AA38" s="2" t="b">
         <v>1</v>
       </c>
@@ -8495,11 +8803,7 @@
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>MAE 510: Dynamics and Vibrations | MAE 591: Seminar | MAE 394: Special Topics</t>
-        </is>
-      </c>
+      <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
@@ -8521,11 +8825,7 @@
       <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
-      <c r="Z40" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z40" s="2" t="inlineStr"/>
       <c r="AA40" s="2" t="b">
         <v>1</v>
       </c>
@@ -8577,7 +8877,11 @@
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>MAE 213: Mechanics of Materials | MAE 593: Applied Project | MAE 520: Stress Analysis</t>
+        </is>
+      </c>
       <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="2" t="inlineStr"/>
       <c r="O41" s="2" t="inlineStr"/>
@@ -8602,7 +8906,11 @@
       <c r="W41" s="2" t="inlineStr"/>
       <c r="X41" s="2" t="inlineStr"/>
       <c r="Y41" s="2" t="inlineStr"/>
-      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 352 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA41" s="2" t="b">
         <v>1</v>
       </c>
@@ -8657,7 +8965,11 @@
           <t>materials</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>top of page This website was built on Wix. Create yours today. Get Started Bio &amp; Nano Lab Home Dr. Kang Lab Members Publication...</t>
+        </is>
+      </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
           <t>MAE 598: Special Topics | MAE 494: Special Topics | MAE 202: Mech.Particles/Rigid Bodies II</t>
@@ -8767,7 +9079,11 @@
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>MAE 494: Special Topics | MAE 598: Special Topics | MAE 301: Applied Experimental Statistic</t>
+        </is>
+      </c>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr"/>
       <c r="O43" s="2" t="inlineStr"/>
@@ -8789,7 +9105,11 @@
       <c r="W43" s="2" t="inlineStr"/>
       <c r="X43" s="2" t="inlineStr"/>
       <c r="Y43" s="2" t="inlineStr"/>
-      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>GWC 464 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA43" s="2" t="b">
         <v>1</v>
       </c>
@@ -8837,7 +9157,11 @@
       </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 301: Applied Experimental Statistic | MAE 241: Intro to Thermodynamics</t>
+        </is>
+      </c>
       <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="2" t="inlineStr"/>
       <c r="O44" s="2" t="inlineStr"/>
@@ -8851,7 +9175,11 @@
       <c r="W44" s="2" t="inlineStr"/>
       <c r="X44" s="2" t="inlineStr"/>
       <c r="Y44" s="2" t="inlineStr"/>
-      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA44" s="2" t="b">
         <v>0</v>
       </c>
@@ -8899,7 +9227,11 @@
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>MAE 301: Applied Experimental Statistic | MAE 202: Mech.Particles/Rigid Bodies II | MAE 417: System Dynamics and Control II</t>
+        </is>
+      </c>
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="inlineStr"/>
@@ -8917,7 +9249,11 @@
       <c r="W45" s="2" t="inlineStr"/>
       <c r="X45" s="2" t="inlineStr"/>
       <c r="Y45" s="2" t="inlineStr"/>
-      <c r="Z45" s="2" t="inlineStr"/>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Otherus</t>
+        </is>
+      </c>
       <c r="AA45" s="2" t="b">
         <v>0</v>
       </c>
@@ -9027,11 +9363,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>MAE 241: Intro to Thermodynamics | MAE 215: Intro to Programming in MATLAB | MAE 384: Adv Math Methods for Engineers</t>
-        </is>
-      </c>
+      <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr"/>
       <c r="O47" s="2" t="inlineStr"/>
@@ -9045,11 +9377,7 @@
       <c r="W47" s="2" t="inlineStr"/>
       <c r="X47" s="2" t="inlineStr"/>
       <c r="Y47" s="2" t="inlineStr"/>
-      <c r="Z47" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="Z47" s="2" t="inlineStr"/>
       <c r="AA47" s="2" t="b">
         <v>0</v>
       </c>
@@ -9097,7 +9425,11 @@
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
-      <c r="L48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>MAE 201: Mech. Particles/Rigid Bodies I | MAE 214: Computer-Aided Engineering I | MAE 202: Mech.Particles/Rigid Bodies II</t>
+        </is>
+      </c>
       <c r="M48" s="2" t="inlineStr"/>
       <c r="N48" s="2" t="inlineStr"/>
       <c r="O48" s="2" t="inlineStr"/>
@@ -9111,7 +9443,11 @@
       <c r="W48" s="2" t="inlineStr"/>
       <c r="X48" s="2" t="inlineStr"/>
       <c r="Y48" s="2" t="inlineStr"/>
-      <c r="Z48" s="2" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA48" s="2" t="b">
         <v>0</v>
       </c>
@@ -9159,7 +9495,11 @@
       </c>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>MAE 570: Intermediate Thermodynamics | MAE 400: Engineering Profession | MAE 494: Special Topics</t>
+        </is>
+      </c>
       <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr"/>
       <c r="O49" s="2" t="inlineStr"/>
@@ -9173,7 +9513,11 @@
       <c r="W49" s="2" t="inlineStr"/>
       <c r="X49" s="2" t="inlineStr"/>
       <c r="Y49" s="2" t="inlineStr"/>
-      <c r="Z49" s="2" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA49" s="2" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Integrate automatic Markdown directory generation directly into asu_profs.py
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -677,11 +677,7 @@
           <t>Refereed Journal Papers M. H. Kasbaoui and M. Herrmann, A high-fidelity methodology for particle-resolved direct numerical simu...</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>MAE 242: Intro to Fluid Mechanics | MAE 574: Multiphase Flow | MAE 501: Linear Algebra in Engineering</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -725,11 +721,7 @@
           <t>School for Engineering of Matter, Transport &amp; Energy</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="Z2" s="2" t="inlineStr"/>
       <c r="AA2" s="2" t="b">
         <v>1</v>
       </c>
@@ -797,7 +789,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Please send your CV to Prof</t>
+          <t>Please send your CV to Prof. Wang ( [email protected] ). We will try to get back to you ASAP with possible available positions. Please also send a 2-page statement on describing your previous research experience as well as how your research interests match Prof. Wang’s group’s research themes. | Please send Prof. Wang ( [email protected] ) with your resumes for applications and for more details on the projects.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -906,7 +898,7 @@
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>If you're interested in joining our group, please email</t>
+          <t>If you're interested in joining our group, please email Prof. Oswald with your CV, research interests, and any supporting materials such as publications or code samples.</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -934,11 +926,7 @@
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>What we're looking for:</t>
-        </is>
-      </c>
+      <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr"/>
@@ -1019,7 +1007,7 @@
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Additionally, they should send an email titled “Prospective Ph</t>
+          <t>To apply, interested candidates should submit an application to Arizona State University via https://webapp4.asu.edu/dgsadmissions/ , specifying their interest in working with Dr. Sun. Additionally, they should send an email titled “Prospective Ph.D. Student” to jiefeng.sun@asu.edu, attaching their CV and a cover letter before submitting their application. | I am seeking multiple highly motivated Master students or undergrads to conduct theses. To apply, interested candidates should fill in this form: https://forms.gle/RCwqu4wkCjhBUoFL7</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -1053,7 +1041,7 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>Dec 19, 2025 We have two openings for fully supported summer interns through SURI program at ASU</t>
+          <t>I am seeking multiple highly motivated Master students or undergrads to conduct theses. To apply, interested candidates should fill in this form: https://forms.gle/RCwqu4wkCjhBUoFL7 | I am a K-12 student/teacher and would like information for a school report, tour, help with my robotics team, a research internship, etc. My students and I are very excited about using robotics as a teaching tool to encourage interest in Science, Technology, Engineering, and Math (STEM) topics. We actively involved in outreach and are have an outreach webpage to answer your questions.</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr"/>
@@ -1421,7 +1409,7 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Potential candidates with strong backgrounds in fluid-structure interaction, soft robotics , machine learning can send their CV to leixinma@asu</t>
+          <t>Undergraduate students : Highly-motivated undergraduate students are encouraged to get in touch. The students are encouraged to apply Fulton Undergraduate Research Initiative (FURI) ( Proposals are due the 3rd Wednesday of every March and October ) , Summer Research Initiative (SURI) etc. No prior research experiences are expected. Email to: leixinma@ asu .edu . | Visiting scholars from different backgrounds are welcome to contact Prof. Ma for projects with mutual interests. Email to: leixinma@asu.edu</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1455,7 +1443,7 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
+          <t>More Home Research People Publications News Openings Facility Teaching Resources | Update: We are currently hiring multiple fully-funded graduate students, undergraduate students and visiting scholars! The first year graduate students will be selected as the prestigious Ira A. Fulton fellowship from the ASU School of Engineering.</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr"/>
@@ -1523,7 +1511,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous velocity and density measurements of fully developed Rayleigh-Taylor turbulent mixing</t>
+          <t>There is an open post-doctoral opening starting Fall 2025 in experimental turbulence research . All students interested in join...</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1815,7 +1803,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Selected Journal Papers Nasim Baharisangari, Kazuma Hirota, Ruixuan Yan, Agung Julius, Zhe Xu , Weighted Graph-Based Sig</t>
+          <t>Search this site Embedded Files Skip to main content Skip to navigation Home Publications Research Teaching Group Members Outre...</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1850,11 +1838,7 @@
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="U13" s="2" t="inlineStr">
-        <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
-        </is>
-      </c>
+      <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="inlineStr"/>
       <c r="W13" s="2" t="inlineStr"/>
       <c r="X13" s="2" t="inlineStr"/>
@@ -1970,7 +1954,7 @@
         <v/>
       </c>
       <c r="D15" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=l7umOqMAAAAJ", "Scholar (l7umOqMAAAAJ)")</f>
         <v/>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1983,7 +1967,11 @@
           <t>Aerospace &amp; Mechanical Engineering</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>l7umOqMAAAAJ</t>
+        </is>
+      </c>
       <c r="H15" s="3">
         <f>HYPERLINK("mailto:mpeet@asu.edu", "mpeet@asu.edu")</f>
         <v/>
@@ -1997,7 +1985,11 @@
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>MAE 593: Applied Project | MAE 318: System Dynamics and Control I | MAE 509: LMI Methods</t>
+        </is>
+      </c>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
@@ -2034,7 +2026,11 @@
       <c r="W15" s="2" t="inlineStr"/>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="inlineStr"/>
-      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 253 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA15" s="2" t="b">
         <v>1</v>
       </c>
@@ -2452,11 +2448,7 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>MAE 557: Mechanics Composite Materials | MAE 494: Special Topics | MAE 521: Structural Optimization</t>
-        </is>
-      </c>
+      <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
@@ -2482,11 +2474,7 @@
       <c r="W20" s="2" t="inlineStr"/>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
-      <c r="Z20" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z20" s="2" t="inlineStr"/>
       <c r="AA20" s="2" t="b">
         <v>1</v>
       </c>
@@ -2672,11 +2660,7 @@
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="U22" s="2" t="inlineStr">
-        <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
-        </is>
-      </c>
+      <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr">
         <is>
@@ -3317,11 +3301,7 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>MAE 502: Partial Diff Equations Engr | MAE 460: Applied Comput Fluid Dynamics | MAE 593: Applied Project</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
@@ -3341,11 +3321,7 @@
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="U29" s="2" t="inlineStr">
-        <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
-        </is>
-      </c>
+      <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
@@ -3354,11 +3330,7 @@
           <t>Log in to www_public</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="b">
         <v>1</v>
       </c>
@@ -3900,7 +3872,7 @@
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>If you are interested, please email Dr</t>
+          <t>If you are interested, please email Dr. Wanxin Jin with your CV, transcript, and a brief description of your research interests. In your email, please mention the topics you are interested in, your relevant background, and whether you are looking for thesis research, independent study, an applied project, hourly research work, or volunteer research experience. | If you are interested, please submit this form: https://forms.gle/Yo5mQcwTrogHTgu77 . If there is a potential fit, you should expect to be contacted within one week; if you do not hear back, please email wjin@asu.edu for follow-up.</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
@@ -3930,7 +3902,7 @@
       </c>
       <c r="U35" s="2" t="inlineStr">
         <is>
-          <t>Looking for ASU Undergraduate and Master Students</t>
+          <t>ASU undergraduate and master students are welcome to join IRIS Lab research projects in robotics, embodied AI, vision and perception, robot learning, control, and autonomy. Students interested in a thesis, independent study, or sustained applied research project are especially encouraged to reach out. | If you are interested, please email Dr. Wanxin Jin with your CV, transcript, and a brief description of your research interests. In your email, please mention the topics you are interested in, your relevant background, and whether you are looking for thesis research, independent study, an applied project, hourly research work, or volunteer research experience.</t>
         </is>
       </c>
       <c r="V35" s="2" t="inlineStr"/>
@@ -4102,13 +4074,21 @@
           <t>Dylan Joralmon~, Soham Khairnar, Xiangjia Li*, "Rapid Fabrication of Multi-Metal 3D Objects with Adjustable Gradients by Contin...</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>MAE 301: Applied Experimental Statistic | MAE 593: Applied Project | MAE 494: Special Topics</t>
+        </is>
+      </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
           <t>2026 The J. Orin Edson Entrepreneurship &amp; Innovation Seed Funding Award ASU 2025 1st place Skysong Startup Competition C</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>If you are interested in joining us, please send the full CV (with GPA; working and research experiences; publications) to Prof. Li (email: xiangjia.li AT asu.edu).</t>
+        </is>
+      </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
           <t>Biomimetic Additive Manufacturing (3D Printing); Bioinspired Material and Structure Design; Stereolithography; Photopolymerization based 3D Printing; Multi-material and Multi-scale 3D printing; Biofabrication; Biomaterial; Ceramic Printing; Nanocomposite Printing; Physical Field Assisted Printing; 4D Printing; Flexible Sensor; Biomedical Device; Tissue Repair and Regeneration.</t>
@@ -4140,7 +4120,7 @@
       </c>
       <c r="U37" s="2" t="inlineStr">
         <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
+          <t>The labMI is looking for creative, motivated and energetic Ph.D., Master and Undergraduate students from diverse science and engineering field!</t>
         </is>
       </c>
       <c r="V37" s="2" t="inlineStr"/>
@@ -4155,7 +4135,11 @@
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
+        </is>
+      </c>
       <c r="AA37" s="2" t="b">
         <v>1</v>
       </c>
@@ -4367,7 +4351,11 @@
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>MAE 510: Dynamics and Vibrations | MAE 591: Seminar | MAE 394: Special Topics</t>
+        </is>
+      </c>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
@@ -4389,7 +4377,11 @@
       <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
-      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA40" s="2" t="b">
         <v>1</v>
       </c>
@@ -4572,7 +4564,7 @@
       </c>
       <c r="U42" s="2" t="inlineStr">
         <is>
-          <t>Welcome and we are looking forward to working with Dr</t>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
         </is>
       </c>
       <c r="V42" s="2" t="inlineStr"/>
@@ -5113,11 +5105,7 @@
           <t>Refereed Journal Papers M. H. Kasbaoui and M. Herrmann, A high-fidelity methodology for particle-resolved direct numerical simu...</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>MAE 242: Intro to Fluid Mechanics | MAE 574: Multiphase Flow | MAE 501: Linear Algebra in Engineering</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -5161,11 +5149,7 @@
           <t>School for Engineering of Matter, Transport &amp; Energy</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
+      <c r="Z2" s="2" t="inlineStr"/>
       <c r="AA2" s="2" t="b">
         <v>1</v>
       </c>
@@ -5233,7 +5217,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Please send your CV to Prof</t>
+          <t>Please send your CV to Prof. Wang ( [email protected] ). We will try to get back to you ASAP with possible available positions. Please also send a 2-page statement on describing your previous research experience as well as how your research interests match Prof. Wang’s group’s research themes. | Please send Prof. Wang ( [email protected] ) with your resumes for applications and for more details on the projects.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -5342,7 +5326,7 @@
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>If you're interested in joining our group, please email</t>
+          <t>If you're interested in joining our group, please email Prof. Oswald with your CV, research interests, and any supporting materials such as publications or code samples.</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -5370,11 +5354,7 @@
         <f>HYPERLINK("http://sparky.fulton.asu.edu/oswald/", "http://sparky.fulton.asu.edu/oswald/")</f>
         <v/>
       </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>What we're looking for:</t>
-        </is>
-      </c>
+      <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr"/>
@@ -5455,7 +5435,7 @@
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Additionally, they should send an email titled “Prospective Ph</t>
+          <t>To apply, interested candidates should submit an application to Arizona State University via https://webapp4.asu.edu/dgsadmissions/ , specifying their interest in working with Dr. Sun. Additionally, they should send an email titled “Prospective Ph.D. Student” to jiefeng.sun@asu.edu, attaching their CV and a cover letter before submitting their application. | I am seeking multiple highly motivated Master students or undergrads to conduct theses. To apply, interested candidates should fill in this form: https://forms.gle/RCwqu4wkCjhBUoFL7</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -5489,7 +5469,7 @@
       </c>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>Dec 19, 2025 We have two openings for fully supported summer interns through SURI program at ASU</t>
+          <t>I am seeking multiple highly motivated Master students or undergrads to conduct theses. To apply, interested candidates should fill in this form: https://forms.gle/RCwqu4wkCjhBUoFL7 | I am a K-12 student/teacher and would like information for a school report, tour, help with my robotics team, a research internship, etc. My students and I are very excited about using robotics as a teaching tool to encourage interest in Science, Technology, Engineering, and Math (STEM) topics. We actively involved in outreach and are have an outreach webpage to answer your questions.</t>
         </is>
       </c>
       <c r="V5" s="2" t="inlineStr"/>
@@ -5857,7 +5837,7 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Potential candidates with strong backgrounds in fluid-structure interaction, soft robotics , machine learning can send their CV to leixinma@asu</t>
+          <t>Undergraduate students : Highly-motivated undergraduate students are encouraged to get in touch. The students are encouraged to apply Fulton Undergraduate Research Initiative (FURI) ( Proposals are due the 3rd Wednesday of every March and October ) , Summer Research Initiative (SURI) etc. No prior research experiences are expected. Email to: leixinma@ asu .edu . | Visiting scholars from different backgrounds are welcome to contact Prof. Ma for projects with mutual interests. Email to: leixinma@asu.edu</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -5891,7 +5871,7 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
+          <t>More Home Research People Publications News Openings Facility Teaching Resources | Update: We are currently hiring multiple fully-funded graduate students, undergraduate students and visiting scholars! The first year graduate students will be selected as the prestigious Ira A. Fulton fellowship from the ASU School of Engineering.</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr"/>
@@ -5959,7 +5939,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Simultaneous velocity and density measurements of fully developed Rayleigh-Taylor turbulent mixing</t>
+          <t>There is an open post-doctoral opening starting Fall 2025 in experimental turbulence research . All students interested in join...</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -6251,7 +6231,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Selected Journal Papers Nasim Baharisangari, Kazuma Hirota, Ruixuan Yan, Agung Julius, Zhe Xu , Weighted Graph-Based Sig</t>
+          <t>Search this site Embedded Files Skip to main content Skip to navigation Home Publications Research Teaching Group Members Outre...</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -6286,11 +6266,7 @@
         <f>HYPERLINK("https://sites.google.com/site/zhexudavid00710/research?authuser=0", "https://sites.google.com/site/zhexudavid00710/research?authuser=0")</f>
         <v/>
       </c>
-      <c r="U13" s="2" t="inlineStr">
-        <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
-        </is>
-      </c>
+      <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="inlineStr"/>
       <c r="W13" s="2" t="inlineStr"/>
       <c r="X13" s="2" t="inlineStr"/>
@@ -6406,7 +6382,7 @@
         <v/>
       </c>
       <c r="D15" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Matthew%20Peet%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=l7umOqMAAAAJ", "Scholar (l7umOqMAAAAJ)")</f>
         <v/>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -6419,7 +6395,11 @@
           <t>Aerospace &amp; Mechanical Engineering</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>l7umOqMAAAAJ</t>
+        </is>
+      </c>
       <c r="H15" s="3">
         <f>HYPERLINK("mailto:mpeet@asu.edu", "mpeet@asu.edu")</f>
         <v/>
@@ -6433,7 +6413,11 @@
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>MAE 593: Applied Project | MAE 318: System Dynamics and Control I | MAE 509: LMI Methods</t>
+        </is>
+      </c>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr">
@@ -6470,7 +6454,11 @@
       <c r="W15" s="2" t="inlineStr"/>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="inlineStr"/>
-      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 253 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA15" s="2" t="b">
         <v>1</v>
       </c>
@@ -6888,11 +6876,7 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>MAE 557: Mechanics Composite Materials | MAE 494: Special Topics | MAE 521: Structural Optimization</t>
-        </is>
-      </c>
+      <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
@@ -6918,11 +6902,7 @@
       <c r="W20" s="2" t="inlineStr"/>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
-      <c r="Z20" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z20" s="2" t="inlineStr"/>
       <c r="AA20" s="2" t="b">
         <v>1</v>
       </c>
@@ -7108,11 +7088,7 @@
         <f>HYPERLINK("http://sites.google.com/view/3denergy", "http://sites.google.com/view/3denergy")</f>
         <v/>
       </c>
-      <c r="U22" s="2" t="inlineStr">
-        <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
-        </is>
-      </c>
+      <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr">
         <is>
@@ -7753,11 +7729,7 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>MAE 502: Partial Diff Equations Engr | MAE 460: Applied Comput Fluid Dynamics | MAE 593: Applied Project</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
@@ -7777,11 +7749,7 @@
         <f>HYPERLINK("http://www.public.asu.edu/~hhuang38", "http://www.public.asu.edu/~hhuang38")</f>
         <v/>
       </c>
-      <c r="U29" s="2" t="inlineStr">
-        <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
-        </is>
-      </c>
+      <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
@@ -7790,11 +7758,7 @@
           <t>Log in to www_public</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
+      <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="b">
         <v>1</v>
       </c>
@@ -8336,7 +8300,7 @@
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>If you are interested, please email Dr</t>
+          <t>If you are interested, please email Dr. Wanxin Jin with your CV, transcript, and a brief description of your research interests. In your email, please mention the topics you are interested in, your relevant background, and whether you are looking for thesis research, independent study, an applied project, hourly research work, or volunteer research experience. | If you are interested, please submit this form: https://forms.gle/Yo5mQcwTrogHTgu77 . If there is a potential fit, you should expect to be contacted within one week; if you do not hear back, please email wjin@asu.edu for follow-up.</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
@@ -8366,7 +8330,7 @@
       </c>
       <c r="U35" s="2" t="inlineStr">
         <is>
-          <t>Looking for ASU Undergraduate and Master Students</t>
+          <t>ASU undergraduate and master students are welcome to join IRIS Lab research projects in robotics, embodied AI, vision and perception, robot learning, control, and autonomy. Students interested in a thesis, independent study, or sustained applied research project are especially encouraged to reach out. | If you are interested, please email Dr. Wanxin Jin with your CV, transcript, and a brief description of your research interests. In your email, please mention the topics you are interested in, your relevant background, and whether you are looking for thesis research, independent study, an applied project, hourly research work, or volunteer research experience.</t>
         </is>
       </c>
       <c r="V35" s="2" t="inlineStr"/>
@@ -8538,13 +8502,21 @@
           <t>Dylan Joralmon~, Soham Khairnar, Xiangjia Li*, "Rapid Fabrication of Multi-Metal 3D Objects with Adjustable Gradients by Contin...</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>MAE 301: Applied Experimental Statistic | MAE 593: Applied Project | MAE 494: Special Topics</t>
+        </is>
+      </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
           <t>2026 The J. Orin Edson Entrepreneurship &amp; Innovation Seed Funding Award ASU 2025 1st place Skysong Startup Competition C</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>If you are interested in joining us, please send the full CV (with GPA; working and research experiences; publications) to Prof. Li (email: xiangjia.li AT asu.edu).</t>
+        </is>
+      </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
           <t>Biomimetic Additive Manufacturing (3D Printing); Bioinspired Material and Structure Design; Stereolithography; Photopolymerization based 3D Printing; Multi-material and Multi-scale 3D printing; Biofabrication; Biomaterial; Ceramic Printing; Nanocomposite Printing; Physical Field Assisted Printing; 4D Printing; Flexible Sensor; Biomedical Device; Tissue Repair and Regeneration.</t>
@@ -8576,7 +8548,7 @@
       </c>
       <c r="U37" s="2" t="inlineStr">
         <is>
-          <t>Actively recruiting / Openings mentioned on lab site</t>
+          <t>The labMI is looking for creative, motivated and energetic Ph.D., Master and Undergraduate students from diverse science and engineering field!</t>
         </is>
       </c>
       <c r="V37" s="2" t="inlineStr"/>
@@ -8591,7 +8563,11 @@
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
+        </is>
+      </c>
       <c r="AA37" s="2" t="b">
         <v>1</v>
       </c>
@@ -8803,7 +8779,11 @@
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>MAE 510: Dynamics and Vibrations | MAE 591: Seminar | MAE 394: Special Topics</t>
+        </is>
+      </c>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
@@ -8825,7 +8805,11 @@
       <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
-      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
       <c r="AA40" s="2" t="b">
         <v>1</v>
       </c>
@@ -9008,7 +8992,7 @@
       </c>
       <c r="U42" s="2" t="inlineStr">
         <is>
-          <t>Welcome and we are looking forward to working with Dr</t>
+          <t>Actively recruiting / Openings mentioned on lab site</t>
         </is>
       </c>
       <c r="V42" s="2" t="inlineStr"/>
@@ -9227,11 +9211,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>MAE 301: Applied Experimental Statistic | MAE 202: Mech.Particles/Rigid Bodies II | MAE 417: System Dynamics and Control II</t>
-        </is>
-      </c>
+      <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="inlineStr"/>
@@ -9249,11 +9229,7 @@
       <c r="W45" s="2" t="inlineStr"/>
       <c r="X45" s="2" t="inlineStr"/>
       <c r="Y45" s="2" t="inlineStr"/>
-      <c r="Z45" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Otherus</t>
-        </is>
-      </c>
+      <c r="Z45" s="2" t="inlineStr"/>
       <c r="AA45" s="2" t="b">
         <v>0</v>
       </c>
@@ -9301,7 +9277,11 @@
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>MAE 318: System Dynamics and Control I | MAE 417: System Dynamics and Control II | MAE 215: Intro to Programming in MATLAB</t>
+        </is>
+      </c>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="inlineStr"/>
@@ -9315,7 +9295,11 @@
       <c r="W46" s="2" t="inlineStr"/>
       <c r="X46" s="2" t="inlineStr"/>
       <c r="Y46" s="2" t="inlineStr"/>
-      <c r="Z46" s="2" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
       <c r="AA46" s="2" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Update docs and pipeline to 29-column schema including Lab Facilities and Equipment
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB43"/>
+  <dimension ref="A1:AC43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -480,12 +480,13 @@
     <col width="49" customWidth="1" min="20" max="20"/>
     <col width="65" customWidth="1" min="21" max="21"/>
     <col width="53" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="49" customWidth="1" min="24" max="24"/>
-    <col width="56" customWidth="1" min="25" max="25"/>
-    <col width="54" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
-    <col width="49" customWidth="1" min="28" max="28"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="49" customWidth="1" min="25" max="25"/>
+    <col width="56" customWidth="1" min="26" max="26"/>
+    <col width="65" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="49" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -601,30 +602,35 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>Lab Facilities &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>Funding Sponsors</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Software / Code Repo</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Latest Project / Highlight</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Office Location</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Directory URL</t>
         </is>
@@ -677,7 +683,11 @@
           <t>Refereed Journal Papers M. H. Kasbaoui and M. Herrmann, A high-fidelity methodology for particle-resolved direct numerical simu...</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 574: Multiphase Flow | MAE 501: Linear Algebra in Engineering</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -707,25 +717,30 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>AFOSR</t>
         </is>
       </c>
-      <c r="X2" s="3">
+      <c r="Y2" s="3">
         <f>HYPERLINK("https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz", "https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master")</f>
         <v/>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>School for Engineering of Matter, Transport &amp; Energy</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
-      <c r="AA2" s="2" t="b">
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB2" s="3">
+      <c r="AC2" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -825,24 +840,29 @@
       <c r="V3" s="2" t="inlineStr"/>
       <c r="W3" s="2" t="inlineStr">
         <is>
+          <t>AFM</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
           <t>NASA, NSF</t>
         </is>
       </c>
-      <c r="X3" s="2" t="inlineStr"/>
-      <c r="Y3" s="2" t="inlineStr">
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>News&amp;Awards</t>
         </is>
       </c>
-      <c r="Z3" s="2" t="inlineStr">
+      <c r="AA3" s="2" t="inlineStr">
         <is>
           <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="b">
+      <c r="AB3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB3" s="3">
+      <c r="AC3" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -930,20 +950,21 @@
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr"/>
-      <c r="Y4" s="2" t="inlineStr">
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>Multiscale polymer analysis</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr">
+      <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>ENGRC 353 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="b">
+      <c r="AB4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB4" s="3">
+      <c r="AC4" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1047,20 +1068,21 @@
       <c r="V5" s="2" t="inlineStr"/>
       <c r="W5" s="2" t="inlineStr"/>
       <c r="X5" s="2" t="inlineStr"/>
-      <c r="Y5" s="2" t="inlineStr">
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>Mission and Core Values</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr">
+      <c r="AA5" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="b">
+      <c r="AB5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB5" s="3">
+      <c r="AC5" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1138,15 +1160,16 @@
       <c r="W6" s="2" t="inlineStr"/>
       <c r="X6" s="2" t="inlineStr"/>
       <c r="Y6" s="2" t="inlineStr"/>
-      <c r="Z6" s="2" t="inlineStr">
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr">
         <is>
           <t>ENGRC 361 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA6" s="2" t="b">
+      <c r="AB6" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB6" s="3">
+      <c r="AC6" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1198,7 +1221,11 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 593: Applied Project | MAE 564: Advanced Aerodynamics</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr">
@@ -1225,10 +1252,15 @@
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="inlineStr"/>
       <c r="Z7" s="2" t="inlineStr"/>
-      <c r="AA7" s="2" t="b">
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>Engineering research centre Room 383 551 E Tyler mall (Tempe, AZ 85281)</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB7" s="3">
+      <c r="AC7" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1337,15 +1369,16 @@
       <c r="W8" s="2" t="inlineStr"/>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="2" t="inlineStr"/>
-      <c r="Z8" s="2" t="inlineStr">
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA8" s="2" t="b">
+      <c r="AB8" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB8" s="3">
+      <c r="AC8" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1447,22 +1480,27 @@
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr"/>
-      <c r="W9" s="2" t="inlineStr"/>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>Towing Tank, FDM</t>
+        </is>
+      </c>
       <c r="X9" s="2" t="inlineStr"/>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr">
         <is>
           <t>Ocean and Soft Intelligent Structure Interaction Lab</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr">
+      <c r="AA9" s="2" t="inlineStr">
         <is>
           <t>ERC 485 (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="b">
+      <c r="AB9" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB9" s="3">
+      <c r="AC9" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1550,20 +1588,21 @@
       <c r="V10" s="2" t="inlineStr"/>
       <c r="W10" s="2" t="inlineStr"/>
       <c r="X10" s="2" t="inlineStr"/>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr">
         <is>
           <t>Want to be part of CMAT Lab?</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr">
+      <c r="AA10" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="b">
+      <c r="AB10" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB10" s="3">
+      <c r="AC10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1645,15 +1684,16 @@
       <c r="W11" s="2" t="inlineStr"/>
       <c r="X11" s="2" t="inlineStr"/>
       <c r="Y11" s="2" t="inlineStr"/>
-      <c r="Z11" s="2" t="inlineStr">
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr">
         <is>
           <t>ENGRC 311 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA11" s="2" t="b">
+      <c r="AB11" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB11" s="3">
+      <c r="AC11" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1746,15 +1786,16 @@
       <c r="W12" s="2" t="inlineStr"/>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr"/>
-      <c r="Z12" s="2" t="inlineStr">
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr">
         <is>
           <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA12" s="2" t="b">
+      <c r="AB12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB12" s="3">
+      <c r="AC12" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1843,15 +1884,16 @@
       <c r="W13" s="2" t="inlineStr"/>
       <c r="X13" s="2" t="inlineStr"/>
       <c r="Y13" s="2" t="inlineStr"/>
-      <c r="Z13" s="2" t="inlineStr">
+      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AA13" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA13" s="2" t="b">
+      <c r="AB13" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB13" s="3">
+      <c r="AC13" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -1925,15 +1967,16 @@
       <c r="W14" s="2" t="inlineStr"/>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="inlineStr"/>
-      <c r="Z14" s="2" t="inlineStr">
+      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA14" s="2" t="b">
+      <c r="AB14" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB14" s="3">
+      <c r="AC14" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2026,15 +2069,16 @@
       <c r="W15" s="2" t="inlineStr"/>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="inlineStr"/>
-      <c r="Z15" s="2" t="inlineStr">
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="inlineStr">
         <is>
           <t>ENGRC 253 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA15" s="2" t="b">
+      <c r="AB15" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB15" s="3">
+      <c r="AC15" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2086,11 +2130,7 @@
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>MAE 241: Intro to Thermodynamics | MAE 593: Applied Project | MAE 588: Nanoscale Heat Transfer</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
@@ -2123,15 +2163,12 @@
       <c r="W16" s="2" t="inlineStr"/>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="2" t="inlineStr"/>
-      <c r="Z16" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 307 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="AA16" s="2" t="b">
+      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="AA16" s="2" t="inlineStr"/>
+      <c r="AB16" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB16" s="3">
+      <c r="AC16" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2228,15 +2265,16 @@
       <c r="W17" s="2" t="inlineStr"/>
       <c r="X17" s="2" t="inlineStr"/>
       <c r="Y17" s="2" t="inlineStr"/>
-      <c r="Z17" s="2" t="inlineStr">
+      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr">
         <is>
           <t>ENGRC 465 (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="b">
+      <c r="AB17" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB17" s="3">
+      <c r="AC17" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2314,15 +2352,16 @@
       <c r="W18" s="2" t="inlineStr"/>
       <c r="X18" s="2" t="inlineStr"/>
       <c r="Y18" s="2" t="inlineStr"/>
-      <c r="Z18" s="2" t="inlineStr">
+      <c r="Z18" s="2" t="inlineStr"/>
+      <c r="AA18" s="2" t="inlineStr">
         <is>
           <t>ENGRC 377 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA18" s="2" t="b">
+      <c r="AB18" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB18" s="3">
+      <c r="AC18" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2343,7 +2382,7 @@
         <v/>
       </c>
       <c r="D19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
         <v/>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2356,7 +2395,11 @@
           <t>Aerospace &amp; Mechanical Engineering</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>OmBV67MAAAAJ</t>
+        </is>
+      </c>
       <c r="H19" s="3">
         <f>HYPERLINK("mailto:Tianyu.Yang@asu.edu", "Tianyu.Yang@asu.edu")</f>
         <v/>
@@ -2370,7 +2413,11 @@
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>MAE 241: Intro to Thermodynamics</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
@@ -2393,10 +2440,15 @@
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr"/>
       <c r="Z19" s="2" t="inlineStr"/>
-      <c r="AA19" s="2" t="b">
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="AB19" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB19" s="3">
+      <c r="AC19" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2448,7 +2500,11 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>MAE 557: Mechanics Composite Materials | MAE 494: Special Topics | MAE 521: Structural Optimization</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
@@ -2475,10 +2531,15 @@
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
       <c r="Z20" s="2" t="inlineStr"/>
-      <c r="AA20" s="2" t="b">
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB20" s="3">
+      <c r="AC20" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2564,15 +2625,16 @@
       <c r="W21" s="2" t="inlineStr"/>
       <c r="X21" s="2" t="inlineStr"/>
       <c r="Y21" s="2" t="inlineStr"/>
-      <c r="Z21" s="2" t="inlineStr">
+      <c r="Z21" s="2" t="inlineStr"/>
+      <c r="AA21" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA21" s="2" t="b">
+      <c r="AB21" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB21" s="3">
+      <c r="AC21" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2664,24 +2726,29 @@
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr">
         <is>
+          <t>3D Printer</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
           <t>NSF</t>
         </is>
       </c>
-      <c r="X22" s="2" t="inlineStr"/>
-      <c r="Y22" s="2" t="inlineStr">
+      <c r="Y22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr">
         <is>
           <t>3D Energy Device Laboratory</t>
         </is>
       </c>
-      <c r="Z22" s="2" t="inlineStr">
+      <c r="AA22" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 363 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA22" s="2" t="b">
+      <c r="AB22" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB22" s="3">
+      <c r="AC22" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2778,15 +2845,16 @@
       <c r="W23" s="2" t="inlineStr"/>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="inlineStr"/>
-      <c r="Z23" s="2" t="inlineStr">
+      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="AA23" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA23" s="2" t="b">
+      <c r="AB23" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB23" s="3">
+      <c r="AC23" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2863,15 +2931,16 @@
       <c r="W24" s="2" t="inlineStr"/>
       <c r="X24" s="2" t="inlineStr"/>
       <c r="Y24" s="2" t="inlineStr"/>
-      <c r="Z24" s="2" t="inlineStr">
+      <c r="Z24" s="2" t="inlineStr"/>
+      <c r="AA24" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA24" s="2" t="b">
+      <c r="AB24" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB24" s="3">
+      <c r="AC24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -2960,15 +3029,16 @@
       <c r="W25" s="2" t="inlineStr"/>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="inlineStr"/>
-      <c r="Z25" s="2" t="inlineStr">
+      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AA25" s="2" t="inlineStr">
         <is>
           <t>ISTB4, ROOM 379 781 S Terrace Rd (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA25" s="2" t="b">
+      <c r="AB25" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB25" s="3">
+      <c r="AC25" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3054,15 +3124,16 @@
       <c r="W26" s="2" t="inlineStr"/>
       <c r="X26" s="2" t="inlineStr"/>
       <c r="Y26" s="2" t="inlineStr"/>
-      <c r="Z26" s="2" t="inlineStr">
+      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AA26" s="2" t="inlineStr">
         <is>
           <t>ENGRC 463 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA26" s="2" t="b">
+      <c r="AB26" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB26" s="3">
+      <c r="AC26" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3147,15 +3218,16 @@
       <c r="W27" s="2" t="inlineStr"/>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="inlineStr"/>
-      <c r="Z27" s="2" t="inlineStr">
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr">
         <is>
           <t>ENGRC 379 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA27" s="2" t="b">
+      <c r="AB27" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB27" s="3">
+      <c r="AC27" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3245,15 +3317,16 @@
       <c r="W28" s="2" t="inlineStr"/>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
-      <c r="Z28" s="2" t="inlineStr">
+      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AA28" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA28" s="2" t="b">
+      <c r="AB28" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB28" s="3">
+      <c r="AC28" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3301,7 +3374,11 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>MAE 502: Partial Diff Equations Engr | MAE 460: Applied Comput Fluid Dynamics | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
@@ -3325,16 +3402,21 @@
       <c r="V29" s="2" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
-      <c r="Y29" s="2" t="inlineStr">
+      <c r="Y29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
         <is>
           <t>Log in to www_public</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr"/>
-      <c r="AA29" s="2" t="b">
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB29" s="3">
+      <c r="AC29" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3430,20 +3512,21 @@
       <c r="V30" s="2" t="inlineStr"/>
       <c r="W30" s="2" t="inlineStr"/>
       <c r="X30" s="2" t="inlineStr"/>
-      <c r="Y30" s="2" t="inlineStr">
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
         <is>
           <t>Nanostructured Materials</t>
         </is>
       </c>
-      <c r="Z30" s="2" t="inlineStr">
+      <c r="AA30" s="2" t="inlineStr">
         <is>
           <t>ENGRC 355 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA30" s="2" t="b">
+      <c r="AB30" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB30" s="3">
+      <c r="AC30" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3530,13 +3613,18 @@
       <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr">
         <is>
+          <t>Rykaczewski Lab</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 309 (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA31" s="2" t="b">
+      <c r="AB31" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB31" s="3">
+      <c r="AC31" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3618,15 +3706,16 @@
       <c r="W32" s="2" t="inlineStr"/>
       <c r="X32" s="2" t="inlineStr"/>
       <c r="Y32" s="2" t="inlineStr"/>
-      <c r="Z32" s="2" t="inlineStr">
+      <c r="Z32" s="2" t="inlineStr"/>
+      <c r="AA32" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA32" s="2" t="b">
+      <c r="AB32" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB32" s="3">
+      <c r="AC32" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3711,15 +3800,16 @@
       <c r="W33" s="2" t="inlineStr"/>
       <c r="X33" s="2" t="inlineStr"/>
       <c r="Y33" s="2" t="inlineStr"/>
-      <c r="Z33" s="2" t="inlineStr">
+      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AA33" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA33" s="2" t="b">
+      <c r="AB33" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB33" s="3">
+      <c r="AC33" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3800,15 +3890,16 @@
       <c r="W34" s="2" t="inlineStr"/>
       <c r="X34" s="2" t="inlineStr"/>
       <c r="Y34" s="2" t="inlineStr"/>
-      <c r="Z34" s="2" t="inlineStr">
+      <c r="Z34" s="2" t="inlineStr"/>
+      <c r="AA34" s="2" t="inlineStr">
         <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA34" s="2" t="b">
+      <c r="AB34" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB34" s="3">
+      <c r="AC34" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -3906,29 +3997,30 @@
         </is>
       </c>
       <c r="V35" s="2" t="inlineStr"/>
-      <c r="W35" s="2" t="inlineStr">
+      <c r="W35" s="2" t="inlineStr"/>
+      <c r="X35" s="2" t="inlineStr">
         <is>
           <t>NSF</t>
         </is>
       </c>
-      <c r="X35" s="3">
+      <c r="Y35" s="3">
         <f>HYPERLINK("https://github.com/asu-iris", "https://github.com/asu-iris")</f>
         <v/>
       </c>
-      <c r="Y35" s="2" t="inlineStr">
+      <c r="Z35" s="2" t="inlineStr">
         <is>
           <t>Recent Updates</t>
         </is>
       </c>
-      <c r="Z35" s="2" t="inlineStr">
+      <c r="AA35" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA35" s="2" t="b">
+      <c r="AB35" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB35" s="3">
+      <c r="AC35" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4010,15 +4102,16 @@
       <c r="W36" s="2" t="inlineStr"/>
       <c r="X36" s="2" t="inlineStr"/>
       <c r="Y36" s="2" t="inlineStr"/>
-      <c r="Z36" s="2" t="inlineStr">
+      <c r="Z36" s="2" t="inlineStr"/>
+      <c r="AA36" s="2" t="inlineStr">
         <is>
           <t>ENGRC 409 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA36" s="2" t="b">
+      <c r="AB36" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB36" s="3">
+      <c r="AC36" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4124,26 +4217,27 @@
         </is>
       </c>
       <c r="V37" s="2" t="inlineStr"/>
-      <c r="W37" s="2" t="inlineStr">
+      <c r="W37" s="2" t="inlineStr"/>
+      <c r="X37" s="2" t="inlineStr">
         <is>
           <t>NSF</t>
         </is>
       </c>
-      <c r="X37" s="2" t="inlineStr"/>
-      <c r="Y37" s="2" t="inlineStr">
+      <c r="Y37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
         <is>
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr">
+      <c r="AA37" s="2" t="inlineStr">
         <is>
           <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA37" s="2" t="b">
+      <c r="AB37" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB37" s="3">
+      <c r="AC37" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4218,10 +4312,11 @@
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="2" t="inlineStr"/>
       <c r="Z38" s="2" t="inlineStr"/>
-      <c r="AA38" s="2" t="b">
+      <c r="AA38" s="2" t="inlineStr"/>
+      <c r="AB38" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB38" s="3">
+      <c r="AC38" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4295,15 +4390,16 @@
       <c r="W39" s="2" t="inlineStr"/>
       <c r="X39" s="2" t="inlineStr"/>
       <c r="Y39" s="2" t="inlineStr"/>
-      <c r="Z39" s="2" t="inlineStr">
+      <c r="Z39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA39" s="2" t="b">
+      <c r="AB39" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB39" s="3">
+      <c r="AC39" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4377,15 +4473,16 @@
       <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
-      <c r="Z40" s="2" t="inlineStr">
+      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="AA40" s="2" t="inlineStr">
         <is>
           <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA40" s="2" t="b">
+      <c r="AB40" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB40" s="3">
+      <c r="AC40" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4462,15 +4559,16 @@
       <c r="W41" s="2" t="inlineStr"/>
       <c r="X41" s="2" t="inlineStr"/>
       <c r="Y41" s="2" t="inlineStr"/>
-      <c r="Z41" s="2" t="inlineStr">
+      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AA41" s="2" t="inlineStr">
         <is>
           <t>ENGRC 352 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA41" s="2" t="b">
+      <c r="AB41" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB41" s="3">
+      <c r="AC41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4570,24 +4668,29 @@
       <c r="V42" s="2" t="inlineStr"/>
       <c r="W42" s="2" t="inlineStr">
         <is>
+          <t>SEM</t>
+        </is>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
           <t>NSF, ONR</t>
         </is>
       </c>
-      <c r="X42" s="2" t="inlineStr"/>
-      <c r="Y42" s="2" t="inlineStr">
+      <c r="Y42" s="2" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr">
         <is>
           <t>Highlighted as a cover in Small</t>
         </is>
       </c>
-      <c r="Z42" s="2" t="inlineStr">
+      <c r="AA42" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA42" s="2" t="b">
+      <c r="AB42" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB42" s="3">
+      <c r="AC42" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4661,15 +4764,16 @@
       <c r="W43" s="2" t="inlineStr"/>
       <c r="X43" s="2" t="inlineStr"/>
       <c r="Y43" s="2" t="inlineStr"/>
-      <c r="Z43" s="2" t="inlineStr">
+      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AA43" s="2" t="inlineStr">
         <is>
           <t>GWC 464 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA43" s="2" t="b">
+      <c r="AB43" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB43" s="3">
+      <c r="AC43" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -4680,198 +4784,198 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB7" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC7" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB8" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC8" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB9" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC9" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC10" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC12" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T13" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC13" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC14" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC15" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC16" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T17" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC18" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB21" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC21" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T23" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T24" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC24" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T25" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC25" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC26" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T27" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId122"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId123"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T29" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB29" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC29" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T30" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId137"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T31" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC31" r:id="rId141"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId145"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId146"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId147"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId148"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T33" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC33" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId151"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId152"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId153"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T34" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC34" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId157"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId158"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T35" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y35" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId165"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T37" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB37" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC37" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId171"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId174"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId175"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB39" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC39" r:id="rId178"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T41" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId187"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T42" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId196"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4883,7 +4987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AC49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4908,12 +5012,13 @@
     <col width="49" customWidth="1" min="20" max="20"/>
     <col width="65" customWidth="1" min="21" max="21"/>
     <col width="53" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="49" customWidth="1" min="24" max="24"/>
-    <col width="56" customWidth="1" min="25" max="25"/>
-    <col width="54" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
-    <col width="49" customWidth="1" min="28" max="28"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="49" customWidth="1" min="25" max="25"/>
+    <col width="56" customWidth="1" min="26" max="26"/>
+    <col width="65" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="49" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5029,30 +5134,35 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>Lab Facilities &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>Funding Sponsors</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Software / Code Repo</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Latest Project / Highlight</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Office Location</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Is Field Match</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Directory URL</t>
         </is>
@@ -5105,7 +5215,11 @@
           <t>Refereed Journal Papers M. H. Kasbaoui and M. Herrmann, A high-fidelity methodology for particle-resolved direct numerical simu...</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 574: Multiphase Flow | MAE 501: Linear Algebra in Engineering</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -5135,25 +5249,30 @@
           <t>CFD</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>AFOSR</t>
         </is>
       </c>
-      <c r="X2" s="3">
+      <c r="Y2" s="3">
         <f>HYPERLINK("https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz", "https://bitbucket.org/krgasu/leap/downloads/leap-v0.8.2.tar.gz, https://bitbucket.org/krgasu/leap/src/master")</f>
         <v/>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>School for Engineering of Matter, Transport &amp; Energy</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
-      <c r="AA2" s="2" t="b">
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB2" s="3">
+      <c r="AC2" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5253,24 +5372,29 @@
       <c r="V3" s="2" t="inlineStr"/>
       <c r="W3" s="2" t="inlineStr">
         <is>
+          <t>AFM</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
           <t>NASA, NSF</t>
         </is>
       </c>
-      <c r="X3" s="2" t="inlineStr"/>
-      <c r="Y3" s="2" t="inlineStr">
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>News&amp;Awards</t>
         </is>
       </c>
-      <c r="Z3" s="2" t="inlineStr">
+      <c r="AA3" s="2" t="inlineStr">
         <is>
           <t>ENGRC 327 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="b">
+      <c r="AB3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB3" s="3">
+      <c r="AC3" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5358,20 +5482,21 @@
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr"/>
-      <c r="Y4" s="2" t="inlineStr">
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>Multiscale polymer analysis</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr">
+      <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>ENGRC 353 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="b">
+      <c r="AB4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB4" s="3">
+      <c r="AC4" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5475,20 +5600,21 @@
       <c r="V5" s="2" t="inlineStr"/>
       <c r="W5" s="2" t="inlineStr"/>
       <c r="X5" s="2" t="inlineStr"/>
-      <c r="Y5" s="2" t="inlineStr">
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>Mission and Core Values</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr">
+      <c r="AA5" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="b">
+      <c r="AB5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB5" s="3">
+      <c r="AC5" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5566,15 +5692,16 @@
       <c r="W6" s="2" t="inlineStr"/>
       <c r="X6" s="2" t="inlineStr"/>
       <c r="Y6" s="2" t="inlineStr"/>
-      <c r="Z6" s="2" t="inlineStr">
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr">
         <is>
           <t>ENGRC 361 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA6" s="2" t="b">
+      <c r="AB6" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB6" s="3">
+      <c r="AC6" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5626,7 +5753,11 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>MAE 242: Intro to Fluid Mechanics | MAE 593: Applied Project | MAE 564: Advanced Aerodynamics</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr">
@@ -5653,10 +5784,15 @@
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="inlineStr"/>
       <c r="Z7" s="2" t="inlineStr"/>
-      <c r="AA7" s="2" t="b">
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>Engineering research centre Room 383 551 E Tyler mall (Tempe, AZ 85281)</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB7" s="3">
+      <c r="AC7" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5765,15 +5901,16 @@
       <c r="W8" s="2" t="inlineStr"/>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="2" t="inlineStr"/>
-      <c r="Z8" s="2" t="inlineStr">
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 475 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA8" s="2" t="b">
+      <c r="AB8" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB8" s="3">
+      <c r="AC8" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5875,22 +6012,27 @@
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr"/>
-      <c r="W9" s="2" t="inlineStr"/>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>Towing Tank, FDM</t>
+        </is>
+      </c>
       <c r="X9" s="2" t="inlineStr"/>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr">
         <is>
           <t>Ocean and Soft Intelligent Structure Interaction Lab</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr">
+      <c r="AA9" s="2" t="inlineStr">
         <is>
           <t>ERC 485 (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="b">
+      <c r="AB9" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB9" s="3">
+      <c r="AC9" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -5978,20 +6120,21 @@
       <c r="V10" s="2" t="inlineStr"/>
       <c r="W10" s="2" t="inlineStr"/>
       <c r="X10" s="2" t="inlineStr"/>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr">
         <is>
           <t>Want to be part of CMAT Lab?</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr">
+      <c r="AA10" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 479 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="b">
+      <c r="AB10" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB10" s="3">
+      <c r="AC10" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6073,15 +6216,16 @@
       <c r="W11" s="2" t="inlineStr"/>
       <c r="X11" s="2" t="inlineStr"/>
       <c r="Y11" s="2" t="inlineStr"/>
-      <c r="Z11" s="2" t="inlineStr">
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr">
         <is>
           <t>ENGRC 311 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA11" s="2" t="b">
+      <c r="AB11" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB11" s="3">
+      <c r="AC11" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6174,15 +6318,16 @@
       <c r="W12" s="2" t="inlineStr"/>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr"/>
-      <c r="Z12" s="2" t="inlineStr">
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr">
         <is>
           <t>ENGRC 375 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA12" s="2" t="b">
+      <c r="AB12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB12" s="3">
+      <c r="AC12" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6271,15 +6416,16 @@
       <c r="W13" s="2" t="inlineStr"/>
       <c r="X13" s="2" t="inlineStr"/>
       <c r="Y13" s="2" t="inlineStr"/>
-      <c r="Z13" s="2" t="inlineStr">
+      <c r="Z13" s="2" t="inlineStr"/>
+      <c r="AA13" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA13" s="2" t="b">
+      <c r="AB13" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB13" s="3">
+      <c r="AC13" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6353,15 +6499,16 @@
       <c r="W14" s="2" t="inlineStr"/>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="inlineStr"/>
-      <c r="Z14" s="2" t="inlineStr">
+      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA14" s="2" t="b">
+      <c r="AB14" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB14" s="3">
+      <c r="AC14" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6454,15 +6601,16 @@
       <c r="W15" s="2" t="inlineStr"/>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="inlineStr"/>
-      <c r="Z15" s="2" t="inlineStr">
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="inlineStr">
         <is>
           <t>ENGRC 253 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA15" s="2" t="b">
+      <c r="AB15" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB15" s="3">
+      <c r="AC15" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6514,11 +6662,7 @@
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>MAE 241: Intro to Thermodynamics | MAE 593: Applied Project | MAE 588: Nanoscale Heat Transfer</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
@@ -6551,15 +6695,12 @@
       <c r="W16" s="2" t="inlineStr"/>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="2" t="inlineStr"/>
-      <c r="Z16" s="2" t="inlineStr">
-        <is>
-          <t>ENGRC 307 (Tempe, AZ 85287-6106)</t>
-        </is>
-      </c>
-      <c r="AA16" s="2" t="b">
+      <c r="Z16" s="2" t="inlineStr"/>
+      <c r="AA16" s="2" t="inlineStr"/>
+      <c r="AB16" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB16" s="3">
+      <c r="AC16" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6656,15 +6797,16 @@
       <c r="W17" s="2" t="inlineStr"/>
       <c r="X17" s="2" t="inlineStr"/>
       <c r="Y17" s="2" t="inlineStr"/>
-      <c r="Z17" s="2" t="inlineStr">
+      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr">
         <is>
           <t>ENGRC 465 (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="b">
+      <c r="AB17" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB17" s="3">
+      <c r="AC17" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6742,15 +6884,16 @@
       <c r="W18" s="2" t="inlineStr"/>
       <c r="X18" s="2" t="inlineStr"/>
       <c r="Y18" s="2" t="inlineStr"/>
-      <c r="Z18" s="2" t="inlineStr">
+      <c r="Z18" s="2" t="inlineStr"/>
+      <c r="AA18" s="2" t="inlineStr">
         <is>
           <t>ENGRC 377 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA18" s="2" t="b">
+      <c r="AB18" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB18" s="3">
+      <c r="AC18" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6771,7 +6914,7 @@
         <v/>
       </c>
       <c r="D19" s="3">
-        <f>HYPERLINK("https://scholar.google.com/citations?view_op=search_authors&amp;mauthors=Tianyu%20Yang%20Arizona%20State%20University", "Google Scholar Search")</f>
+        <f>HYPERLINK("https://scholar.google.com/citations?hl=en&amp;user=OmBV67MAAAAJ", "Scholar (OmBV67MAAAAJ)")</f>
         <v/>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -6784,7 +6927,11 @@
           <t>Aerospace &amp; Mechanical Engineering</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>OmBV67MAAAAJ</t>
+        </is>
+      </c>
       <c r="H19" s="3">
         <f>HYPERLINK("mailto:Tianyu.Yang@asu.edu", "Tianyu.Yang@asu.edu")</f>
         <v/>
@@ -6798,7 +6945,11 @@
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>MAE 241: Intro to Thermodynamics</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
@@ -6821,10 +6972,15 @@
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr"/>
       <c r="Z19" s="2" t="inlineStr"/>
-      <c r="AA19" s="2" t="b">
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="AB19" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB19" s="3">
+      <c r="AC19" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6876,7 +7032,11 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>MAE 557: Mechanics Composite Materials | MAE 494: Special Topics | MAE 521: Structural Optimization</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
@@ -6903,10 +7063,15 @@
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
       <c r="Z20" s="2" t="inlineStr"/>
-      <c r="AA20" s="2" t="b">
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 427 (TEMPE, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="AB20" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB20" s="3">
+      <c r="AC20" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -6992,15 +7157,16 @@
       <c r="W21" s="2" t="inlineStr"/>
       <c r="X21" s="2" t="inlineStr"/>
       <c r="Y21" s="2" t="inlineStr"/>
-      <c r="Z21" s="2" t="inlineStr">
+      <c r="Z21" s="2" t="inlineStr"/>
+      <c r="AA21" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA21" s="2" t="b">
+      <c r="AB21" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB21" s="3">
+      <c r="AC21" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7092,24 +7258,29 @@
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr">
         <is>
+          <t>3D Printer</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
           <t>NSF</t>
         </is>
       </c>
-      <c r="X22" s="2" t="inlineStr"/>
-      <c r="Y22" s="2" t="inlineStr">
+      <c r="Y22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr">
         <is>
           <t>3D Energy Device Laboratory</t>
         </is>
       </c>
-      <c r="Z22" s="2" t="inlineStr">
+      <c r="AA22" s="2" t="inlineStr">
         <is>
           <t>551 E Tyler Mall ERC 363 (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA22" s="2" t="b">
+      <c r="AB22" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB22" s="3">
+      <c r="AC22" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7206,15 +7377,16 @@
       <c r="W23" s="2" t="inlineStr"/>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="inlineStr"/>
-      <c r="Z23" s="2" t="inlineStr">
+      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="AA23" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA23" s="2" t="b">
+      <c r="AB23" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB23" s="3">
+      <c r="AC23" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7291,15 +7463,16 @@
       <c r="W24" s="2" t="inlineStr"/>
       <c r="X24" s="2" t="inlineStr"/>
       <c r="Y24" s="2" t="inlineStr"/>
-      <c r="Z24" s="2" t="inlineStr">
+      <c r="Z24" s="2" t="inlineStr"/>
+      <c r="AA24" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA24" s="2" t="b">
+      <c r="AB24" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB24" s="3">
+      <c r="AC24" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7388,15 +7561,16 @@
       <c r="W25" s="2" t="inlineStr"/>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="inlineStr"/>
-      <c r="Z25" s="2" t="inlineStr">
+      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AA25" s="2" t="inlineStr">
         <is>
           <t>ISTB4, ROOM 379 781 S Terrace Rd (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA25" s="2" t="b">
+      <c r="AB25" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB25" s="3">
+      <c r="AC25" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7482,15 +7656,16 @@
       <c r="W26" s="2" t="inlineStr"/>
       <c r="X26" s="2" t="inlineStr"/>
       <c r="Y26" s="2" t="inlineStr"/>
-      <c r="Z26" s="2" t="inlineStr">
+      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AA26" s="2" t="inlineStr">
         <is>
           <t>ENGRC 463 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA26" s="2" t="b">
+      <c r="AB26" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB26" s="3">
+      <c r="AC26" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7575,15 +7750,16 @@
       <c r="W27" s="2" t="inlineStr"/>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="inlineStr"/>
-      <c r="Z27" s="2" t="inlineStr">
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr">
         <is>
           <t>ENGRC 379 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA27" s="2" t="b">
+      <c r="AB27" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB27" s="3">
+      <c r="AC27" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7673,15 +7849,16 @@
       <c r="W28" s="2" t="inlineStr"/>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
-      <c r="Z28" s="2" t="inlineStr">
+      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AA28" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA28" s="2" t="b">
+      <c r="AB28" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB28" s="3">
+      <c r="AC28" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7729,7 +7906,11 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>MAE 502: Partial Diff Equations Engr | MAE 460: Applied Comput Fluid Dynamics | MAE 593: Applied Project</t>
+        </is>
+      </c>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
@@ -7753,16 +7934,21 @@
       <c r="V29" s="2" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
-      <c r="Y29" s="2" t="inlineStr">
+      <c r="Y29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
         <is>
           <t>Log in to www_public</t>
         </is>
       </c>
-      <c r="Z29" s="2" t="inlineStr"/>
-      <c r="AA29" s="2" t="b">
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>ENGRC 359 (Tempe, AZ 85287-6106)</t>
+        </is>
+      </c>
+      <c r="AB29" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB29" s="3">
+      <c r="AC29" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7858,20 +8044,21 @@
       <c r="V30" s="2" t="inlineStr"/>
       <c r="W30" s="2" t="inlineStr"/>
       <c r="X30" s="2" t="inlineStr"/>
-      <c r="Y30" s="2" t="inlineStr">
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
         <is>
           <t>Nanostructured Materials</t>
         </is>
       </c>
-      <c r="Z30" s="2" t="inlineStr">
+      <c r="AA30" s="2" t="inlineStr">
         <is>
           <t>ENGRC 355 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA30" s="2" t="b">
+      <c r="AB30" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB30" s="3">
+      <c r="AC30" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -7958,13 +8145,18 @@
       <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr">
         <is>
+          <t>Rykaczewski Lab</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
           <t>ENGRC 309 (Tempe, AZ 85287)</t>
         </is>
       </c>
-      <c r="AA31" s="2" t="b">
+      <c r="AB31" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB31" s="3">
+      <c r="AC31" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8046,15 +8238,16 @@
       <c r="W32" s="2" t="inlineStr"/>
       <c r="X32" s="2" t="inlineStr"/>
       <c r="Y32" s="2" t="inlineStr"/>
-      <c r="Z32" s="2" t="inlineStr">
+      <c r="Z32" s="2" t="inlineStr"/>
+      <c r="AA32" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA32" s="2" t="b">
+      <c r="AB32" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB32" s="3">
+      <c r="AC32" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8139,15 +8332,16 @@
       <c r="W33" s="2" t="inlineStr"/>
       <c r="X33" s="2" t="inlineStr"/>
       <c r="Y33" s="2" t="inlineStr"/>
-      <c r="Z33" s="2" t="inlineStr">
+      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AA33" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA33" s="2" t="b">
+      <c r="AB33" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB33" s="3">
+      <c r="AC33" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8228,15 +8422,16 @@
       <c r="W34" s="2" t="inlineStr"/>
       <c r="X34" s="2" t="inlineStr"/>
       <c r="Y34" s="2" t="inlineStr"/>
-      <c r="Z34" s="2" t="inlineStr">
+      <c r="Z34" s="2" t="inlineStr"/>
+      <c r="AA34" s="2" t="inlineStr">
         <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA34" s="2" t="b">
+      <c r="AB34" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB34" s="3">
+      <c r="AC34" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8334,29 +8529,30 @@
         </is>
       </c>
       <c r="V35" s="2" t="inlineStr"/>
-      <c r="W35" s="2" t="inlineStr">
+      <c r="W35" s="2" t="inlineStr"/>
+      <c r="X35" s="2" t="inlineStr">
         <is>
           <t>NSF</t>
         </is>
       </c>
-      <c r="X35" s="3">
+      <c r="Y35" s="3">
         <f>HYPERLINK("https://github.com/asu-iris", "https://github.com/asu-iris")</f>
         <v/>
       </c>
-      <c r="Y35" s="2" t="inlineStr">
+      <c r="Z35" s="2" t="inlineStr">
         <is>
           <t>Recent Updates</t>
         </is>
       </c>
-      <c r="Z35" s="2" t="inlineStr">
+      <c r="AA35" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA35" s="2" t="b">
+      <c r="AB35" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB35" s="3">
+      <c r="AC35" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8438,15 +8634,16 @@
       <c r="W36" s="2" t="inlineStr"/>
       <c r="X36" s="2" t="inlineStr"/>
       <c r="Y36" s="2" t="inlineStr"/>
-      <c r="Z36" s="2" t="inlineStr">
+      <c r="Z36" s="2" t="inlineStr"/>
+      <c r="AA36" s="2" t="inlineStr">
         <is>
           <t>ENGRC 409 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA36" s="2" t="b">
+      <c r="AB36" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB36" s="3">
+      <c r="AC36" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8552,26 +8749,27 @@
         </is>
       </c>
       <c r="V37" s="2" t="inlineStr"/>
-      <c r="W37" s="2" t="inlineStr">
+      <c r="W37" s="2" t="inlineStr"/>
+      <c r="X37" s="2" t="inlineStr">
         <is>
           <t>NSF</t>
         </is>
       </c>
-      <c r="X37" s="2" t="inlineStr"/>
-      <c r="Y37" s="2" t="inlineStr">
+      <c r="Y37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
         <is>
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="Z37" s="2" t="inlineStr">
+      <c r="AA37" s="2" t="inlineStr">
         <is>
           <t>ERC457 551 E Tyler Mall (Tempe, AZ 85281)</t>
         </is>
       </c>
-      <c r="AA37" s="2" t="b">
+      <c r="AB37" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB37" s="3">
+      <c r="AC37" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8646,10 +8844,11 @@
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="2" t="inlineStr"/>
       <c r="Z38" s="2" t="inlineStr"/>
-      <c r="AA38" s="2" t="b">
+      <c r="AA38" s="2" t="inlineStr"/>
+      <c r="AB38" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB38" s="3">
+      <c r="AC38" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8723,15 +8922,16 @@
       <c r="W39" s="2" t="inlineStr"/>
       <c r="X39" s="2" t="inlineStr"/>
       <c r="Y39" s="2" t="inlineStr"/>
-      <c r="Z39" s="2" t="inlineStr">
+      <c r="Z39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA39" s="2" t="b">
+      <c r="AB39" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB39" s="3">
+      <c r="AC39" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8805,15 +9005,16 @@
       <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
-      <c r="Z40" s="2" t="inlineStr">
+      <c r="Z40" s="2" t="inlineStr"/>
+      <c r="AA40" s="2" t="inlineStr">
         <is>
           <t>ENGRC 411 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA40" s="2" t="b">
+      <c r="AB40" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB40" s="3">
+      <c r="AC40" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8890,15 +9091,16 @@
       <c r="W41" s="2" t="inlineStr"/>
       <c r="X41" s="2" t="inlineStr"/>
       <c r="Y41" s="2" t="inlineStr"/>
-      <c r="Z41" s="2" t="inlineStr">
+      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AA41" s="2" t="inlineStr">
         <is>
           <t>ENGRC 352 (TEMPE, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA41" s="2" t="b">
+      <c r="AB41" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB41" s="3">
+      <c r="AC41" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -8998,24 +9200,29 @@
       <c r="V42" s="2" t="inlineStr"/>
       <c r="W42" s="2" t="inlineStr">
         <is>
+          <t>SEM</t>
+        </is>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
           <t>NSF, ONR</t>
         </is>
       </c>
-      <c r="X42" s="2" t="inlineStr"/>
-      <c r="Y42" s="2" t="inlineStr">
+      <c r="Y42" s="2" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr">
         <is>
           <t>Highlighted as a cover in Small</t>
         </is>
       </c>
-      <c r="Z42" s="2" t="inlineStr">
+      <c r="AA42" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA42" s="2" t="b">
+      <c r="AB42" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB42" s="3">
+      <c r="AC42" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9089,15 +9296,16 @@
       <c r="W43" s="2" t="inlineStr"/>
       <c r="X43" s="2" t="inlineStr"/>
       <c r="Y43" s="2" t="inlineStr"/>
-      <c r="Z43" s="2" t="inlineStr">
+      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AA43" s="2" t="inlineStr">
         <is>
           <t>GWC 464 (Tempe, AZ 85287-6106)</t>
         </is>
       </c>
-      <c r="AA43" s="2" t="b">
+      <c r="AB43" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB43" s="3">
+      <c r="AC43" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9159,15 +9367,16 @@
       <c r="W44" s="2" t="inlineStr"/>
       <c r="X44" s="2" t="inlineStr"/>
       <c r="Y44" s="2" t="inlineStr"/>
-      <c r="Z44" s="2" t="inlineStr">
+      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="AA44" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA44" s="2" t="b">
+      <c r="AB44" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="AB44" s="3">
+      <c r="AC44" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9211,7 +9420,11 @@
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>MAE 301: Applied Experimental Statistic | MAE 202: Mech.Particles/Rigid Bodies II | MAE 417: System Dynamics and Control II</t>
+        </is>
+      </c>
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="inlineStr"/>
@@ -9230,10 +9443,15 @@
       <c r="X45" s="2" t="inlineStr"/>
       <c r="Y45" s="2" t="inlineStr"/>
       <c r="Z45" s="2" t="inlineStr"/>
-      <c r="AA45" s="2" t="b">
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Otherus</t>
+        </is>
+      </c>
+      <c r="AB45" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="AB45" s="3">
+      <c r="AC45" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9295,15 +9513,16 @@
       <c r="W46" s="2" t="inlineStr"/>
       <c r="X46" s="2" t="inlineStr"/>
       <c r="Y46" s="2" t="inlineStr"/>
-      <c r="Z46" s="2" t="inlineStr">
+      <c r="Z46" s="2" t="inlineStr"/>
+      <c r="AA46" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA46" s="2" t="b">
+      <c r="AB46" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="AB46" s="3">
+      <c r="AC46" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9347,7 +9566,11 @@
       </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>MAE 241: Intro to Thermodynamics | MAE 215: Intro to Programming in MATLAB | MAE 384: Adv Math Methods for Engineers</t>
+        </is>
+      </c>
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr"/>
       <c r="O47" s="2" t="inlineStr"/>
@@ -9362,10 +9585,15 @@
       <c r="X47" s="2" t="inlineStr"/>
       <c r="Y47" s="2" t="inlineStr"/>
       <c r="Z47" s="2" t="inlineStr"/>
-      <c r="AA47" s="2" t="b">
+      <c r="AA47" s="2" t="inlineStr">
+        <is>
+          <t>Campus: Tempe</t>
+        </is>
+      </c>
+      <c r="AB47" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="AB47" s="3">
+      <c r="AC47" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9427,15 +9655,16 @@
       <c r="W48" s="2" t="inlineStr"/>
       <c r="X48" s="2" t="inlineStr"/>
       <c r="Y48" s="2" t="inlineStr"/>
-      <c r="Z48" s="2" t="inlineStr">
+      <c r="Z48" s="2" t="inlineStr"/>
+      <c r="AA48" s="2" t="inlineStr">
         <is>
           <t>Campus: Tempe</t>
         </is>
       </c>
-      <c r="AA48" s="2" t="b">
+      <c r="AB48" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="AB48" s="3">
+      <c r="AC48" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9479,11 +9708,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>MAE 570: Intermediate Thermodynamics | MAE 400: Engineering Profession | MAE 494: Special Topics</t>
-        </is>
-      </c>
+      <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr"/>
       <c r="O49" s="2" t="inlineStr"/>
@@ -9497,15 +9722,12 @@
       <c r="W49" s="2" t="inlineStr"/>
       <c r="X49" s="2" t="inlineStr"/>
       <c r="Y49" s="2" t="inlineStr"/>
-      <c r="Z49" s="2" t="inlineStr">
-        <is>
-          <t>Campus: Tempe</t>
-        </is>
-      </c>
-      <c r="AA49" s="2" t="b">
+      <c r="Z49" s="2" t="inlineStr"/>
+      <c r="AA49" s="2" t="inlineStr"/>
+      <c r="AB49" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="AB49" s="3">
+      <c r="AC49" s="3">
         <f>HYPERLINK("https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/", "https://faculty.engineering.asu.edu/directory/semte/aerospace-and-mechanical-engineering/")</f>
         <v/>
       </c>
@@ -9516,222 +9738,222 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC2" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC3" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC4" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC5" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC6" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB7" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC7" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB8" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC8" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB9" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC9" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC10" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC12" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T13" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC13" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC14" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC15" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC16" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T17" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC18" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB21" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC21" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T23" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T24" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC24" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T25" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC25" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC26" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T27" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId122"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId123"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T29" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB29" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC29" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T30" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId137"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T31" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC31" r:id="rId141"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId145"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId146"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId147"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId148"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T33" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC33" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId151"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId152"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId153"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T34" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC34" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId157"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId158"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T35" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X35" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y35" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId165"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T37" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB37" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC37" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId171"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId174"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId175"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB39" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC39" r:id="rId178"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T41" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId187"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T42" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB44" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC44" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId204"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId205"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId208"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId209"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId210"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB47" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC47" r:id="rId212"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId213"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId214"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId216"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId217"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId218"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId220"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(asu): preserve raw OpenAlex API JSON extractions in openalex_cache for all professors
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -2552,8 +2552,16 @@
           <t>Micro-scale Thermal Partial Oxidation Reformer and Integrated Solid Oxide Fuel Cell Operating with Jet Fuel,</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>"Multi-year assessment of energy storage capacity for a carbon-neutral grid in Arizona and the impact of wind energy integration" [Renewable Energy] (2026) [DOI: https://doi.org/10.1016/j.renene.2026.126276] | "Analysis of gas turbines with diffusion, premixed and rich-quench-lean combustor designs utilizing ternary CH4/H2/NH3 fuel blends" [Energy Conversion and Management] (2026) [DOI: https://doi.org/10.1016/j.enconman.2026.121736] | "Micro-scale thermal partial oxidation reformer and integrated solid oxide fuel cell operating with jet fuel" [Journal of Power Sources] (2026) [DOI: https://doi.org/10.1016/j.jpowsour.2026.240198]</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>"A review of energy storage technologies for demand-side management in industrial facilities" [Journal of Cleaner Production] (2021, 100 cites) [DOI: https://doi.org/10.1016/j.jclepro.2021.127322] | "Techno-Economic Assessment of CHP Systems in Wastewater Treatment Plants" [Environments] (2020, 78 cites) [DOI: https://doi.org/10.3390/environments7100074] | "Thermodynamic and emission analysis of a hydrogen/methane fueled gas turbine" [Energy Conversion and Management X] (2023, 50 cites) [DOI: https://doi.org/10.1016/j.ecmx.2023.100394]</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
           <t>MAE 593: Applied Project | MAE 436: Combustion | MAE 536: Combustion</t>
@@ -2565,8 +2573,16 @@
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Advancements in Solid Oxide Fuel Cells (54) | Fuel Cells and Related Materials (31) | Catalytic Processes in Materials Science (30)</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Advancements in Solid Oxide Fuel Cells (54) | Fuel Cells and Related Materials (31) | Catalytic Processes in Materials Science (30)</t>
+        </is>
+      </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
           <t>Energy management and efficiency, energy transition, energy storage, solid oxide fuel cells, partial oxidation, cogeneration, combustion, and synthesis of hydrogen</t>
@@ -3811,16 +3827,8 @@
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>"Large Language Model Assisted Discovery of Optimal Dopants for Enhanced Thermoelectric Performance in CoSb$_3$ Based Skutterudites" [arXiv (Cornell University)] (2026) [DOI: https://doi.org/10.48550/arxiv.2604.06048] | "Large Language Model Assisted Discovery of Optimal Dopants for Enhanced Thermoelectric Performance in CoSb$_3$ Based Skutterudites" [arXiv (Cornell University)] (2026) [DOI: http://arxiv.org/abs/2604.06048] | "AI and 3D printing help researchers create heat- and pressure-resistant materials for aerospace and defense applications" (2026) [DOI: https://doi.org/10.64628/aai.rjqc4cr7j]</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>"Prediction and Characterization of MXene Nanosheet Anodes for Non-Lithium-Ion Batteries" [ACS Nano] (2014, 1046 cites) [DOI: https://doi.org/10.1021/nn503921j] | "Single-Layer Group-III Monochalcogenide Photocatalysts for Water Splitting" [Chemistry of Materials] (2013, 852 cites) [DOI: https://doi.org/10.1021/cm401661x] | "Computational Screening of 2D Materials for Photocatalysis" [The Journal of Physical Chemistry Letters] (2015, 833 cites) [DOI: https://doi.org/10.1021/jz502646d]</t>
-        </is>
-      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr">
         <is>
           <t>MAE 551: Appl Machine Learn Mech Engr | MAE 451: Appl Machine Learn Mech Engr | MAE 202: Mech.Particles/Rigid Bodies II</t>
@@ -3828,16 +3836,8 @@
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr">
-        <is>
-          <t>2D Materials and Applications (58) | Graphene research and applications (43) | MXene and MAX Phase Materials (23)</t>
-        </is>
-      </c>
-      <c r="R28" s="2" t="inlineStr">
-        <is>
-          <t>2D Materials and Applications (58) | Graphene research and applications (43) | MXene and MAX Phase Materials (23)</t>
-        </is>
-      </c>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="inlineStr">
         <is>
           <t>Quantum simulations Machine learning Quantum computing</t>
@@ -5578,11 +5578,7 @@
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>"A Rapid Poly(ethylene glycol)-Assisted Magnetic Isolation Approach for High-Throughput Extracellular Vesicle Isolation and Subsequent Biomarker Analysis" [ACS Nano] (2026) [DOI: https://doi.org/10.1021/acsnano.6c09351] | "Impact of sarcopenia on short- and long-term outcomes after resection of perihilar cholangiocarcinoma: a two-center study" [BMC Cancer] (2026) [DOI: https://doi.org/10.1186/s12885-026-16305-7] | "Genotypic features of Spinocerebellar Ataxia in Northern China: A Comparative Analysis with Southern China" [The Cerebellum] (2026) [DOI: https://doi.org/10.1007/s12311-026-02058-3]</t>
-        </is>
-      </c>
+      <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr">
         <is>
           <t>"Plant-Derived Exosomal MicroRNAs Shape the Gut Microbiota" [Cell Host &amp; Microbe] (2018, 1030 cites) [DOI: https://doi.org/10.1016/j.chom.2018.10.001] | "MVP-mediated exosomal sorting of miR-193a promotes colon cancer progression" [Nature Communications] (2017, 502 cites) [DOI: https://doi.org/10.1038/ncomms14448] | "CD36 gene transfer confers capacity for phagocytosis of cells undergoing apoptosis." [The Journal of Experimental Medicine] (1995, 394 cites) [DOI: https://doi.org/10.1084/jem.181.5.1857]</t>
@@ -7944,8 +7940,16 @@
           <t>Micro-scale Thermal Partial Oxidation Reformer and Integrated Solid Oxide Fuel Cell Operating with Jet Fuel,</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>"Multi-year assessment of energy storage capacity for a carbon-neutral grid in Arizona and the impact of wind energy integration" [Renewable Energy] (2026) [DOI: https://doi.org/10.1016/j.renene.2026.126276] | "Analysis of gas turbines with diffusion, premixed and rich-quench-lean combustor designs utilizing ternary CH4/H2/NH3 fuel blends" [Energy Conversion and Management] (2026) [DOI: https://doi.org/10.1016/j.enconman.2026.121736] | "Micro-scale thermal partial oxidation reformer and integrated solid oxide fuel cell operating with jet fuel" [Journal of Power Sources] (2026) [DOI: https://doi.org/10.1016/j.jpowsour.2026.240198]</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>"A review of energy storage technologies for demand-side management in industrial facilities" [Journal of Cleaner Production] (2021, 100 cites) [DOI: https://doi.org/10.1016/j.jclepro.2021.127322] | "Techno-Economic Assessment of CHP Systems in Wastewater Treatment Plants" [Environments] (2020, 78 cites) [DOI: https://doi.org/10.3390/environments7100074] | "Thermodynamic and emission analysis of a hydrogen/methane fueled gas turbine" [Energy Conversion and Management X] (2023, 50 cites) [DOI: https://doi.org/10.1016/j.ecmx.2023.100394]</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
           <t>MAE 593: Applied Project | MAE 436: Combustion | MAE 536: Combustion</t>
@@ -7957,8 +7961,16 @@
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Advancements in Solid Oxide Fuel Cells (54) | Fuel Cells and Related Materials (31) | Catalytic Processes in Materials Science (30)</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Advancements in Solid Oxide Fuel Cells (54) | Fuel Cells and Related Materials (31) | Catalytic Processes in Materials Science (30)</t>
+        </is>
+      </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
           <t>Energy management and efficiency, energy transition, energy storage, solid oxide fuel cells, partial oxidation, cogeneration, combustion, and synthesis of hydrogen</t>
@@ -9203,16 +9215,8 @@
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>"Large Language Model Assisted Discovery of Optimal Dopants for Enhanced Thermoelectric Performance in CoSb$_3$ Based Skutterudites" [arXiv (Cornell University)] (2026) [DOI: https://doi.org/10.48550/arxiv.2604.06048] | "Large Language Model Assisted Discovery of Optimal Dopants for Enhanced Thermoelectric Performance in CoSb$_3$ Based Skutterudites" [arXiv (Cornell University)] (2026) [DOI: http://arxiv.org/abs/2604.06048] | "AI and 3D printing help researchers create heat- and pressure-resistant materials for aerospace and defense applications" (2026) [DOI: https://doi.org/10.64628/aai.rjqc4cr7j]</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>"Prediction and Characterization of MXene Nanosheet Anodes for Non-Lithium-Ion Batteries" [ACS Nano] (2014, 1046 cites) [DOI: https://doi.org/10.1021/nn503921j] | "Single-Layer Group-III Monochalcogenide Photocatalysts for Water Splitting" [Chemistry of Materials] (2013, 852 cites) [DOI: https://doi.org/10.1021/cm401661x] | "Computational Screening of 2D Materials for Photocatalysis" [The Journal of Physical Chemistry Letters] (2015, 833 cites) [DOI: https://doi.org/10.1021/jz502646d]</t>
-        </is>
-      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr">
         <is>
           <t>MAE 551: Appl Machine Learn Mech Engr | MAE 451: Appl Machine Learn Mech Engr | MAE 202: Mech.Particles/Rigid Bodies II</t>
@@ -9220,16 +9224,8 @@
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr">
-        <is>
-          <t>2D Materials and Applications (58) | Graphene research and applications (43) | MXene and MAX Phase Materials (23)</t>
-        </is>
-      </c>
-      <c r="R28" s="2" t="inlineStr">
-        <is>
-          <t>2D Materials and Applications (58) | Graphene research and applications (43) | MXene and MAX Phase Materials (23)</t>
-        </is>
-      </c>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="inlineStr">
         <is>
           <t>Quantum simulations Machine learning Quantum computing</t>
@@ -10970,11 +10966,7 @@
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>"A Rapid Poly(ethylene glycol)-Assisted Magnetic Isolation Approach for High-Throughput Extracellular Vesicle Isolation and Subsequent Biomarker Analysis" [ACS Nano] (2026) [DOI: https://doi.org/10.1021/acsnano.6c09351] | "Impact of sarcopenia on short- and long-term outcomes after resection of perihilar cholangiocarcinoma: a two-center study" [BMC Cancer] (2026) [DOI: https://doi.org/10.1186/s12885-026-16305-7] | "Genotypic features of Spinocerebellar Ataxia in Northern China: A Comparative Analysis with Southern China" [The Cerebellum] (2026) [DOI: https://doi.org/10.1007/s12311-026-02058-3]</t>
-        </is>
-      </c>
+      <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr">
         <is>
           <t>"Plant-Derived Exosomal MicroRNAs Shape the Gut Microbiota" [Cell Host &amp; Microbe] (2018, 1030 cites) [DOI: https://doi.org/10.1016/j.chom.2018.10.001] | "MVP-mediated exosomal sorting of miR-193a promotes colon cancer progression" [Nature Communications] (2017, 502 cites) [DOI: https://doi.org/10.1038/ncomms14448] | "CD36 gene transfer confers capacity for phagocytosis of cells undergoing apoptosis." [The Journal of Experimental Medicine] (1995, 394 cites) [DOI: https://doi.org/10.1084/jem.181.5.1857]</t>
@@ -11160,8 +11152,16 @@
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
-      <c r="M45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>"Hierarchical models for small area estimation using zero-inflated forest inventory variables: comparison and implementation" [Canadian Journal of Forest Research] (2026) [DOI: https://doi.org/10.1139/cjfr-2025-0175] | "Leveraging national forest inventory data to estimate forest carbon density status and trends for small areas" [Forest Ecology and Management] (2025) [DOI: https://doi.org/10.1016/j.foreco.2025.122999] | "Hierarchical models for small area estimation using zero-inflated forest inventory variables: comparison and implementation" [arXiv (Cornell University)] (2025) [DOI: https://doi.org/10.48550/arxiv.2503.22103]</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>"Estimating forest canopy fuel parameters using LIDAR data" [Remote Sensing of Environment] (2005, 581 cites) [DOI: https://doi.org/10.1016/j.rse.2004.10.013] | "Aboveground biomass density models for NASA’s Global Ecosystem Dynamics Investigation (GEDI) lidar mission" [Remote Sensing of Environment] (2022, 481 cites) [DOI: https://doi.org/10.1016/j.rse.2021.112845] | "Light Detection and Ranging (LIDAR): An Emerging Tool for Multiple Resource Inventory" [Journal of Forestry] (2005, 390 cites) [DOI: https://doi.org/10.1093/jof/103.6.286]</t>
+        </is>
+      </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
           <t>MAE 301: Applied Experimental Statistic | MAE 202: Mech.Particles/Rigid Bodies II | MAE 417: System Dynamics and Control II</t>
@@ -11169,8 +11169,16 @@
       </c>
       <c r="O45" s="2" t="inlineStr"/>
       <c r="P45" s="2" t="inlineStr"/>
-      <c r="Q45" s="2" t="inlineStr"/>
-      <c r="R45" s="2" t="inlineStr"/>
+      <c r="Q45" s="2" t="inlineStr">
+        <is>
+          <t>Remote Sensing and LiDAR Applications (93) | Forest ecology and management (59) | Forest Ecology and Biodiversity Studies (31)</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>Remote Sensing and LiDAR Applications (93) | Forest ecology and management (59) | Forest Ecology and Biodiversity Studies (31)</t>
+        </is>
+      </c>
       <c r="S45" s="2" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr"/>
       <c r="U45" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: add comprehensive MASTER_PIPELINE_BLUEPRINT.md and update ASU 2023-2026 recent papers
</commit_message>
<xml_diff>
--- a/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
+++ b/universities_wise/arizona_state_university/asu_aerospace_mechanical_faculty.xlsx
@@ -642,7 +642,7 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Recent Papers (2024-2026)</t>
+          <t>Recent Papers (2023-2026)</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -1067,8 +1067,16 @@
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
-      <c r="AA3" s="2" t="inlineStr"/>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>"Heterogeneous Feature Knowledge Distillation based on Enhanced Feature Projector Correlation" [Neural Networks] (2025) [DOI: https://doi.org/10.1016/j.neunet.2025.108409] | "Deep learning and multi-omics reveal programmed cell death-associated diagnostic signatures and prognostic biomarkers in gastric cancer" [Frontiers in Immunology] (2025) [DOI: https://doi.org/10.3389/fimmu.2025.1690200] | "Research on flexible job shop scheduling based on deep reinforcement learning with transformer-graph neural network" [Journal of Control and Decision] (2025) [DOI: https://doi.org/10.1080/23307706.2025.2557020] | "Astra: Toward General-Purpose Mobile Robots via Hierarchical Multimodal Learning" [arXiv (Cornell University)] (2025) [DOI: https://doi.org/10.48550/arxiv.2506.06205] | "Optimizing the flexible job shop scheduling problem via deep reinforcement learning with mean multichannel graph attention" [Applied Soft Computing] (2025) [DOI: https://doi.org/10.1016/j.asoc.2025.113128]</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>"Lubricated pipelining: stability of core-annular flow" [Journal of Fluid Mechanics] (1989, 202 cites) [DOI: https://doi.org/10.1017/s0022112089000960] | "Lubricated pipelining: stability of core—annular flow. Part 5. Experiments and comparison with theory" [Journal of Fluid Mechanics] (1992, 163 cites) [DOI: https://doi.org/10.1017/s0022112092000041] | "Pool-boiling enhancement by novel metallic nanoporous surface" [Experimental Thermal and Fluid Science] (2012, 112 cites) [DOI: https://doi.org/10.1016/j.expthermflusci.2012.06.008]</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
           <t>MAE 242: Intro to Fluid Mechanics | MAE 384: Adv Math Methods for Engineers | MAE 501: Linear Algebra in Engineering</t>
@@ -1076,8 +1084,16 @@
       </c>
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>Fluid Dynamics and Thin Films (12) | Rheology and Fluid Dynamics Studies (11) | Hydraulic Fracturing and Reservoir Analysis (7)</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Fluid Dynamics and Thin Films (12) | Rheology and Fluid Dynamics Studies (11) | Hydraulic Fracturing and Reservoir Analysis (7)</t>
+        </is>
+      </c>
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr">
@@ -1990,7 +2006,11 @@
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr"/>
-      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>"Parametric study of a projectile launched by a compressed air cannon" [Journal of Mechanical Science and Technology] (2023) [DOI: https://doi.org/10.1007/s12206-023-1029-x]</t>
+        </is>
+      </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
           <t>"Adjoint-based control of loud events in a turbulent jet" [Journal of Fluid Mechanics] (2014, 46 cites) [DOI: https://doi.org/10.1017/jfm.2013.654] | "LES Investigation of a Mach 1.3 Jet With and Without Plasma Actuators" [47th AIAA Aerospace Sciences Meeting including The New Horizons Forum and Aerospace Exposition] (2009, 38 cites) [DOI: https://doi.org/10.2514/6.2009-290] | "A High-Order, Overset-Mesh Algorithm for Adjoint-Based Optimization for Aeroacoustics Control" (2010, 21 cites) [DOI: https://doi.org/10.2514/6.2010-3818]</t>
@@ -2771,9 +2791,17 @@
       <c r="AN12" s="2" t="inlineStr"/>
       <c r="AO12" s="2" t="inlineStr"/>
       <c r="AP12" s="2" t="inlineStr"/>
-      <c r="AQ12" s="2" t="inlineStr"/>
+      <c r="AQ12" s="2" t="inlineStr">
+        <is>
+          <t>DOE, NASA</t>
+        </is>
+      </c>
       <c r="AR12" s="2" t="inlineStr"/>
-      <c r="AS12" s="2" t="inlineStr"/>
+      <c r="AS12" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Remote SensingGroup</t>
+        </is>
+      </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
@@ -3070,7 +3098,7 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Recent Papers (2024-2026)</t>
+          <t>Recent Papers (2023-2026)</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -3495,8 +3523,16 @@
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
-      <c r="AA3" s="2" t="inlineStr"/>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>"Heterogeneous Feature Knowledge Distillation based on Enhanced Feature Projector Correlation" [Neural Networks] (2025) [DOI: https://doi.org/10.1016/j.neunet.2025.108409] | "Deep learning and multi-omics reveal programmed cell death-associated diagnostic signatures and prognostic biomarkers in gastric cancer" [Frontiers in Immunology] (2025) [DOI: https://doi.org/10.3389/fimmu.2025.1690200] | "Research on flexible job shop scheduling based on deep reinforcement learning with transformer-graph neural network" [Journal of Control and Decision] (2025) [DOI: https://doi.org/10.1080/23307706.2025.2557020] | "Astra: Toward General-Purpose Mobile Robots via Hierarchical Multimodal Learning" [arXiv (Cornell University)] (2025) [DOI: https://doi.org/10.48550/arxiv.2506.06205] | "Optimizing the flexible job shop scheduling problem via deep reinforcement learning with mean multichannel graph attention" [Applied Soft Computing] (2025) [DOI: https://doi.org/10.1016/j.asoc.2025.113128]</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>"Lubricated pipelining: stability of core-annular flow" [Journal of Fluid Mechanics] (1989, 202 cites) [DOI: https://doi.org/10.1017/s0022112089000960] | "Lubricated pipelining: stability of core—annular flow. Part 5. Experiments and comparison with theory" [Journal of Fluid Mechanics] (1992, 163 cites) [DOI: https://doi.org/10.1017/s0022112092000041] | "Pool-boiling enhancement by novel metallic nanoporous surface" [Experimental Thermal and Fluid Science] (2012, 112 cites) [DOI: https://doi.org/10.1016/j.expthermflusci.2012.06.008]</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
           <t>MAE 242: Intro to Fluid Mechanics | MAE 384: Adv Math Methods for Engineers | MAE 501: Linear Algebra in Engineering</t>
@@ -3504,8 +3540,16 @@
       </c>
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>Fluid Dynamics and Thin Films (12) | Rheology and Fluid Dynamics Studies (11) | Hydraulic Fracturing and Reservoir Analysis (7)</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Fluid Dynamics and Thin Films (12) | Rheology and Fluid Dynamics Studies (11) | Hydraulic Fracturing and Reservoir Analysis (7)</t>
+        </is>
+      </c>
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr">
@@ -4418,7 +4462,11 @@
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr"/>
-      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>"Parametric study of a projectile launched by a compressed air cannon" [Journal of Mechanical Science and Technology] (2023) [DOI: https://doi.org/10.1007/s12206-023-1029-x]</t>
+        </is>
+      </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
           <t>"Adjoint-based control of loud events in a turbulent jet" [Journal of Fluid Mechanics] (2014, 46 cites) [DOI: https://doi.org/10.1017/jfm.2013.654] | "LES Investigation of a Mach 1.3 Jet With and Without Plasma Actuators" [47th AIAA Aerospace Sciences Meeting including The New Horizons Forum and Aerospace Exposition] (2009, 38 cites) [DOI: https://doi.org/10.2514/6.2009-290] | "A High-Order, Overset-Mesh Algorithm for Adjoint-Based Optimization for Aeroacoustics Control" (2010, 21 cites) [DOI: https://doi.org/10.2514/6.2010-3818]</t>
@@ -5199,9 +5247,17 @@
       <c r="AN12" s="2" t="inlineStr"/>
       <c r="AO12" s="2" t="inlineStr"/>
       <c r="AP12" s="2" t="inlineStr"/>
-      <c r="AQ12" s="2" t="inlineStr"/>
+      <c r="AQ12" s="2" t="inlineStr">
+        <is>
+          <t>DOE, NASA</t>
+        </is>
+      </c>
       <c r="AR12" s="2" t="inlineStr"/>
-      <c r="AS12" s="2" t="inlineStr"/>
+      <c r="AS12" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Remote SensingGroup</t>
+        </is>
+      </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>
@@ -6406,7 +6462,7 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Recent Papers (2024-2026)</t>
+          <t>Recent Papers (2023-2026)</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -6831,8 +6887,16 @@
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
-      <c r="AA3" s="2" t="inlineStr"/>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>"Heterogeneous Feature Knowledge Distillation based on Enhanced Feature Projector Correlation" [Neural Networks] (2025) [DOI: https://doi.org/10.1016/j.neunet.2025.108409] | "Deep learning and multi-omics reveal programmed cell death-associated diagnostic signatures and prognostic biomarkers in gastric cancer" [Frontiers in Immunology] (2025) [DOI: https://doi.org/10.3389/fimmu.2025.1690200] | "Research on flexible job shop scheduling based on deep reinforcement learning with transformer-graph neural network" [Journal of Control and Decision] (2025) [DOI: https://doi.org/10.1080/23307706.2025.2557020] | "Astra: Toward General-Purpose Mobile Robots via Hierarchical Multimodal Learning" [arXiv (Cornell University)] (2025) [DOI: https://doi.org/10.48550/arxiv.2506.06205] | "Optimizing the flexible job shop scheduling problem via deep reinforcement learning with mean multichannel graph attention" [Applied Soft Computing] (2025) [DOI: https://doi.org/10.1016/j.asoc.2025.113128]</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>"Lubricated pipelining: stability of core-annular flow" [Journal of Fluid Mechanics] (1989, 202 cites) [DOI: https://doi.org/10.1017/s0022112089000960] | "Lubricated pipelining: stability of core—annular flow. Part 5. Experiments and comparison with theory" [Journal of Fluid Mechanics] (1992, 163 cites) [DOI: https://doi.org/10.1017/s0022112092000041] | "Pool-boiling enhancement by novel metallic nanoporous surface" [Experimental Thermal and Fluid Science] (2012, 112 cites) [DOI: https://doi.org/10.1016/j.expthermflusci.2012.06.008]</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
           <t>MAE 242: Intro to Fluid Mechanics | MAE 384: Adv Math Methods for Engineers | MAE 501: Linear Algebra in Engineering</t>
@@ -6840,8 +6904,16 @@
       </c>
       <c r="AD3" s="2" t="inlineStr"/>
       <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>Fluid Dynamics and Thin Films (12) | Rheology and Fluid Dynamics Studies (11) | Hydraulic Fracturing and Reservoir Analysis (7)</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Fluid Dynamics and Thin Films (12) | Rheology and Fluid Dynamics Studies (11) | Hydraulic Fracturing and Reservoir Analysis (7)</t>
+        </is>
+      </c>
       <c r="AH3" s="2" t="inlineStr"/>
       <c r="AI3" s="2" t="inlineStr"/>
       <c r="AJ3" s="2" t="inlineStr">
@@ -7754,7 +7826,11 @@
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr"/>
-      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>"Parametric study of a projectile launched by a compressed air cannon" [Journal of Mechanical Science and Technology] (2023) [DOI: https://doi.org/10.1007/s12206-023-1029-x]</t>
+        </is>
+      </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
           <t>"Adjoint-based control of loud events in a turbulent jet" [Journal of Fluid Mechanics] (2014, 46 cites) [DOI: https://doi.org/10.1017/jfm.2013.654] | "LES Investigation of a Mach 1.3 Jet With and Without Plasma Actuators" [47th AIAA Aerospace Sciences Meeting including The New Horizons Forum and Aerospace Exposition] (2009, 38 cites) [DOI: https://doi.org/10.2514/6.2009-290] | "A High-Order, Overset-Mesh Algorithm for Adjoint-Based Optimization for Aeroacoustics Control" (2010, 21 cites) [DOI: https://doi.org/10.2514/6.2010-3818]</t>
@@ -8535,9 +8611,17 @@
       <c r="AN12" s="2" t="inlineStr"/>
       <c r="AO12" s="2" t="inlineStr"/>
       <c r="AP12" s="2" t="inlineStr"/>
-      <c r="AQ12" s="2" t="inlineStr"/>
+      <c r="AQ12" s="2" t="inlineStr">
+        <is>
+          <t>DOE, NASA</t>
+        </is>
+      </c>
       <c r="AR12" s="2" t="inlineStr"/>
-      <c r="AS12" s="2" t="inlineStr"/>
+      <c r="AS12" s="2" t="inlineStr">
+        <is>
+          <t>Environmental Remote SensingGroup</t>
+        </is>
+      </c>
       <c r="AT12" s="2" t="inlineStr">
         <is>
           <t>Goldwater 466 (TEMPE, AZ 85287-6106)</t>

</xml_diff>